<commit_message>
Add Form Issue , Return , Damage
</commit_message>
<xml_diff>
--- a/data/master_data.xlsx
+++ b/data/master_data.xlsx
@@ -7,15 +7,18 @@
     <sheet name="Stores" sheetId="2" r:id="rId2"/>
     <sheet name="Users" sheetId="3" r:id="rId3"/>
     <sheet name="Suppliers" sheetId="4" r:id="rId4"/>
-    <sheet name="Customers" sheetId="5" r:id="rId5"/>
-    <sheet name="Projects" sheetId="6" r:id="rId6"/>
-    <sheet name="IssueTypes" sheetId="7" r:id="rId7"/>
-    <sheet name="ItemNames" sheetId="8" r:id="rId8"/>
-    <sheet name="Specifications" sheetId="9" r:id="rId9"/>
-    <sheet name="SpecificationValues" sheetId="10" r:id="rId10"/>
-    <sheet name="Items" sheetId="11" r:id="rId11"/>
-    <sheet name="ItemNames_Template15" sheetId="12" r:id="rId12"/>
-    <sheet name="Items_Template15" sheetId="13" r:id="rId13"/>
+    <sheet name="Transporters" sheetId="5" r:id="rId5"/>
+    <sheet name="Customers" sheetId="6" r:id="rId6"/>
+    <sheet name="Projects" sheetId="7" r:id="rId7"/>
+    <sheet name="IssueTypes" sheetId="8" r:id="rId8"/>
+    <sheet name="Units" sheetId="9" r:id="rId9"/>
+    <sheet name="ItemCategories" sheetId="10" r:id="rId10"/>
+    <sheet name="ItemNames" sheetId="11" r:id="rId11"/>
+    <sheet name="Specifications" sheetId="12" r:id="rId12"/>
+    <sheet name="SpecificationValues" sheetId="13" r:id="rId13"/>
+    <sheet name="Items" sheetId="14" r:id="rId14"/>
+    <sheet name="ItemNames_Template15" sheetId="15" r:id="rId15"/>
+    <sheet name="Items_Template15" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -409,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -445,13 +448,31 @@
       <c r="K1" t="str">
         <v>updated_at</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="L1" t="str">
+        <v>cin</v>
+      </c>
+      <c r="M1" t="str">
+        <v>logo_url</v>
+      </c>
+      <c r="N1" t="str">
+        <v>terms_conditions</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>FIRM-1</v>
       </c>
       <c r="B2" t="str">
-        <v>Umang (Main)</v>
+        <v>Umang Communications Pvt Ltd</v>
+      </c>
+      <c r="C2" t="str">
+        <v>18AABCU2874Q1ZL</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Adagudam, Near Hanuman Mandir, Lokhra Road, Guwahati - 781034 (Assam)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>9864023964</v>
       </c>
       <c r="H2" t="str">
         <v>system</v>
@@ -463,15 +484,38 @@
         <v>system</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-04-11T08:38:18.325Z</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>2026-04-22T12:34:58.074Z</v>
+      </c>
+      <c r="L2" t="str">
+        <v>U74900AS2011PTC010451</v>
+      </c>
+      <c r="M2" t="str">
+        <v>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/4gHYSUNDX1BST0ZJTEUAAQEAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADb/2wBDAAMCAgICAgMCAgIDAwMDBAYEBAQEBAgGBgUGCQgKCgkICQkKDA8MCgsOCwkJDRENDg8QEBEQCgwSExIQEw8QEBD/2wBDAQMDAwQDBAgEBAgQCwkLEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBD/wAARCABhAMQDASIAAhEBAxEB/8QAHQABAAEFAQEBAAAAAAAAAAAAAAgDBQYHCQQBAv/EAEgQAAEDBAECAwQFBwkFCQAAAAECAwQABQYRBwgSEyExCRQiQTI3UWGBFhdxdZGztBUjNkJSYnJ2oSQ0dIKyMzlEc4OSk6Kj/8QAGwEBAAIDAQEAAAAAAAAAAAAAAAQFAgMGAQf/xAA5EQABAwMCBAMGAwYHAAAAAAABAAIDBBEhBTESQVFxE2GhBiKBkbHBFDLwNDVCUtHhFSMzQ4KS8f/aAAwDAQACEQMRAD8A6p0pSiJSlKIlKUoiUrSfKXPF6xzm7AOD8EtlvuN2yN73u9OSkrWIFtTsqUkIUnTikodIKjodg2D3DW7KkTU0kDGPkFuMXHa9r+mFrZK2Qua3lgpSlKjrYlKUoiUpSiJSlKIlKUoiUpSiJSlKIlKUoiUpSiJSlKIsR5S5Twzh3Dpeb5zcvdIEbSEIQO56S8Qe1lpH9ZatHy9AASSACRzK5n66eauTrm61jN9lYZYkqIjw7TIU1IUnfkp2QnS1K18klKfu+Zdd3LN85B5zu+MvSXEWXD3lWyDF2QkOgDx3SPmpS9jf9lKBUcq+r+zXs3T00DaqpaHSOF85DQdsdep+XnyWp6nJLIYojZox3U1OiLqy5If5Ot3FvIuTz8itOQlbESTcXlPyYkoJUpGnVErUhfb2FKidEpI0AQZ88iZ7j3GGFXfO8plBi3WeOp9zzHc4r0Q2jfqtailKR9qhXN32f/CF9zXlSHylMiLYxrEXFvGSsaTJm9hDbSD8+3uDij6AJSD9IVcusPnqf1Gcl2jhLi58zLHEubcNlbSvgulyWrww5serSO4pSfQ7WrzBTqq1bRqfUdZEVOA1jWgyEYA39SLfXqpdJWyU1FxyZJNm35/2W7ehix37krKc36qM6a7rlkstdttQVspZjpKS4G9/1E9rTKT66aWD6mpjVjPGuC2njHALFgVmAESxwW4oXrt8VYG3HSPtWsqWfvUayBqXEkKKGJTTigNkIWCdfhXHapViuqnysFm7NHRowB8lc0kPgRBh33Pc7qtSvilJSkqUoAAbJJ8gKpsyosglLElpwgbIQsHX7KrrKSqtKoOTYTKy29LZQseqVOAEfhVRt1p5AcZcStB9FJOwfxr2xRfulUnpUWOQl+S02T5gLWBv9tfWZEeQCWH23APIlCgrX7KWO6KpSlUUTYbrgablsrWfRKXAT+yvLIq1KVSelRY5CX5LTZI2AtYG/wBtN0VWlfAQoBSSCD5gj51TelxY5CX5LTZI2AtYG/20tdFVpXwEEbB2DVKXLiQI7kydKZjsNDucddWEIQPtJPkKAXwEValWO0Z1hOQSvcbDmNjuUnRPgw7gy8vQ9fhQomr5WTmOYbOFl4CHZCUpSsV6lRYHM9+6XuT5PHvN13uF0wXJ5b0/F8okFTzkLvX3OQ5J81KShSgAobKQUnXadNynrWXUXw1budOKrthEhLSLgUe92mSsf7vNQCW1b+SVbKFf3Vq+eqsdNmgZL4VULxvweo6OB6j1Fwo1SyQt44j7w28/I91GzqT6JXeb8nc5i4QyyxSBf0ofmRnpO40hwAJ8dh5sLSe4AFSTobCj3eehivHHs5GMfQvLOobPrZb7LAT478O3SShBQPM+NKdCQ2n7e0EkHyUk1EOw53ydxdPl23GcwyDGpLDy2ZTEKe7H06k9qgtKFAEgjXn9lUct5L5Dz4o/LbOb9fUtHubRcLg6+hs61tKVqIT+Ar6jFpeqxxCmjqh4YwDw+9bpvbbnuuVfV0jnmV0R4ul8XUpupXrFxpOK/mM6bIrdoxRhkw5lyisljx2vMKZjpOlJQrZ73FfEvZ+RJVR9m3xL+U/JNy5SucXugYmx4EIqHkqc+kp2PkexrvJ+wuINQ+ZZekvNx47S3XXVBCEISVKUonQAA9ST8q7M9MvEDXCXDljwxxpKbmtv3+7rT/XmugFwbHqEAJbB+YbFV+vmDQNLNJTfmlwSdz/MSefT4qTp4k1Cq8aXZvyHQD9cln+Vf0XvH/ASP3aq5vezI+vq/f5QlfxsOukOVf0XvH/ASP3aq5vezI+vq/f5QlfxsOub0P8AdFd2b91ZV/7ZB3P2XQfmH6o83/y5cv4ZyoI+y9+sjMv1G1+/TU7uYfqjzf8Ay5cv4ZyoI+y9+sjMv1G1+/TTSf3FW/8AH6pWft8HxWsuvRtbvVTlTTSCta2ralKUjZJMJjQFSt9mhl/8scM3nEnne57Hr0tSE7+jHkIStP8A+iX60F1IQo1y9oPAt0xoOR5V/wAaZdQfRSFNxAofiCayT2e0+Tx91B53xLcnSlT0aRHUD5d8qBJKQNf4FvH8K6LUmCp9nmRfxNjjePofS6rqZxi1Ev5FzgsH9olla8m6iX7DHUpxvGbRGglKfMBakqkrV+nteSD/AIPurensu/6B5v8AreP+5NRkcV+d7lPmzkxX87Ft9ovd2jrPmAhxwRmE/pDT3l/hqTfsu/6B5v8AreP+5NNZYKf2fNKN2CMHubEpROMmoeL/ADcVuyk3z5yGnirh3K87DobkW63OCGT85bmm2B/8i0b+7dcfOK86uHGnJON8isB1RtFzbkuEb282FDxm9/PubUpJ/wAVTh9p3yN7ji+LcWw39O3WSu8TkpPmGWQUNJP3KWtZ/S0K1Xzn09/kh0acY5k1B7LpbnVS7uoJ0rw7lpxJX97ZSw3r7VGtHsw2GhoWfiBmpcW/AAgetx8Qs9UL55z4f+0L/G4+30XS6DNi3KFHuMF9D8aU0h5l1B2laFAFKh9xBBrnN7UH6zcP/UK/4hdSd6FeSPzhdPNkjyX/ABJ+LqXYpOz59rIBYP6PBW0N/ak1GL2oP1m4f+oV/wAQuqj2bpXUWvfh37t4h6H6qZqUon0/xBzst8+z95u/OPxT+Qd6meJfcKCIg71fE9bzvwF/f2aLZ+wIQT5qrQ3tQfrOw/8AUK/4hda4xqbfui3qagSZq33LMtDSnla/32zSgD3aH0lI9dDy8RjXpWwfaaTIlx5Cwi4QJDciNKxzxmXW1dyHG1PrKVJI9QQQQau6WgZTa/HUwf6crXOHe2R9/jZQZah0unuik/MwgH54U97nmNl494rVm+RPFu3WWzImPlP0lBLQISkfNSjpIHzJArmFdrtz911cnyYlnaddiRyX2ICpJbt1njb7UqWT5FZ+atFazvQ0NCWvXvf5Fm6ULVb2CQi+XC1297R/qJZXI/6o6a/Xs1sYg2rg245G2hJmXy+PF1zXn4bKEIQjfzAJcV/zmqjSnM0jTJNVDQZS7hbfl5/X5KZVg1lS2kJs0C5tzUW+UugzmziTFpGeM3KzXuJaWzKmfyS+6JEVCfNToStCe5KfUlJ2ACdaBNSV9n51H5Bybarnxfnl2euV7sEdMyBNfUVvSYPcELS4s+alNrUgdx8yHBv6OzvPPeo3gbBr3OwfPs+t0C4stpTLgyGHl6Q62FAK7UFJCkKB9fQ1jfCWb9Iq7+3i3BrmKs3mQw4Qi3WxTUh1pI7ldzqmwpQGgfiUfSsavVarU9Ocyup3OO7XhpAA6k227YIXsNJFS1IMEgA2Lb7retKUri1dpSlKIuSXXdg8TCeo+/KgM+FGyBlm+JRry73gQ6R+l1DqvxqPlTE9p4uOeZcZbSE+OnGW1LPz7DKkdu/xCv8AWohW+BNus+Na7bFdlTJjyI8dhpJUt1xaglKEgepJIAH319z0GYy6ZDI/+UemPsuDr2BlU9reqkx0A8MHknmFvMbtDLljwoInrKk/A7OJPuzf4EKd/wDTAP0q6o1qzpp4Yh8F8S2nDAhs3RxPv14fRo+LNcA7/P5pQAltJ+aUA+pNbTr5T7Rap/itc6Rp9xuG9hz+Jz2sut02l/CQBp3OT+vJeG+xnJtkuENlPct+K60kfaVIIA/1rmb7NW4xYHUHcIkp5LbtwxmZGYSo6K3BIjOFI+09rSz+hJrqBXL7qD6XOYuEOVpHI3EFqvEuyuzl3K1zbK0t2RbFKJUWXEIBUlKdlIUQUqQQCdkpqx9mZIZoanT5HhplA4Sdri/9R6qNqjXsfFUNFw059F0K5ymx7bwtns6U4G22cauaiSdefuzmh+knQH3moP8Asuozq87zeYEEttWiM0pX2KU8SB/9D+ytT5Vyt1jc62lPH15bym8w31IS9ChWEMeOQQUl4stJJSCAfiPaCNkeW6nH0T9Ol24EwGfJy5LKMnyZ5qROZaWFiIy2lQaYKh5KUO9xSiPLa9DfbszZ6RugaPNTTyNdJKRYNN8AjsevLotMcx1CsZJG0hrQclRY6gf+8VtH+ZcX/wCmJVl6jbtc+AOsvJMxsbSkLltPXCLo67jNgqbWo/cHnHD/AMu/Ws/5x4y5Iu3XpasutfH2SzLE3kGOPLuke0vuREttpi+IsvJQUBKe1Xcd6Had61V49o5w1muW5piOZYPhV7v63rY9bpotVuelFnwXe9suBtJ7e7x1gE+vYfsq2o6uATUkEjhwvh4TnyBz8iFDmhfwTSNBu19x6rWvTXiXg9JnPOdOt798hN2llZHp4KPFcA/T47X/ALRW5vZd/wBA83/W8f8AcmrxgvFGT4v7Pu9YirFronJbzbZ8x61iG572XnHiEI8HXf3+Ehv4dbrGOjS1cmcO8CcqXe4cdZPFvraw/abe/Z5CJEt/3cpb8Noo7lp8Qp2Ug6G/sqDqNU2vpKxrXC7pWgZ3twt+WFvpojTzQkjAYSfjcqM/WLyMeSOovJblHUJMGyvpssJJ2pJajEpXrXqlTviq8vkurrn3WvzXyTg9y49yW2Y2qz3RhMd1ti1rQpCUqSpBQe8hJSpKSPLyIFbk9nxwVnVo5VvfInImGX2ym024swjd7e9GW9JkqIU4jxUgr7W0OBRG9eKN+tdCK2anrlDpkkdGIBL4QFncVrHG2D0BvfdY0tDPVNdMZCzjJuLf3C5qezS5H/kDlG88bzX+2NlMHx4yFH/xcbatAfLbSnif/LTXr9qD9ZuH/qFf8QurZy9xJyvxH1dyOROOONcovNpavbGQx3rVaZEhpaXSHJDHc2gpG1F5Hbv6JHpusy9onx7yFn2e4jdMJwDJr7FRYlJcct9okSA0ovKUEL7EHsVog9p0alMfTv1uDUGOAbKwk5GCG8/hb5LWRI2hkpnA3a70utg9cPCP5wuCLNyJZIffe8Lt7T7vYn4nrcptPjJ+/wAPQcG/QJc15qrn3mPI15zfG8SsN6JdXiNvctUV8q2VxS6XG0n/AAdxQP7qUj5V2vskNDmLwLfcIoUlUBpl9h5HkQWwFJUk/iCDXKDnrpO5NwLlS+WLCOOsnvuOqe96tcu3WqRLbEdz4ktKW2lQ70eaCD5nt3rRFRvZHVInh1HUEXYS5hPQ4I9fXyWzWKV4ImjH5sH7KZnXJicjJuktmdFZW6vHnbZdilI2ewILCjr7Al8k/cCflWOezMz23XPjG+8duymxc7JdFz0Mk6UqI+hACgPnpxCwSPTuRv1FStZsNvvuDNYxkNvEiFPtSYM2K8kgLbW0ELQoeo2CR9tc1uT+lTqA6cM9dzDhpF+uVoacW5b7nZAp2XHZJ34MlpA7joeSj2ltQGzrzSKrSZINSoJdJmeGO4uJhO3b9dfJS6tslNUNq2NuLWIClHzj0I41zZyTdOSblyDcrW/ckR0LjMw23EIDTKGgQoqB8wjf41E7oBYRF6pYUVtzvSzBuTaVf2gGyN1b7/zF1r80Ql4XIczG4R5CfCkRLXYvdS6k+RDqmGkkoPzCj269RUkOiro3zbivKG+WOSpTVuuKIrseFZmVpdWgOp0pb7iSUg63pCSfUEka7TcSGXSdKmp9QqGuJbwsaM2wR0B6bjFt1CaGVlWySnjIAN3EqatKUr5ounSlK1Z1Kc027grim65g86g3R5BhWaOdbemrSezy+aUaK1f3UEepFbqeCSqlbDELucbBYSSNiYXv2C5udcWdN511IZM5Fkh6HYvCskcg7A8BP86PwfU9W8PZ49Njs2cjnvM7eRFilTeNsOp/7V3zSuXo/wBVPmlH2q7leXaknTnSh0xX7qKzFeQ5MJTWH2+T4t1nqUQuc8T3GO2r1K1b2tQ+ik79SkHrBbLbb7NbototMNmJChMojxo7KAltppACUoSB5AAAACvoHtHqzNMo26RSm7g0Bx6C23c8/Luue02kdVTGslGL3Hf+gXppSlfOV0iVqWxdQ9pvl77BhGSRcWecnsw8qcYbVb31QwsvqIQsuNN/zTnY4tISsp0PPVbarQGI8T8w2izDhmbNx+Nx5FZu0VdyYdW7cLjElh4MMllSAlhTZe2tYWe7w0ga2an0ccD2PMxF8bm2LG5HU3tYc7nuI8zpA5vB+tvTfKuEDqms7kBy73zjvKbHb5ljn5DYJM5DHbeYsRgvuBsIcUWnC0O9KHAnafPdeZnq/wAEk/k0I1gvLi8kxu4ZKlGmwYrURuQpbTvxeThMV5A1sbSdmsYncIc3ZnjdsxXM28VhsYVi13stokwZrzirtMk25cFl51Km0iO2ltaiobWe4+XkKx+0dIvIFpvN3uKLhaXWpKbtGgtqkK/2eNKtsxKGx8HkPfbhIUR8knfn6VctptJIPG4B2cBxI5gZ/wCp73GNhCMtXccIx27X+4Wx7f1fYJczh6IlgvKnMws9zvLSCGwYaITchTjb3xeS1GK8lOtjaTvVXfJupfFsYsMXIJeP3Z5mVhf5bJQ14feIvix2/BO1a8TcpB/s/CfP0rVGHdImaWXMhdrndbabeXpDLfY6pS4sR+1T23QhPaASZtxdXrY2kb38q9o4D5pyTG3rXlMTGLfIsuCs4Tavc7i68meUyYzq5ThU0nwUlMVACNKO1Hzo+l0nxW8D/dxfPUn6CwPzRstXwHiGeWOgH1ytqL6jsLduUKHbIc2fHuK8dEaWz2eG4m8OPIjq8zsBHgKKxrY2NbO6q4RzxFznJYtst2A5OxYbsuW3Z8jcYbVBnKjEhw6QsuMoV2q8NTiUhevLzIB1lb+l7Lcczu9zLFcLevGn8rxm9WiM48pK4UKHLlSZUcJCdAJclL8MbPwkAkaq94fgPUbgWLN8b43JxVmxYzbblGtM73lxUm6LcSsQEuoU3qN4SlpU4pKl9xQABomo8tNp/ARA4E4tc2sC29+4dYW235C42MlqLjxAbeQ8/pb7dje2Op+xXfF8wyfE8Kvt8bwq6vwbgxHXHbWqK0hajPbLriQpg+EsDR7yUn4a+MdUFhh20XTL8JyDHW3MckZOyiQY77j8RD0ZltKAy4ra3Vy2whJI8977fKsOxbpgzjj2HdrPZMzTfYGQ4FJxiWielqP7tLQg+5qR4TY8Rvb8kKUvawFAkq9KuWcdO2XZjEtEJq522Gu28eox9L61qWE3VmbAlMkpCdqZ7oRCj66PoazMOl+IGgjgJ3ub2t0735dF5x1fDe2emLX/APPNXe8dVVmxDHsgu3IPHmTYzcMejwZ71rle7uPPwZUlMdEhpTbikKCVq0tJIUkjWt1dMm6kcasj8uDaLDPvswXO22m2txX47TdxemwzLaKHXVpQhHhJUe5ZGyABvYrDMj4b5c5SuU7MM9tuMWu4+DZLVDtcKc5KZVFjXdidLedcW2nzWGdIQEnQGifMmrJG6Yc5xaz5bj1vtuL5fj0/IIsmDZL46pIkWhqMttuN43hqVHdZKmw24nfwteZG9V6yn0wi7yA7oHY/h2N+WeebnItdeGSqv7ox1tnny+XL4ZstzXXmeFZuH3uXbhiF/itxkhL1mlMJYnId95EctkKUE/TOwru7VJ0oHRFWbG+o60XnLIOD3vCcgxy8yLsuzSY9x8AiJJMMy2ApbTi0qDzSV9hSSe5BBA8icfTwXmr3S3K4bmzIartLdK2mPf3nI8KMbgH0RUSFjxVpaZHYlRG9pGvLRr38gdOdticXzrBwpEZsuTM3iHkVunTpr8hSrgwtGlvPOqccUC0Ft6JIAVrWt1HZHpw4o3HJe4A8gMWJztknY3tvjO0uqcOAwACR1Objbf8AVlSmdUTvdaJFi4eyq82/IbpKtFnmxpMFDc2Qw5ISQkOPJUkFMVxYKgAU689nVbNn57BtmY4vhMy2y0T8ohTpjJ+AojiKGS4hw7+kfHSB27Hwnz9N4V+ZqfabFw9jlhXF9149uMeROU4spLraLfIjrWgaPctTrwUd69VH7qrcs4vyVJ5DwjP+ObLZLs5jkS7xJUW53JcIKEsRghSVoac3rwFbGh6itT2UcsjWRAAWfkk7ji4b3NhsOm6ya6ZjS5+Tjl2va3xVvndRdwtmVZHjFw4dyhkYvbXbxOmGTBLSYSUvlt4APFRDhjrCRruB13BNXvjDnCHyJePyduGF33F7o9aWr7CYufgKTNt61BIeaWy4tJ7VKQFJVpQ70+Xn5Wa7cZZxkV0zy/zmLXEk5fx/EsDcduWpxDNxSmZ4qSsoBLQVJQAvWyAT2j0qjxFxvyXCy61ZhyTFsNu/JvE0YpbYdqmuSy8C40t2Q6tbbYTv3doJQAfVWz6VskjojC4gAOAGxN72Gwub5wegWLXTh4BuRc8uV/6LddKUqkU5YzyNyLiXFOITs4za5e5WqAE96wgrWtajpDaEjzUpRIAH4nQBIhRG495M6+eRI3IeZRZuKcU2pSmrSws6flNd3xFoHyK16He7rtToJT3lJqedytVrvMUwbxbYs6MVBZZkspdQVA7B7VAjYPpXpSlKEhCEhKUjQAGgBVrQakNNY50Df804Dj/CPIdT1PLkolRTGpcA8+4OXU+Z6eStWKYpjuD47AxPFLSxbbTbWQxGjMjSUJH+pJOyVHZJJJJJJq7UpVY5xeS5xuSpQAaLBKUpWK9SlKURKUpREpSlESlKURKUpREpSlESlKURKUpREpSlESlKURKUpREpSlESlKURKUpREpSlESlKURKUpREpSlESlKURKUpREpSlESlKURKUpRF//9k=</v>
+      </c>
+      <c r="N2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1.Bill should be address to UMANG COMMUNICATIONS PRIVATE LIMITED.
+2.Xerox copy of the following should be attached along with the bill.
+(a) Purchase order, (b)Necessary supporting document
+3.Terms of payment with in 45 days of the submission of the bill.
+4.In case of any variation or non conformity to your specification, the said bill shall not be eligible for any payment.
+5.Payment shall be process on the completion of job/delivery of materials to our satisfaction only . All dispute are subject to Guwahati Jurisdiction.</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>FIRM-2</v>
       </c>
       <c r="B3" t="str">
-        <v>Umang (Project)</v>
+        <v>Umang Communications Pvt Ltd Unit 2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>18AABCU2874Q5ZH</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Kalapahar Industrial Estate, Bishnupur Main Road, Guwahati-781016 (Assam)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>9865689752</v>
       </c>
       <c r="H3" t="str">
         <v>system</v>
@@ -483,494 +527,1949 @@
         <v>system</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-04-11T08:38:18.325Z</v>
+        <v>2026-04-21T06:43:54.353Z</v>
+      </c>
+      <c r="L3" t="str">
+        <v>U74900AS2011PTC010451</v>
+      </c>
+      <c r="M3" t="str">
+        <v>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/4gHYSUNDX1BST0ZJTEUAAQEAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADb/2wBDAAMCAgICAgMCAgIDAwMDBAYEBAQEBAgGBgUGCQgKCgkICQkKDA8MCgsOCwkJDRENDg8QEBEQCgwSExIQEw8QEBD/2wBDAQMDAwQDBAgEBAgQCwkLEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBD/wAARCACQARkDASIAAhEBAxEB/8QAHQABAAICAwEBAAAAAAAAAAAAAAgJBgcEBQoCA//EAFQQAAEDAwIEAwQDCgoEDQUAAAECAwQABQYHEQgSEyEJMUEUIlFhFTJxFhcjOEJydYGRtCQzNjdSYnOys7UYdHaDGTVVV2OTlJWhsdHS0zRDVpKj/8QAGwEAAgMBAQEAAAAAAAAAAAAAAAQDBQYBAgf/xAA8EQABAwIDBQUGBQIHAQEAAAABAAIDBBEFITESE0FhcTJRscHRBhQikaHwFTRCgeEjsjVSYnKCovEzwv/aAAwDAQACEQMRAD8AtTpSlCEpSlCEpSugyPUHAsPeaj5bm9gsjr3dtu43JmMpf5ocUCf1V0AuNguFwaLkrv6Vw7Vd7TfoDV1sd0iXGE+N2pMR9LzSx5e6tJIP6jXMrhFtV0G+YSvla0NoU44tKUJBUpSjsAB5kmvqoteIZr43o/ojKxizzg1kucJctcNKFbLZiEASn/lshQbB8wp0EfVNSwQuqJBG3UqGonbTROlfoFszSHih0g10ya94rprepdzk2FHVkvmE43HUjn5ApDihsoE+XxA3rbNRH8NLR773egqc2uUXp3bPJAuKiobKTBb3RGSfkQXHR8nhUuKkq444pnMi0GXqo6KSWaBsk3aOeX0+iUpSlk0lKUoQlKUoQlKUoQlKUoQlKUoQlKUoQlKUoQlKUoQlKUoQlKUoQlKUoQlKUoQlca53O3WW3Sbvd58eFBhtKfkyZDgbaZbSN1LWpWwSkAEkmuTVUXiDcYMvVDI5mi+n9xLeHWOSWrlJZX2u8xs9xuPNhtQ2SPJShz9wEbN0VG+tk2G6cT3JGvrmUEW8dmeA7ysj4qvEoyK/zp2C8PcxdpszZLD2SchTMl+hMYH+Jb+CyOoexHJ6wSuVzuV5nv3W8XCTOmyllx+TJdU666s+alLUSVH5k1xqVtaalipW7MY9SsDVVk1Y/blN+XAdFtnhy4js64dM5iZHjlxkO2d15CbxZy5uxOj7jnHKeyXAN+Rwd0n4pJBvHx++23KLDbclsz/Xt92hszoju312XUBaFfrSoGvO/V7nCvbblaOG/TWBdkKRKbxqCpSFHulKmkqQk7+RCVJG3pttVHj0LAGyjU5dVofZud5L4SfhGfRbKut0t1jtku9Xea1DgwGHJMqQ8rlQy0hJUtaifIAAkn5VTll+RZDx4cXsC3w1SWrRdJ6bdbm9u8GzMFS3HNvILLYddIP5a+XfyqQ3ibcUHszP+jlhNx/CvBuTlEhlfdKDspqHuPU+64v5dNPqoVyvCm0W9hs2Qa7XiJs9clGyWUrT5MIUFSXU/JTgQgHzHScHrUVHH7hSurH9oizf3+79FPXS/iNY2hZ2Wm7v24eXUqflptVvsVqh2S0RURYNvjtxYrDY2S002kJQgfIJAH6q5dKVQarSAWyCUpShCUpShCUpShCUpShCUpShCUpShCUpShCUpShCUpShCUpShCUpShCUpShCUr4dS4tpaGnOmtSSEr235Tt2O3rUHOHziozrSbVq8cMvFjkBduTU4iyZNL2Qh8OHdtDi9gOk4CFNrP1SShW2wCZ4ad87XOZq3O3G3Lolp6plO9rZMg7K/C/ceqkvxPZhc8C4fM/yuyqUifCsckRnEq5VNOuJ6aXAfigrCh+bVD1ehHPsMtOouEX3A76kmBf7e/b3ykAqQl1BTzp3/KTuFA+hAqjbXTQHUXh+zCTi2c2Z9tjqrFvuaGz7LcGQfdcaX5bkbEoJ5k77ECr7AJYw10Z7XiFnPaSKQuZKB8IFuh/la3pXKtdqul7ns2uy22VPmyFcjMaKyp11xXwShIJJ+QFTY4b/AAzM6zCZCyjXXnxjHwQ79DocH0lLT5hK9txHSfXclzzHKk+8LuoqoqVu1KbeKz9NSTVbtmJt/AdStacE3CZd+IfN2b/f4bjGBWCShd0kLBSJzidlCG0fUqG3OR9VB8wVJ3sV4weKCycMenITaRFey68NKjWC3bDka2GxkuJHk03uNh+UrZI7cxTytZ9cdGOC/TGJaYNsgxXWY5asGMW8pbckKG/vHzKG+bcreVuSd/rLOxp61c1azTW3OrhqDnlx9quU4hKUIBSzGZTvyMtJ3PKhIPYeZJJJKiSaWKN+LzCaUWjGg7/vj8lfzSx4JAYITeV2p7vvh81wbVb8u1b1Ci2xt9+7ZJlt1S11n1lS5EqQ7sVrV81K3J9Buavl0wwCzaV6e4/p3YE7QbBAahIVy7F1SR77qh/SWsqWfmo1Wz4WWjQynU276wXaJzwMQj+yW9Sk9lXCQkgqHoemzz7j0LqD6VNvVrjP0H0SzJ7A8/vtxi3dhhqStti2uvICHBuk8yRt5VFjD31EwpoRfZzsPvgPFTYHGylgNXObbRsCe7+T4LedKwvSTV3CdbsOazvT+bIlWh6Q7GS4/HUyrqNnZQ5Vd/M1mlUDmuYS1wsQtKx7ZGhzTcFKVoHUzjj4e9I84uenma5Bc416tBaTKaZtbzqElxpDqdlpGx9xxJ7VtbTLUjFdXcHtmomEynpNlu4dMV15lTS1Bt1bSt0K7j321DvXt8EsbA9zSAeKjZUwyPMbHAuGovmsopWidVuNXQPRfNJeAZ5frlFvMJtp15pi2PPICXEBaNlJGx90iutwTj24btRswtODYzk9ycut6kpiQ0P2t5pC3VfVSVqGw38hv6kV7FJOW7YYba3sozW0wfuy8X0tfipEUpWr9b+JHSjh5Zs72p15kwvp1T6YSY8RyQpfRCOoSEA7AdRHc/GomMdI7ZYLlTySMiaXvNgOJW0KVFr/AISvhR//ACu8/wDcsj/21Ju2XGLd7bEu0FRVHmsNyGVEbEoWkKSSPTsRXuWnlhtvGkX71HDUw1F904G3cVyqUrUGtfFbovw/Xi3WHUq/Sok+5xlTGGY0JyQeiFFHMrkB5QVBQG/nyn4V4jjfK7ZYLle5JWQt25DYc1t+lae0V4sNFeIC9z8d01v8uXcLbFE15mTCcjno84QVJ5wObZSkg7eXMPjW4aJI3xO2Xix5ojlZM3bjII5JSlRiuPiOcLVruEq2TMovCZEN5bDoFmfIC0KKVDfbv3Br1FBLNfdtJt3LzNURU9t64C/eVJ2ldfj1/tGVWG3ZNj85uZbLtFamw5DZ911lxIUhQ+0EGuwqIi2RUoIIuEpUZp3iK8L1uvEixSsnu6ZcaSuI4kWd8gOJUUkb7bEbjzqTNSyQSQ23jSL96iiqIp77pwNtbFKU8qjpqnx98NWlVwk2SZlsjIbrDJS9DsEb2rkUPNJeJSzzA9iOpuD5gVyKGSY7MbSTyXZp4qdu1K4Ac1IulQog+K/oE/JDU3Cs7itK7dX2SIvb7QJG+32b1IzR7iO0a13jOOaa5rFuMphHPIt7qVMTGR8VMuAKKdyBzpBTv61LLR1EI2pGEBQw19NUO2Y3glbLpSlLJtKjNxy8LEXiF07XescgtjOsaZW9anEgBU1kbqXDUfXm7lG/1V+oClVJmlSwzPp5BIzUKGogZUxmKQZFVF8N/iI6maJxmMK1EgP5jjUMhhpEh4t3G3oT25G3FA9RKfRtzy2ACkgbVO/E+NDhK1etAgT9QLHDTKQDItmUtJiBPryLL46Kz+atQ+dQX8Sfh9a0v1Va1MxyGGrBna3ZDyEJ2RGuSdi+n5BzmDo+Ki7t2TUPK1PuFLiDBUM+Enu71jxiVXhchppPiA7+7r/6rxW9buD3TGI7crPqHphZ0P8A8Z9CyoanHdviiNutXp6Go1a8eKdjdviSbFoBY3rpPVu2L7dWC1FaH9NpgkOOH4dQIAPmlQ7VWfSvUWCwMdtSEu6rzNj9RI3YiAaOWq7rM81yvUPJJuX5tfpd4vFwX1JEuUvmWo+gA8kpA7BKQEgAAAAV07bbjziWWW1LcWoJSlI3KifIAepr5qT3h56JnVvX6BernD6thwkIvU0qTuhchKv4K0fTcuDn2PYpZWKsppGU0RedAFUwRPq5hGNXH7Ksy4TtGG9CNC8cwd+Olu7OM/SN5UPNU94BTgJ9eQcrQPqGxVbfiZ/jUXP9D27/AAzVwlU9+Jn+NRc/0Pbv8M1mcHkdLWOe7Ug+IWtx2NsNA2NmgIH0Kmt4ZX4rNv8A01cP74qV1RR8Mr8Vm3/pq4f3xUrqrq/81J1KtMN/KR/7R4KlTxAvxvdQf7W3f5dGqyTw+/xQdP8A+zuX+ZSqrb8QL8b3UH+1t3+XRqsk8Pv8UHT/APs7l/mUqrnEv8Oh/wCP9pVDhP8Aik3/AC/uCr18ST8bLJP9Qtv7q3Ue8GyeVhGa2DM4XN7RYbpFubQB2JUy6lwD9qakJ4kn42WSf6hbf3VutQap4b9zdk0+yBtrZrKcWbuBWB2LrcqRGUPtCWGyfzhVvRke7RtPEDwVJXB3vcr28HE/VX0wJsW5wY9ygvJdjS2kPsuJ8loUAUkfaCKqo8VTNfpzXey4cw9zMYzYm+onf6smS4pxf7WwxU9uDTNfu+4YtPr4t7qPR7Si1vkndXUiKVGJV8z0gr582/rVTfErf5mr3FNmku2K9oduuSqtMA77hxDS0xWNvkUto/bVFhEGxVv2v0X9PVaPHKnbombP67fK1/Rabr0IaffyCxr9Dw/8FFUR622KHi+s+e4zbk7RbRk90gsDbbZtqW4hP/gkVe5p9/ILGv0PD/wUVNjztuONw438kv7ONLJJWnhbzWQVSNxv6nffU4lcuu0eR1bfZ5AsUAg7pDMXdCik+qVO9VY/Pq3fiD1Kb0g0WzDUQupQ/aLY6qHzeSpbmzcdP63VtiqXuG7Tp3WLXrDcHlIVJYul2beuPN7xXFa3ekbk+pbbWNz6kVHgkYYH1LtALeZUvtBKZDHSM1cb+Q81kPBfqj96XiPxDIJEjo264S/oa4knZPs8r8HzK/qoWW3P93V4VUM8SGmy9H9dcywFpksxrbdHHIA8tobuzsfb7GnED7QauW4ZNUBrFoRh2fOvh2bNtyGLgd+/trJLT5I9N3EKUPkoV3G4w9rKlmhFvMea57PymN0lI/UG/kfJbQrz1Z1/LbIf0rL/AMZVehWvPdmbLknPb7HZTzOO3eUhA323JeUBXfZ/tSft5rz7TdmL9/JWP+Fvr590WIXHQfIZvNcMcCrhZStXdyAtf4VofHpuq3H9V0AdkVPKqCtLNQMq0B1dtOawoz0e7YvcSiZCd3QpaUktyIyx6cyStB+G+/mKvdw/LLHneK2nM8amCVa73DanRHR+U24kKG49FDfYjzBBB8qWxml3M29b2XeP3mnMBrN/BuX9pnhw+WioQy/+dC9fp+T+8Kr0D15+Mv8A50L1+n5P7wqr/Lrc4lltcy8T3OnFgR3JL6/6LaElSj+wGmcdzEX7+SU9nDYzE8vNV8eJDxcXiz3F7h602u7kNYZSrJ58ZZS4Q4ndMJCh3SCghThHmFJRvtzgwr0V4dNW+IC6PW7TXGFzGYhAmXB9wMw4u/kFuq7cx/op5lEd9tt6xPKcgvupGc3TJrhzyrvklzdluAHcrefcKuUfrVsB9gq9bQzSax6JaWWDTmxR2ki2RUe2PITsZUtQBefUfUqXue/kOUeQFMzytwembHGPiP2T6JSnhdjtU+SUkMH2B6qsbJ/C84lsfsq7tbn8SyB5tPMqBbbk6JB7bkJ67TaFH5c+59N6jLYr7mulGbMXqzSbhj2S49MPKSlTT8Z9BIUhaT3+KVIUNiCQQQSK9B9RE4i/DzxnX7Vw6mN5svGGpkNpq6RotuD7kyQ3ukPBZcSlBLfTSfdVvyb+ZNL0mNbRLKq1u+30TVdgGwA+jvtA6X+t1u3hu1nha+aO2DUhhptiXMaLFyjN78sea0eV5I33PKSOZO535Vp371s6tV8O3DviPDXhsvC8NvV7uMWdNNxfXc3m1qD6m0IUUBtCAlJDae3c9vOtqVQz7veO3XZvktHT7zdN33atn1SlKVEplpLjL0nb1i4d8rxxmMl2526MbzajtuoSowKwlPzWjqNf7w1R5XovICgUqAII2IPrVAetGIt4Dq9muFMNdNiyX+dCjp/6FD6w2fsKAk/rrTYBMS18R4Z+qyXtLAA5kw45Hy81hlKUrRLLpV1HAroV94/Qe1sXWH0cjyflvV35k7LbU4kdFg+o6bfKCPRanPjVcnAfoKvXDXO3uXSD1sZxNSLxdypO7bhSr8BHPoeo4O49UIc+FXR1m8dqtKdvU+Xr8lq/Z2j1qndB5ny+aVT34mf41Fz/AEPbv8M1cJVQvifwlReJ9x9W+0zH4DyfsBcR/wCaDSmB/mv2PknfaH8n+481MzwyvxWbf+mrh/fFSuqJHhfzWZXDA2w0sKVDyCey4N/qqIbXt/8AqtJ/XUt6SxD81J1KsMNN6OPoFSp4gX43uoP9rbv8ujVZJ4ff4oOn/wDZ3L/MpVVp8ectqbxbahvMq5kplxGif6yITCFD9qTVmvAXEVC4SdPGVeaokt39S5r6x/eq4xPLD4R/t/tKocJzxOY/7v7gq7PEk/GyyT/ULb+6t12/EJhvtHBFw+agtNbewG5Wd9YHmH3nHWwfs9nd2/ONdR4kn42WSf6hbf3VupG3vDfuy8KO09Jrnk2O3pvLHbfl6Nwc6p/6lTtNbzdQUzuYHzBCT3W+qKtvJx+TgfJfh4dmsjWK8LmqiZj6VOafrlX5tKj5NOxCtCAPm7Gd+0qqJvBXiTuoHFTgUKUFPpjXU3qQtff/AOlQqQCr7VtpH2qrCNPtVLjgmFah4dE6nSzmzx7cpSD9RbUxl3mPyLQkI/3lSr8JzDfpPVnLs5da5mrDY0QkEjsl6U8CCPnyR3R9ijUk8fukdRN/m9LeJXinl99kpoP8uvzv4AKL3En+MVql/tpe/wB+eq8rT7+QWNfoeH/goqjbiT/GK1S/20vf789V5On38gsa/Q8P/BRVdjX/AMIenkFZYB+Yn6+ZUJ/Fh1O+jMJxPSWDI2evkxd4npSe4jxxyNJUPgpxxSh82a194Tmmv0lm+XarTI+7Nkgt2iEpQ7F+QrncUn5pbaSD8nq0Rx3anffR4mcqmRpHVt2PuJx6DsdwERt0ubH1BfL6gfgoViulnFLrvopjz2K6YZ19CWuRLXOdYRbIb5W+pKUFZW60pR91tA232G1PR0Un4eII7Bzszfnn/Cr5a+L8TNRLctabC3LLxzUpfFj0z+jsyxDVmFH2avMNyzTlJHYPsHqNKV81NuLH2M1lHhM6o+0WvMdG50ndcRxGQW5BO56a+VmSB8AFCOdvi4o1DPVLio151pxxvEtTs7+m7UzKRNbYXa4TPI+hKkpWFtMpUDyrWPPbZRrn8HuqP3ouIrDspkSOjbpE0Wq5EnZPssn8EpSvkgqS59rYrr6KT8PNPJYuGluWY9FxlfF+JCpiuGk5355H1V5Vefe//wA6Fx/T737wa9BFefe//wA6Fx/T737waQwDWToPNWPtLpF1PkpX+JzoF9wmpcXWOwQuSy5qoon8idksXRCd1E+g6qBz/NSHTW0vCx18+kLTdOH7IZu79uDl2x8uK+swpX8IYT+atQcA8yHHD5JqYfEDo/atdtJMg02ufTbcuMcrgSVjf2Waj3mHfjsFgBW3cpKh61STh2TZpoDq5ByGNHcgZHht2Ul+K6eX8I0soeYXt+Soc7atvRRqWkIxKiNO7tN08vRRVrThNe2pZ2Ha+fqFwsv/AJ0L1+n5P7wqrwuI511jh61PeYUUuN4belJIOxBEJ3uKovud1avmbS72w0ptu4XVyUhC9uZKXHioA7eo3q/3Msdj5fiF8xOXt0L3bZNuc3HbkeaU2d/1KrmNHYdCTwv5LuADeNnDeNv/ANKhnRZqO/rHgjEsAsOZNa0OA+XIZTYO/wCqr/q88UORdMPyZiUphTFysk9LhbcGxbfZc35VD5KTsa9AeF5ZaM7xGzZpYHw9br5BZnxlg7/g3EBQB+BG+xHoQRXn2gabxv4Zr37NOFpGccvNRF4v+O7N+HDVdnT7HsIsd2iuWiPcTImuvJcC3FuJKdkEDYdMftNaQ/4WvVT/AJrMU/6+T/7qlVxE8CWBcR2ft6g5Lmd/tctu3s24MQUslsobUtQV76Cdz1D6+gqA3G5wo4lwuy8Pj4rkt3u4yNuct83ANAtFgsBPLyJHn1Tvv8BRQNw+drInNu+3NcxJ2J07nzNdaMHLTRTy4JOLPKeKRvMl5Ni1qs33NG3hn2Fbiur7R7Rzc3OT5dBO23xNSgqurwhP4jVb8+x/+U6rFaqsSiZDVOZGLAW8ArnCpnz0bJJDcm/iUpSlIqxSqQeN9huPxW6jNtEFJuiFnb4qYaUf/Emrvqof4o8iRlXEXqPe2VBTTmSTmWlA9lNtOlpCv1pQD+ur7AAd848vNZz2lI3DBz8lq+vpttx5xLLLaluLUEpSkblRPkAPU181Mvw3uGpWp+of33cqgFWM4ZIQuIlxPuTboNlNp+aWgUuK/rFodwVVo6idtNEZX6BZSlpn1crYWan7up28F+gDfD9opbbJcYqUZLe9rrfV7e8mQtI5WN/g0jZG3lzc5H1q3xSlYKWV0zzI/Ur6TDE2CMRM0CVW14sul9yF6w/WOHGU5BXDVj09xKTsy4hxbzBV+eHHhv8A1APUVZLXR5vhGK6jYrccKzWzMXWzXVroyorwOyhuCCCO6VAgKSoEEEAggipqKp90mEvDj0UFfSe+07ob2J06qn3g34xblwwXS52u7WV++YlfFoelxGHQh+NISOUPs83uklOyVJO3MEo94cveX2X+K5oxCsLz2EYXlV0vK2z7OxPYZix0L27dRxLq1bb7dkpO/fuPOtXaneE5l7F1ky9IdQrTLtiyVsw791GJDQ/odVpC0uH+sUo+z1OAW/wteJaXLSxLnYbBaJ95926OqSB9iGVKP7K0Ev4ZVv3z3Z9bLMxfi9EzcMblwyB+R9VF3Ir7k+p+cT8hufVuV/ya5LkOJaQSp6S+5uEISNz3UoJSkfICr3NEsDc0v0hw/T59SFSLFZosOSpH1VSEtjqqHyLhWR9tR94WfD3wvQi8R88zS8N5Zlsb34agwW4VuXt9dpBJLjnfs4rbbzCUnvUuKrsWro6nZih7LVa4Lh0lIHTT9p33n1VN3iSfjZZJ/qFt/dW6n9woYxGzbgYxrDZnL0L9jlxtrnMNwEvOyGz/AHq1dxTeH1m2v+st01Nsuf2S1RLhHispjSo7y3ElplLZJKe3cp3qUHD3pjcNGtGsY0yutzj3CXYYzjDsmOlSW3Cp5a90hXcdlgd/hXqsq4n0cUcbvibb6BeKGjmjr5pJG/C69udyqGJkSTb5b8CY0pqRGcUy6hXmhaTsoH7CDVrHhVYZ9CaD3rL3meV7Jb87017fWjx20Np/Y4X613ql4W+Y5pqTlGYY7qPYLfbb7d5VyjRH4rxWwh51TnTJSNvdKiBt6AVNTh90qGiOjmMaXqmMy3bHFWiRIZSUoeecdW64tIPfYrcVtvTOKYhDUUwZG65JF/vqlcHwyemqjJK2wANj98lSzxKfjFapf7Z3r99dq4/M9R2NI+GKTqM8tCV2TFGHowX5LlKYQhhB/OdU2n9dRD1V8MHUHUHU/Ls8ham49Fj5JfZ92aYdivlbSJEhbqUKIGxICwDt8KknxMcO+ca2aHWLR3F8utlnER2Gq5yJTbikyW47RSltIT32LnKvv/QFRVtRT1O5ZtZDX6KSgpaqk379jM9nTM5qn7TTDbnqvqfjuEMuuuS8mu7ERx4nmUkOuDqOknz5UlSyfkauAHADwiAAfeejnb1N2uH/AM9ak4VPDzvug+r8LU7L81s97Ra4clEKPDjupUiS6jp9QlfbYNrdHx3Iqb9eMUxEySNFO82A4XGalwfCxFE41TBtE8QDko+f6AXCJ/zOxv8Ava4f/PVRWuOnT+kur2W6dPJWEWO6PR4xX5rjE87Cz+c0ptX66v4qF3F1wB3jiG1Sb1JxHMLTYlv21mJcGZjDiy880VBLoKP+jLaNj/QFcwvETFKRUPOyRxuc13F8LE0INMwBwPAAXC31wr6o/fh0Bw3OH5HWnvW9MS5KJ3V7YwSy8o/DmUgrHyWKpOv/APOhcf0+9+8GrguDPh0zrhoxC+4VlOX2y+2+fcEXGAIbbiDHcU2EPBXP6KCGiNvUK+NReuPhW6jTctlZGjVLG0tSLiuaGzFf5glTpXy+W2+x2qagqKalnl+L4Tp9UviVLVVlPD8HxC99OXirJ6q98UbQP7mczt+uuPQuW25MUwbyG0+61cEI/BuH4dVpO35zSie6qtCrCtZ9LbHrTpjkGmmQAJj3qIppt7l5jGkD3mXkj4ocSlW3rtt5GqqgqjSTiThoeiusRoxW07o+Oo6/eSoNtn/GUT+3b/vCvRPVY0TwmNSo8pmQrVfGSGnErIESR32O/wAKs5qwxmqhqdjdOva/kqzAaOekEm+ba9rfVVF+I1w63HS/VqVqhZbes4rm8hUtTqE+5FuSt1PtK28uc7up38+ZYH1DXE4RuPXIuHm2DAsws0jJMMDinYzbLoTLtqlHdfR5vdWhRJPTUU+8SQobkG2XMcMxbUHGp+H5pZIt3s1zaLUqJITuhafMEEd0qBAIUCCkgEEEA1X9qz4Tsp24P3HRTUKK1FdUVItmQpWOj335UyWkqKh6AKb37d1HzqalxCnqIBT1nDj96FQVmGVVLUGqoePDx6hbCyHxXdC4VqMjGsLzG6XFSN240liPFbCtvJbodWR9qUqqAfEdxL5/xL5VHyDMkxIcK2JcatVsiI2ahtrIKvePvLWrkRzKJ78o2CR2rc0LwtOJWTNTGkz8MiMlWypC7o6pIHx2SyVH9n7KkHo34VuBYzNZvWsOWvZY80oLTa4LaokLceji9y66Ps6fz3FTxyYbQf1Izc/M+iWljxbEv6cgs35D1K6XwjbBeoWP6kZFLtclm2XORao8KUtshuQ4wJXVSg/lcvVb328uYVYNXDtFotVgtkWy2K2xbfb4TSWY0WK0lpplsdglCEgBIHwArmVn6uo96mdNa1//ABaeipvc4Gw3vb1ulKUpZNLEtWs8haX6ZZRqFPWkN2C1yJqUq/8AuOpQem39ql8qR81CqAJMmRNkuzJTynX31qdccUdytajuSfmSas18VTWoWXD7JobaJQEvIVpu13Sk90wmV/gUKHwW8kq/3HzqtC02m5366RLJZYD864T30RosZhBW486shKUJSO5JJAArW4HBuoDK79XgPsrFe0NRvqgQt/T4n7Cy3RfSHLNctRbVpzh0fml3BzmekKSS1Djp26j7hHklI/WSUpHdQFXnaWaa4xpBgNm06xCL0bZZo4ZQSBzvL83Hlkea1rKlKPxUdthsK1BwWcLEHhu09Dl6ZYfza/oQ9epSSFBgeaIjav6CN/eI+svc9wE7SKqoxWv97k2GdkfU9/orvBsN9yj3kg+N30Hd6pSlKqVdJWttbNfMH0JtdtlZSzdblcr5IMS0WWzxParhcXgAVJaa3G4G6dySAOZI8yAdk1F3VabDsfHXpDdcqktRrVMxm7QbQ9IWEtJuRJ5wCewWptbaR8SpIHc0xTRtkfZ2gBPWwulqqV0Ud2ZEkC/dc2uthaacU+lmpGI5PlheueM/cSFHI7dkET2WbawEqUFOtgq7EIXtsSSUkbb9qxHB+OzSbNMns2PysYzfGoeTSPZbBe77Z/ZrbdHSdkpZeC1d1HbbcAdwDse1a94xMt04znRnXewaW2+M9lmP/Qpyy4QoKUmS0JDKghcpA/C9NttaVJKt0dNY27GuXxq5ZgeT8K2NW3T26W+TOyK6WRGFsRHkKc6yXUchaSDuORvmQf6JUEnYnanY6aJ9rtI2jbXs5A30z1+QSElXMwOs8HYF9O1mRbXLS3UrdeL8TOnmWa6X/h7gRbwxk2OxlyZDshhtMR5KekSlpYcK1K2eSdigdkq+HfCrXx56LXnAM51Jt9ryl2z4BLhxLiRDY6j6pT5ZaUwOvspPMNyVFJ2I7E9qiZrPkk/SXX7UzXi1trVIsOUv2BXT81G4WB0MlX9VLzCFb+h+2unRhv3AcPHEHiC2um9ARpyJKdttpC0Rlvf/ANFrphmHwkNcb57P1IDvEJV2JzguaLZbfDuBLfqDfopu55xq6PaeaU4frBeIuQSbPm//ABbHhxWVyk7IKl9RCnUpTykcqtlK94jz862Jjmr+L5Pqhk+ktvi3JF5xOHCmznXWkCOtuUjnbDagsqJA890jY+RNVb6swp0zGc50jlxnEW/QVq+CCtQ90+35BEQzt9rC1kfAdqm5pjc7bZ+OLWCPdbhHiOTsXsEqOl91KC601HSlxadz3CSRufSoZ6GKOMubrYn6tt9CpqfEJpZQ11rXaPo6/wD2asouHGto9aMFt2ot1i5BEstxytzEOq7FZ5o8pvm53nAHTswAhR5gSrb8ms5yfXLD8Uzx3T24Rbo7cWsVlZgXY7TamDBYWULSFFYJcJHYcvKR+UKgJAxS0ak8PmmuL3RS12fLtdZcUvMq2K474fb50K/bsfiK7TS/Iswe1iyDTPUJpw5JpjpHkOJy5KvKayy8FxpCd+5CmHGu57nbm/Kr26gizI4Xv87D+V4biU1wHcdmx52uR6dCpdX/AIwNLMf0yxLUtcDIppztJ+56wwoCX7tOUDspKWUrKfd7bnn295I3JIFZLohxA4Rrzbrq/jEW72q6WCSmJeLLeYns0+A6oHlDre5ACuVWxBPdKgdiCKh/w9zYdj1M4YrplUlmNa5unNygWd6QsJbTc+u6XAknsFqaUhI9TzJA7mt96m8Qmj+GYzrjlOAMQU5hiEKPHvFzjQUJEq4PNdGChUlI/DFtZSgpJ3RyKGw2qCalY07uNpJPHh2rW++KYgrXvG9kcABqOPZ2r/fBZXg3FbplqOzqOvD4d+uL2mZe+kYzMRC3p4b62yoSEuEvBZYWE78pJKdwN6wzG+PbT7KMtRhNu0h1cRdRIjR5TT2NIHsPXIDbkgB8qaQQebmI+qCRvUa+F+/vaO636UQpWled4XDyTG1YbfpWR2VyDHuN3W6uU08wtX8YpTyumN9lBBT28xUl9HPx3OIX9H4t+41JNSwwl/w3FrjPmB/KjgrJ52s+IAl1jlyLv4WWO8XOkUTTLINV7q9dbfZ8ev0jGnGpEZBky57JA6cdtC1c/NvuncjslRVygE18aQcWeAat5arT9eM5bhuTqimdFtWU2v2J6bGHcus7KUFgDc7bg7BRAIBIhlZJEGz2vBcnyhaG8VtfERdzc3njsww6rplh1zfsEpKXCVHsADUkeIG7Wi/cVvDvZ8UnxpeRQp90nyjFdSpbFsVGTzlwpPZDiUrCd/PZW3n35JSRMOwAcw43vpYfd+q7HWzPG2SMi0WtrtH+cuhWfYpxb6U5npNlusNlbvKrVhTkhq7QnI7SZyC0AolLfUKSFA7pPOAdiOxBA42onF5gmBSbDaYOGZtl16v9layJFpxu0iZKiW5we6++kLAQN9x2J7jvsCCa92oN80f4fZuplpakSMY1Yg37EsiZSSUx7kzMkKgSdvmlKm/gAFnuVAVJu8Yg5meeYfJ0R1ud0/1esunFqEuNOg89vutsKELRuVgpVyrUeYhDgGw7Ap3qV9DBG6/6bn6W1tz8lDHiNRKwDR1h3Z3zyuQDlw6qWmleqOIay4LbdQ8GmOSLTc0r6fWb6brS0KKFtuI/JUlSSCO49QSCCdHXPxBtH7NdLxEuWE6jNW2w3Z6zXG+JsSHLbHkNOdNfM8h0nbcg7cvNspPu7kCsj4KtQZWoejj8u5Y7j1quNnvs+zzl2CMhiBOfZUkqlNJQAnZYWN1DsVAkbAgCMWmem3Ejq9iOsWm+nt8wK0YFftRr7Fu8u5tyXLqhZdaLvRSgFooKA2Bvsd+b3k9iF4qaISSCXINI48+mfyTM1XMYo3Q5lwPDiB3Xyz5qa2Da44VqDn+UacWJM5NzxaPAmvOvttiPNjS2uqy/GWlai4jlKdyQnYqSO/fbVt848tMbNbbhfWNPNSbtZrbc7hbH7pbbI0/ECoZQHXep1wEtHnBSpXLuArcDatV8Rc9vg81Nw3U+xKfVbbhp1cMGcdKdyqZCjBy3rc2/KW4lpG/olCvQd82GnatLvDiu+KSGi3O+4SbPnhX1/apLS33Qo+pSpwp+xIrop4QGvIuHWAz6g/XxXDVTuL4wQHMBJy6Fv0v8luDQziDx/XyJcbhjuE5pYosBuK82/kNqTDbmtyA4ULjqS4sOpAb3JHYBaPPeu9wfVrF9QMrzLDrGzPROwae1brmqQ0lDanXEFaS0QolSdgdyQPsri8Pn8wemv+yFm/cmq09w1XO22/XziNTPuEaMV5TBKQ86lHN/B1eW570sYmOMhaLbOnzATTZpGiION9rX5Er9sh499PsayxWFXDSDV1V1U/IYistY0gmaGCQ44wC+FOoAHNzAeRBO1czKOObTzFr83jT+mep0+4fQ8G9yWLfYEPLhMSmUuoS+nrBTa0hXKsEbBQI3O1cXVpxt7jb4fnmXErbXasmUlSTuFAwuxB9RXHwq5221cdmrci6XCNDa+5KynnkPJbT2AJ7qIFMCKDZDtg9m+v8AqsljNUBxbtjtbOn+na71vbTDU7DdYcKt+f4HdPbrRcUq6a1IKHG1pJSttxB7pWkggg/aNwQTlVRh4DVMy8Y1TvNnKTjt01PvsuxKb/inIZLQStv05DtsNu24NSepKojEUrmN0CfpZTNC2R2pSsZ1J1CxvSrBb1qFlsv2e12OKqS8RtzOEdkNoB81rUUoSPVShXcXy+WbGrRLv+Q3SLbbbAaU/KlynUttMtjzUpSuwFVL8Z/FTeuKbOIGl2k0W4zMTgywiBGjsLL97mn3Q8WgOblG5DaCN9ipR2KtksUNE6skto0alL4jXtoYr6uOg5+ij1qvqTlmump92z2/JdkXS/zB0IrILnSRuEsx2h5kJTyoA23O2/ck1ZXwIcEyNHYTGrGqNuQvN5rJ9hguAKFmZWNjv6e0KB2UfyASkdyrf74K+A23aNJh6n6qsMXDOFI6kOFuHI9m5h6HyckbHYrHup3ITv8AXMzafxLEmub7tT9kZE+Q5eKrMKwlzHe9VWbzmB3czz8OuilKVRLRpSlKEJWHao6Q6ca0Y79yupmKxb3bkuB5pDqltuMuAEc7biClaFbEjdJG4Ox3FZjSvTXOYdppsV5cxrwWuFwVg2nWiGlWlGISsEwPC4Fusk/n9tjK5n/a+dPIrrKdKlO7p93ZRI27eXasTwbg94cNN8zGf4fpjBh3ptwux3lyH30RlnzUy04tSGz37FKQR6bVuWle9/Ln8Rz1z16qP3eH4fgHw6ZDLp3LWmTcN+iuYx8ki5Lg7M5rLrhGut5SuZJT7VKjp5WnPdcHJyp7bI5QQTuDX73/AIfdIMoay1m+4ciSjOnoMjIE+2yUe2uQ+X2Y+64OnyciezfKDt729bEpQJpBo4/Pp6D5BdMER1aPkOfqfme9a1v3DjotkzuZv3vB2ZDmoIiDI1CZIQZwiqSpj6rg6fKpKSeny8xHvb1xNXOF7QzXKdBuupmCs3SdbmRGYlty34zwZBJDalsrSVpBJICt9iTttua2rSgTytIIcbjn+3gFx1PC4FrmCx5Dr4kn91qXOMN4dtLNPcclZrb7VjuJ6dXFi6WXmfeabhTUFXTWlLauZ5wlxZ5VBZWVEkE960/cuJLw9btm1x1Gn5vAXkd3szmPzpyYN1Qp+AvsppSUthBJAA59ucAABWwFdD4sSlDQLGUhRAVl8fcb9j/ApdVT1e4dh7auHeve65voVncUxN1FPuY42kCxzH/mgVsV/wBa/DYyjTW2aR33JrXLxaypAtsNcC7FyJtv3bf6fVSfeO559yDsdx2rh27VXwyLTgLWmMC/2xnG27i1dlw0w7wC/Lb+o685ydR7bt7q1KT2HbsKr24arNaMg1vxez322RbhAkvPh6NKZS604BHcICkqBB7gHv6is40sxTGLjfNbWbjj1tkt2e03N23peioWIi0OOBCmtx7hAA2I222qhxjF6XBp56Z+8O6bC82cM99K6IWy1BFye5M4d7xiTY5GtjG24x5tPBod36WysrAc84suA7U2HbIOb6jxLk1ZrmxeYH8BurK481nm6byVtNJUCnmV23279wa+7Pxb8CVgzXINRLTqTEj5DlLcVq7zfYLooyUxkdNkcimihHKnt7qRv67moYZJorh+WaLYTccWs0CLllssUK9zGWI6ULucNXKl9S9h+EWkjm3O577flVzMowzBrJkWuUqJg2PKRjlrtEu2x3Lc2WY6y0VL5EgDlCyPe5dt6y0Ht3hNS0RwskL7lpaS0EHfRRDho4yteDpYHiFc/hmI3Ejt3YhhBsf1Me62urQ0g8nA6FSoY4gvDmYwu96efdVaXsdyOe9dLnAk226PofluqSpbu7jRUhXMlJHKRykAp2rrdItYvDU0LmS7npjk9ttU+agtPTHIN2lP9MkEtpcebUpKNwCUpIBIBO+1RNl53jzHD7C1XRonpibvJv6rUtk48PZg0EKVuE8/NzbpHfm2+VRrtGO5LmNxfj4vjU+6SQFPrjWyG4+W0b+fIgEhIJA/WK1mA1rcXgqJaproGRvcxxdI0guYS12gtYECxOt1SYjO6hdCYQyRz2hzbMcCAb248jkFaovXrw43dL39GXcut7mGyXlyHLYuHd1AuKf65UHS31Unq+9uFjbyHbtXValaqeGXq5CssLPMkt88Y9ERAtzzcS7sPsxkDZLJdbbStaB6BZOxJPmSarXwGxuNaq43juR2haFfT0KLNgzWCk7F9CVtuNrHwJBSRW/tZcIw206b6o3C14paIkm3ZsxDhvMQ20LjsFiOS02oDdKN1KPKO3c/Go8UxijwjFafDf6jnTbJDg4WG28Mvp+57wvdEKnEKSacsYBHcEFp/Sx77a/6CLcCVOTBuMLgW01xeDheC6i22z2W3JKY8Ri03HlTuSpRJUyVKUSSSpRJJJJJrudDtfeDj6clYHozndtauWVXeReHYjiZrZmXB/l6ikqlJA51cidm0kDt7qapXrNNEVKRrRgK0KKVJyi1EEHYg+1t1qZMFiDHEPdfqPrkqmLH5i9rSxthlochyzyV5mp+kOnOs1liY7qZjDN8t0Gai4R2HXnWgiQhKkpVu2pJPurUCknlO/cGu6yrFrDmuNXLD8ngCbaLxFchTY3UW2HWVp5VJ5kEKTuD5gg121Kyu26wF9NOS2O7Zcm2uvPquBj9itWLWG24zYYgi2y0RGYEJgLUvpMNICG0cyiVHZKQNySTt3JrUGZ8FnDLqDlFxzTMNMW7hebs97RMlG6zmy65sBvytvJSOwHkAK3dSvTJpIztMcQeRXmSCKVobI0EDvF1hcTRrTaDdsOvsXGkonYBbl2nHHfanz7DEWyGVNgFezm7aQndwKPbfffvWKajcJPD1q3lb2cah6dN3e9yG2mnZSrlMZ5kNpCUDkadSjsAB5d/Wtv0rrZpWHaa4g9Vx1PE9uy5oI6Dp4LqsWxXHMIx+FiuI2WJabRbm+lFhxWwhtpO5J2A9SSSSe5JJO5NdrSlRkkm5UoAaLBRR4zeFzWniXv2PWvFtRrRZMJt8fedb5bj4W5MLit3+m2god2b5AkLUnlPPttzE1mvDNwd6ZcNVvMu1I+ncqkIKJd/mMhLvKfNthG5DDfxAJUr8pRAAG+aUwayYwiAGzeXmlRQwCc1BF3HieHTuSlKUsm0pSlCEpSlCEpSlCEpSlCEpSlCEpSlCFD/AMUHDsny3h8tj+NWWXchZckj3CciM0XFsxvZpDZdKR35QpxAJ9N9z2BNVO/QV7/5Gnf9nX/6V6IqVcUWLGji3Wxf97eSo8QwUV02+27Zd1/MLz+YDdsu09zG1ZpaLFJcl2p8PIbdjL5FjYpUk7DfYpJH662tfNbbYiy5SzgOhsnHrxmzK2LxPXOfkp5VklYabKAE83Mo9tgCfI7CrraVVYnT4Zi9Wytq6cl7dkZSPaHBrttoe1pDXhrviAeCAVNRUNXh8boqeewOebGmxta7SblptlcWNlR8zrjmtuvOn17smGTobuDWpFodQVrWm5M9gsKHTHIFAeXvbHY99q52Q69Xu/TNSJf3sZzH3wYMOFy+1LV7D0Gyjm36I6vNvvt7u3xNXZ0pL8FwDetmFENpoAB233s2UTAHPO0gDhe/+XskhMNZiTGlgqjYkG2w3UM3Y/6Zc9TnmqGpObXuRovE0h+4mcn2W8qu30jzLPNuhSen0un2+tvzc/p5VjOM3LUTDJrlyxN++2iU62WVvQ0utLUgkHlJA7jcA/qr0F0q6gqKGnhlp2UwLJHOe4ElwLnG7iQ4HU520HABV0mDzyuje6c3YA1pDbEAaaEd+uq8/llumWQM6t+eXe03S6zYl0Zuj5eS4FyVodSshSykkFW22+x8/I1sTO9ab3muK5fjP3t50P7qsgbvvX9oW57NyttI6XL0hz79Lfm3T5+Xbvd/SlquPDK6rirZ6YGSLZ2TtOFtl20MhYZHPMctFPBh9ZTRyRR1B2X32vhBvdrmnMknMOI1431sV53foK9/8jTv+zr/APStjcOmn+a5PrngsCyYxcpLjWQQJTxTGXyssNSELcdWrbZKEpSSSfhV7lKun4+5zS0R68/4SEfs21jw4yacv5SlKVnlp0pSlCEpSlCEpSlCF//Z</v>
+      </c>
+      <c r="N3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Bill should be address to UMANG COMMUNICATIONS PRIVATE LIMITED 2.
+xerox copy of the following should be attached along with the bill.
+(a) Purchase order, (b)Necessary supporting document
+Terms of payment withing 45 days of the submission of the bill.
+In case of any variation or non conformity to your specification, the said bill shall not be eligible for any payment.
+Payment shall be process on the completion of job/delivery of materials to our satisfaction only . All dispute are subject
+to Guwahati Jurisdiction.</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>FIRM-a7ed8c9d-a4f2-47b5-b070-c7e82f1aaa49</v>
+      </c>
+      <c r="B4" t="str">
+        <v>JB Communications</v>
+      </c>
+      <c r="C4" t="str">
+        <v>18AAPFJ1273K1ZX</v>
+      </c>
+      <c r="E4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dr. B.K. Kakoti Road, Rehabari
+Near Gurunanak Temple
+Guwahati – 781007
+Assam, India</v>
+      </c>
+      <c r="F4" t="str">
+        <v>9864023965</v>
+      </c>
+      <c r="H4" t="str">
+        <v>system</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-04-20T09:51:02.533Z</v>
+      </c>
+      <c r="J4" t="str">
+        <v>system</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2026-04-21T06:43:29.695Z</v>
+      </c>
+      <c r="M4" t="str">
+        <v>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/4gHYSUNDX1BST0ZJTEUAAQEAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADb/2wBDAAMCAgICAgMCAgIDAwMDBAYEBAQEBAgGBgUGCQgKCgkICQkKDA8MCgsOCwkJDRENDg8QEBEQCgwSExIQEw8QEBD/2wBDAQMDAwQDBAgEBAgQCwkLEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBD/wAARCAD2AfIDASIAAhEBAxEB/8QAHQABAAIDAQEBAQAAAAAAAAAAAAgJBQYHBAIDAf/EAGMQAAEDAwIDAwQJDQoICgsAAAEAAgMEBQYHEQgSIRMxQQkiUWEUMkJSV3F2gbQVFhcYNzhidZGUldHTIzNVcoKTobKz0iQoNkdWY3R3GSdTZoWSlqKxtTQ1RGRlc4OjpMHD/8QAHAEBAAIDAQEBAAAAAAAAAAAAAAUGAwQHAgEI/8QAQBEAAQMCAwUFBAgFBAIDAAAAAQACAwQRBSExBhJBUXETYYGRoSKxwdEUFjIzUlPh8BUjNUJyNJKy8TZUYqKj/9oADAMBAAIRAxEAPwC1NERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERFr901CwGyVn1PvWcY/QVXNy9hVXOGKTf0crnA7rN0tVS11OyroqmKoglHMyWJ4exw9II6Fe3RvaAXCwK8h7XGwK/VEReF6RF46m8Wmil7CsulJBJtvySzta7b4iV+f1w2D+HLf+cs/WvQY46BfN4c1kEWP+uGwfw5b/AM5Z+tPrhsH8OW/85Z+tNx3JfN4c1kEWP+uGwfw5b/zln60+uGwfw5b/AM5Z+tNx3JN4c1kEWP8ArhsH8OW/85Z+tPrhsH8OW/8AOWfrTcdyTeHNZBFj/rhsH8OW/wDOWfrXsp6mnqoxNSzxzRnufG4OB+cL4WkahfQQdF+iIi+L6iIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIirt46+KjLZ80r9GsBvdRarRZwILvU0khjmraktBfFztO4jYCGlo25nc++4AViSpD1brJ7jqtmdfUu5pqnILjLIfS51TIT/4q57FUMVVVvllF9wZA8ydfBVzaWqkgp2xxm28c+gWpklxLnEknqSfFb/pLrrqZoreobrg+SVMFO2QPqLbLI59FVN36tkiJ5TuOnMNnDfoQtARdTmhjqGGOVoLTwKoscj4nB8ZsRyV3OkmpFp1d05seodljMVPeKbtHQudzGCZriyWInx5Xtc3fx238VFLj14pcjwm4xaN6cXeW218lM2pvdxpn8s8LJOsdPG4dY3Fuz3OGx5XMAI3K3vyc88s3DqI5HlzYL7Wxxg+5btG7b8rifnVf3Edcq+66+6h1dycXTtyW4U438I4p3Rxj5mMaPmXNcCwaB2NTRvF2RE2B65X52HqrpimIyjDY3tNnPtc+GfmueVFRUVc76mqnkmmlcXPkkcXOc495JPUlfCIunaKkIiIvqIiIiIiIiIsjZMjyHGattwxy/XG1VTCHNnoqp8EgPpDmEFY5F5c0OFnC4X0EtNwpR6Q+UE1iwOeGgzmRmaWYOAeKwiOujb+BOB5x8f3QOJ7twrD9JNYMF1rxSLLsFunsmnJEdTTyAMqKOXbcxys3PK719QR1BI6qk1dB0N1qyvQnO6TMsamdJDuIrjQOeWxV1Nv50b/AEHxa7Y8rtj16g1LG9lKaujMtI0MkHLIHuI0HXzVgwzHpqZ4ZUHeZ36j98ldOiwWDZpYNRMRtWbYxViotl4pm1MD/EA97HDwc1wLXDwLSPBZ1clex0bixwsRkVfmuDwHN0KIiLyvqIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiKjzU37pOWfjyv8ApD1eGqPNTfuk5Z+PK/6Q9dA2C+9n6N95VT2r+7i6n4LWkRF0tUtWh+Tj+94k+UFb/UhXF+OjhSy1uY3HWjT60VF2td1aKi80lKznmop2tDXTBg850bwA5xAJa7nJ2aRt2jycf3vEnygrf6kKkxeb3Z8ctdRe8gutJbbfSM7SoqquZsUUTfS57iAB8a4/UYpPhOOTTQC5LiCOYvp8l0KKiir8LjjlNsgb8lRIQQdiNiEVh2sHEVwGXe9zSX7TwZnXmT93uFpszI3SO8S6d74XSfHu4egrL6PWTgA1urPqRiGC26nvHKXi13Lt6epe0Dcln7qWSbDckMc4gDcgBXh20kkMHbz0kjRxyFh6g+YCrIwZskvZRTsJ6/8AfvVbSK4P7Tnhn+CS1fz0/wC0T7Tnhn+CS1fz0/7RaH17ofy3+nzW19Vqr8bfX5KnxFcH9pzwz/BJav56f9on2nPDP8Elq/np/wBon17ofy3+nzT6rVX42+vyVPiK4P7Tnhn+CS1fz0/7RPtOeGf4JLV/PT/tE+vdD+W/0+afVaq/G31+Sp8RWzZNwIcNORUjoKfCJ7LOWkNqrbcJ2PZv4hsjnxn52lQC4nuGe+8OmUU1K+vN1x67h77Xcez5HHlI54ZWjoJGhzeo6OBBG3VrZbC9pqHFZOxju1/AOGvSxIWhXYLVUDO0fYt5jh10XFkRFYVEKfHkzdU55osj0duNRzMp2/Vy2Bx6taXNjqGD1bmJwA8S8+KngqhOC7JZMX4lcLqA8iKvqZbZK0H24nhfG0H4nuYfmCt7XINsqRtNiRe0ZPAd46H3X8V0LZyoM1Huu/tNvDUe9ERFU1PIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIqPNTfuk5Z+PK/wCkPV4ao81N+6Tln48r/pD10DYL72fo33lVPav7uLqfgtaREXS1S1aH5OP73iT5QVv9SFRU47NcL9qJq5dMCp6+WPGsQqXUMNIxxDJqtg5ZppB7pwfzMbv3Nb02Lnbyr8nH97xJ8oK3+pCq9Nduut+oZP8ApVdvpcqoWC08cu0FVK8XLSbd1zqrViUz2YTAxpyda/gFo69dou9zsF0pL3Za+air6CZlRTVELy2SKRp3a5pHcQQvIivhAcLFVYEg3Cuq0H1JGrukWM6guaxtRdKMezGMGzW1UbjHMAPAdox+3qIW/KAvBlxVaN6S6N/WdqJltRQXGK61M8ULbfUThsDwwjZ0bHN6u5ztvuu7jj14XfhAqR/0LW/slxTEcCrIquRkELiwONrNJFr5cF0mjxSmfTsdLI0OsL3I1Ug0UfRx58Lnwhz/AKFrv2K+hx5cLfwjTD/oWv8A2K0v4NiP/rv/ANrvktn+I0f5rf8AcPmpAIuAfb48LXwkS/oWv/Yr5l48+FyNhezUSeQj3LbLXbn8sIH9KfwbEf8A13/7XfJP4jR/mt/3D5qQKh35TS9WKDSbHMfqjG67Vl+bVUjNxzthigkbK/07byxt+Nw9C+M98pdplaaeaDT3Erzf60DaOasDaOl39O+7pDt6ORu/pHeoI6s6uZvrTl02ZZ1chUVb2iKCGJpZBSwgkiKJm55WjcnvJJJJJJJVp2a2brWVjKupbuNbnnqT04d91B4zjNM6ndBCd4uy7gtMREXUFSFvegk0tPrnp5LCSHtyq1bbeO9XGCPnV1qp94O8NnzXiNwukjgc+G114vNQ4d0bKUdq1x9RkbG343BXBLl23cjTVxMGob7z+ivGyzCKd7joT8EREVFVoRERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERUeam/dJyz8eV/0h6vDVHmpv3Scs/Hlf9IeugbBfez9G+8qp7V/dxdT8FrSIi6WqWrQ/Jx/e8SfKCt/qQqvTXX7t2oXyqu30uVWF+Tj+94k+UFb/UhVemuv3btQvlVdvpcqpOA/1ut6/FWXFf6ZTdPgtHREV2VaRERERERERERERERERfcEE1TNHTU0L5ZZXBkcbGlznuJ2AAHUknwXwurcNestl0O1Ipcwv2FUWQUoAie6Rm9VRA981MSeUSAekdRuA5u5KwVMkkUTnxN3nAZC9r911khYx8ga926DqeSnjwO8NFboxitTmmZ0fY5bkkTWup3gc9voweZsJ9D3nZzx4crG97TvKFYLCM2xjUXF6DMcOu0VxtVyjEkE0Z+YtcO9r2ncFp6gggrOrhGI1c9bVPmqftk5jlbK3gup0cEVNA2OH7I9e/xRERaS2UREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREXEOKviToeHbDKero6OG4ZLenPhtNHKT2Y5AOeaXYg8jOZvQEFxcBuBuR29Va+UTySpvPERPZ5JSYbDaaOkiZ4NL2mdx+M9sOvqHoU/s1hseJ4g2KbNoBcRztw8yFE41WPoqQvj+0TYeP6Ll2X8TOvecV0lde9VchYJHb+x6GtfR07R4ARQlrenpIJ9JK9OC8Uuven1yhuFo1MvVZFE4F1FdKt9bTSN36tMcpOwPcS0td6CFylF2A4fSGPsuybu8rCy56KuoD9/fN+dyrneHrWu0696aUWc2+nbSVYe6judEHc3sarYAXNB8WkOa9p7+V4367rpagZ5Lm7VLmah2J73GnYbbVxt36Ne72Q15+MhrP8Aqqea4vjtEzDsQlp4/sg5dCAbeF7LpGF1LqykZM/U6+BsiIiiFIIiIiIqPNTfuk5Z+PK/6Q9XhqjjUaZlTqFk9REd2S3mte0+kGd5C6BsF97P0b7yqltX9iLqfgteREXS1TFaH5OP73iT5QVv9SFV5a5HfWvUA+nKbr9LlViXk6IHw8OjJHNIE18rXtJ8RtG3f8rT+RV162nfWfPj6cnuv0uRUnAc8brevxVlxX+m03T4LS0RFdlWluuIaK6s5/aTfsK09vd6t7ZnQGpo6V0kYkaAXN3HiA4flWaPDBxDD/M3lf6Ok/Up5eTg+96n+UVZ/ZwqU655iW2VTQ1clO2NpDSRx+at1Fs7DU07JnPILhfgqZDwx8Qo/wAzWWfoyT9S/h4ZeIQf5msu/Rcv6lc4i0fr5V/lN9fmtr6rQfmH0VMY4ZOIRwJGjWW9PTa5R/8ApY646Ca4WiIz3HSDM4Im98jrHU8g+NwZsrrUXobeVV84m+ZXw7KwcJD6Kh6toK621L6O40c9LUR+3injLHt+Np6hfgry8swXDM7oHWvM8VtV6pXNLezrqVk3Lv4tLhu0+sbEKB3FnwLW3CLDXanaNsqfqXQNM9zskj3SupoQN3TQvcS5zGjq5rtyBu4O2GwnsL2xpa+QQzt7Nx0zuL9creXioqu2dnpWGSJ28BrwPkoSoiK4quqSnBDxD1WkOokGH36ucMSymoZT1LXu8yjq3bNiqR70b8rH/gkE78gVqioXVyHCzqQ/VTQnFcnq6gzXCOk+p9wc47vNTTns3Pd63hrZP5a5rtxhjY3Mr4x9rJ3XgfK48ArnsxWl4dSvOmY6cQusIiLnytqIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiKqryhNCKTiUuc4iLfZtsoJydvb7Rdnv8A/b2+ZWqqu7ynmKy02b4bmrIHdlcLXNbHyAdOeCUyAH1kVB29PKfQrZsZKI8UDT/c0j4/BQO0kZfQkjgQfh8VChERdfXPVNjyX94jgzbOLAduettVLWN9O0MzmH+3CsQVNvC/q3HotrPY8xrpHttMjnW+6hvX/BJvNc7YdTyO5JNvHswFcZR1dLcKSGvoamKopqmNs0M0Tw5kjHDdrmuHQgggghck21pHw4h25HsvAz7xkR7vNX/ZqobJSdlxaT5HP5r9kRFT1YURERFgs6yikwnCr9mFc8MgsttqK95PiI43O29ZO2wHiSqNpZJJpHzSvL3vcXOcT1JPeVY/5RbW6lxvBYNHLLWsddslLKi5NYd3U9Ax3M0H0GSRoA/BY/fvCreXVdiKF1PRvqXi3aHLoOPmSqJtNVNmqGwt/sGfU/sIiL12i1V99u1FY7VTuqK241EdJTQt75JZHBrGj1lxAV1JAFyq2ASbBW08EVkksfDHhkU0RZLVxVVc7cbbiWqlew/9QsVZGvtuqrTrjn9DWxlkrMluT9j4tdUPc13xFrgR8auTw3G6XDsRsmJUW3sey26mt8Ww23bFG1gP/dUAvKIaBXi2Zedb8ctslRZ7vFFDeTCzf2JVMaGNleB3MewMHN3BzTud3jfmOy+KRnF5i827W5HW9wPK6uuOULxh8Ybn2dr9LWuoWIi2fTrTPNtVslp8UwWw1Fyrp3DnLGnsqdhOxklf3RsHi4/ENzsF0ySRkTS+Q2A1JVLYx0jg1ouSrHPJxRvZw8yOewgSZBWOaSO8ckI3Hzgj5lKVaJofpbQ6M6XWLTuinbUOtkBNVUBuwnqZHF8rx47F7jsD3NDR4Le1wfFallXXSzx/Zc4kdF1OghdT00cT9QBdERFHrbRERERflVUtNXUs1FWQMmp6iN0Usbxu17HDZzSPEEEhfqvPcbhRWm31N1uVSynpKOF9RPM87NjjY0uc4nwAAJX0XvlqvhtbNUc5vZIsazS/45ASY7VdKqiZud/Nilcwf1VhVl8wvv10Zbe8l5HM+q1xqa7ld3jtZXP2P/WWIX6Gi3uzbv62F1yJ9t47uiKxnyYmQPq9N8vxh8nMLbeoqxoPuRUQhv5N6c/0quZT+8lw0i16jP8ATUWsfkbU/rVd2vaHYRITwLf+QHxUxs84jEGAcb+4qdSIi40ujIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIuEcamlc+qmg14prXRmou9ge29UDGjd73RAiVg8STC6TYDvcGru6LYpKl9HOyoj1aQfJYaiFtTE6J+hFlQuikLxp6A1GjGqFRdrPQcmKZPLJW210bfMp5Sd5qY+95XHdo945u25a7aPS7zR1cddA2oiPsuF/wBOo0XLKmnfSyuhk1CKUHDDxu5JotSwYVmtHUZBiEZ2gbG8ezLcD4QlxAfH/q3Ebe5cO4xfRea2hp8RiMFS27fd3jkV9pqqWjk7WE2Kui064h9GdU6SGfD8/tM1RN09gVE7aesa70GCTZ/q3AIPgSujKhdZCDIsgpYzFS324QsI2LY6p7QR6NgVSZ9goy68ExA5EX9QR7lZYtqnhtpY7nuNvSx96u9yfN8NwqkNdl+V2iyU4G/aXCtjgB+LnI3PqCixrh5RHAcXoqqyaPxHJr05pYy4yxujt9O733nbPmI9AAaffHuVbcksk0jpZpHSPcd3OcdyT6yvlblDsRSU7g+peZLcLWHjqfVa9VtNUSt3YWhvfqfh7llcqyrIc3yGuyvK7tPcrtcpTNU1Ux3c93d3DoAAAA0AAAAAABYpEV0a1rGhrRYBVskuNzqilT5PfR2pzjVsah3Cj5rJhg7cPePNlr3tIhYPSWDmkO3cWs39sFHfT7Acm1OzC24PiFAau53SYRRt7mRt73SPPuWNaC5x8ACritD9IbFofpxbMAsT+3NMDNW1ZYGuq6p+xklI8N9gAOuzWtG523VU2txhtBSGmYf5kgt0bxPwH6KewDDzVVAmcPYZn1PAfE/qt9X51FPBVwSUtVDHNDMwxyRyNDmvaRsWkHoQR4L9FBfjw4rMkxa9v0W02u0ttqI4GSX25Uz+WdpkbzMpo3DqzzC17nN6+c0AjZ2/MsLw2bFakU8GupPADmrrXVkdBCZpdOXM8l1zPdJuBrGb06tzuz4DZri13O6lkuApSSeu/sZkjQR/I2WwYvr9wl4fbW2PENQMJstDEelPRFlPHv6dmtAJ9fUqoWWWSaR800jpJHuLnOcdy4nvJPiV8rox2OE0YZU1L3W78vAG6p42iMby6GFrff5iyuU+2m4dfhixj89CfbTcOvwxYx+ehU1osP1Do/zXenyWT601H4G+vzVyn203Dr8MWMfnoT7abh1+GLGPz0KmtE+odH+a70+SfWmo/A31+auU+2m4dfhixj89CfbTcOvwxYx+ehU1on1Do/zXenyT601H4G+vzVyh4p+HUAn7MWM9P/fAofcXnG/btQLJWaW6QyVH1Fq/3K63iRjonVke/WGFp2c2M+6c4AuHm7Bu5dCxFvYfsfQ0M4nJLyNL2tfnkFq1e0NTVRGIANB1tqiIitigUVmvk2cXNo0PuWRyxbS36+TPY7b20EMbI2/keJlWpabVcL7daOyWmmfU1twqI6WmhYN3SSvcGsaPWSQFdppXgdBphpzj2AW7lMVkoIqZ72jYSy7byyfG+QvcfW5UjbisEVGymGrzfwH62Vm2Ypy+pdMdGj1P6XW1IiLlavSIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIi03VvSnFNZsHrsEzCmL6SrAfDPHt2tJO3fkmjJ7nN3PqIJadwSFUdrfoTnOg2WSY3l1EX00rnOt1ziafY9dED7Zh8HDcczD1aT4ggm6NYDN8DxDUfHqjFc3sFJd7ZUjz4Khm/K7wexw85jxv0c0gjwKseAbRS4M/ccN6M6jl3jv7uKhsVwhmIt3gbPGh+B/eSo2RTh1g8mtfKOee7aK5HFcKU7vFou0giqGfgxzgcj/VzhmwHVxUU810U1b06lezNNO77a2M33nko3Opzt37TM3jd8ziuqUONUOIgGCQE8jkfIqjVWG1VGbSsNueo81pSIilFooiLa8I0p1J1Jqm0mC4ReL04nYyU1K4xM/jynZjB63OAXiSRkTd+QgDmcl6Yx0h3WC57lqi3DS/SXPtYsjZjGA2Ca4VJ2dPL7WCljJ/fJpD0Y3v7+p22AJ6KVejXk2sjuM8V21svkdpo2kO+pNrlbNUyeqSbrHGP4vOT6W96nTgOnWE6X49Di2B47S2i3RHm7OFpLpH+L5Hnd0jj75xJ6BU7F9saakBjo/wCY/n/aPHj4Zd6sOH7Oz1BD6n2W8uJ+Xj5LnnDZwx4hw9Y7y0ojuWT18YFzu72bOf3HsYgerIgfDvcQC7uAb2dEXL6mqlrJTNO67jqVeIII6eMRRCwCKl/iSnuVRxAaiSXYu7cZJcGN5v8AkmzubF83Zhm3q2V0CgVx0cJeV3zJ6nWfTKzTXVtdE03u20rOaoZKxoaKiNg6yBzQ0Oa0cwI5tiHEttGxtdBR1rmzG2+LAnnfTx96hNo6WSopg6MX3Tcju/RQMRfc8E9LNJTVML4ZonFj45GlrmuHeCD1BXwutrn6IiL6iIiIiIiIiIiIiIs9ieA5vnlaLfheJXe+VG4BZQUck3J63FoIaPWdgpk8P3k6rrNW02T68TR01JEWyx4/STh8sx79qiVvmtb6Wxkk7+2btsYzEMXo8MYXVDwDy4noP2Fu0mH1Fa7diblz4ea8nk9OHSrul7ZrvltAWW2388WPxSt/9IqerX1Ox9wwczWnxeSRtydbDF56CgobVQ09stlHDSUlJG2GCCCMMjijaNmta0dAAAAAF6FxvF8UkxeqNRJkNAOQ5fPvXRcPoWYfAIWeJ5lERFFreREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREWuXjTbTrIXukv8AgOOXJ7/bOrLVBMXfGXtO6wQ4etBQS4aK4L169cepD/8AzXQEWdtVOwWa8jxKxOgicbuaPJalZ9ItJ8em9kWDTDE7ZLvv2lHZaaF2/wAbGArbGta1oa1oAA2AA6AL+osb5Hym7yT1XtrGsFmiyIiLwvSIiIiIiIi17IdPNP8ALn9rlmDY/en++uNsgqT+WRpWLt2iejdo7T6l6T4dSdtsZOxsdMzm23232Z4bn8q3VFmbUTNbuteQOVysZhjJ3i0X6LV/sWaY/Bzi/wCiKf8AuJ9izTH4OcX/AERT/wBxbQifSJvxnzKdlH+EeS1f7FmmPwc4v+iKf+4n2LNMfg5xf9EU/wDcW0In0ib8Z8ynZR/hHktX+xZpj8HOL/oin/uJ9izTH4OcX/RFP/cW0In0ib8Z8ynZR/hHktX+xZpj8HOL/oin/uL+waXaZ0z+1ptO8YifvvzMtFO07/GGLZ0T6RL+I+ZTso/wjyX5wQQUsTYKaGOKJg2axjQ1rR6AB3L9ERYVkRERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERRu4neM/FdCZZMSx2jiyDMSwOdSl5FNQBw3a6oc3qXEEERt2JHUloIJ6bxA6pR6NaRZFn7RG+soqbsqCN43a+rlIZCCPFoc4OI961ypsqqq+5hkMtXVSVN0vN5rC97iC+apqZX+rqXOc78pVx2VwCPEy6pqvu2m1uZ1z7gq7juLPogIYPtu48h8yupZlxf8RebVb6ms1Qu1rjc7dlPZpfYEcY96DDyvI9bnOPrWs/Z/14+GzPf+0lZ+0U2dFPJy4PQWGlu+tNRWXa81MYkltdJVGClpNxv2ZfHs+R48XBwbvuADsHHqX2hvC38HM36ar/2ysMm0mBUjjDHFcDi1rbepCiGYNilQO0fJYnm439AVDfhM4ktaY9cMZxu9ZxkOT2rIK1luq6O510tZytfuBKwyFxYWHZ5Ldt2tIKtIXMtNuGrRDSO6G+YFgVJQXItLBWSzzVUzGkbEMfM95ZuOh5dtwto1G1ExXSrDrhnOZ1xpbXbmNMjmM55Huc4NZGxo9s5ziAB69yQASKZjldT4vVtdQxFuQFrC5N+Qv0Vjwymmw+ncKp9+OuQHUrk3EpxfYTw/sFjgphkGWTxh7LXDMGNpmkbtkqH7HkB7w0AucPQDzKCuY8dfEjltQ59PmcVgpi4ubTWijjia30DtHh0h+d67DppbeDXih1PudDXWHNbblF7nqLhGbldd2Vrur3tY5jnbODdzyHoGt6E7bLuH/B58Nv8ABF9/Sz/1Kw0r8GwECKthcZbXJc0HyF7WUTO3EcVJkppAGcLEjzyvdQjxfjd4lcXq2TjUOS7QtcHPprpSxVEcnqLuUSAfxXtU2uGrjcxDWyrgw/KaKLG8ulG0MHac1JXkeEL3dWv/ANW7r6HO67aHqn5NXCq20VFdpJkdytt2ijLoaK5ytnpZ3D3POGh8ZPvjzDu6DvVf1xt9/wANyGe23CCqtV5s1WY5WEmOamqI3ekdQ5rh0I9G4UsKPBdp4XfRQGPHIbpHK40I/dwtA1OJYJIO3Jc08zcHoeBVxHEpqjc9G9F8i1AslLDUXKhZDDSNmG8bZZpmRNe4eIbz823jtt4qv/Szj11rxfOYLrn+SS5Lj9VMBcaGWnhY5kZPV8BY1vI9o6hvtT3EdxHadS9ZZdb/ACfdzym5yRuvVHV0Nsu/INgaqKsg8/bw52OjfsOgLyB3KvxYdmcDp3Uk0NZGC8PLSSM8gNDw1uCFkxrE5RURyU7yG7oI8SdQr2bBfrRlFkocjsFfFW225U7KqlqIju2WJ43a4fMe7vC9xIA3J2AVdvk/OJT62rtHobmdw5bVdZi6wTyu6U1W47up9z3MkPVvok3HXn6dc4+OI77HWJfYoxKv5MkyWnPs2WJ3nUNA7cO6+D5erR4hoeehLSqjUbOVMWJjD2Z3zB4bvPw49/grBDjEL6L6W7hqO/l48O5cX4n+OrOrjnNVi+iuTfUjHrPKYHXGmjY+W4zNOznh7gdogRs0N9sAXEkEAbthfGpqTPwp5Tnd2io63LrBc6ez01e6na2OUVABbNJG3ZpewCToAGkhm49tvABd4w77zfUP5W2j+o9dAq8Bw+CmiiEYNnsF7Zm7gDc8b8eCqVPitXLNJIXnNrsuAyNrDuW16M8eur2LZzT1Wp2SzZJjVdMGXGCWmibJTsces0Bja3Yt7+T2pG42BIcLO7XdLde7bSXm0VsVXQ10LKimqIXczJYntDmvaR3ggghUQqdHk+OJT2FUR6C5pcP8HqHOkxuold0jkO7n0hJ8HHdzPwuZvumhRO1ezsbofplGwAt+0ALXHOw4j3dFv4DjDxJ9HqHXDtCeB5ePvU/pJI4Y3SyvaxjAXOc47BoHeSfAKtTiN479RL7nVVaNG8mdZMZtUxhgq6aJjpbi9p2MznPadoyQeVo23b1duTs3sXlA+I760MfOimIV/Ler5BzXqaJ3nUlC7uh3Hc+Ud48I9+nngquJYdkdn43x/TqtgN/sgi4tzt38PPiFk2gxZzX/AEWnda2pHu+asAt3GnqPLwiXLUOqFIcypL+zGYbgKZnZuc+ETCpMW3JzhnONtuXmDTttu1afwe8WWsuS622jBc7yubILTkXbwubVRR89PK2F8jJI3NaCBuzlLd+XZxO24C5Lb/vIrt/vLpv/AC1y8fBj985gn+2T/RZlKPwihZRVhETbgvtlpZtxblY8lpNr6l1TTgvP9t89bnO/NW/KI/HxxD6gaPUeNYvp1chaqu+tqairr2xMfKyKMsa2OPnBDeYvcS7bccrdiNypcKvXyof+VeBfi+t/tI1Rdl6eKpxSOOZoc3PI6ZAq0Y5K+Ghe+M2OWY6hZThb4xdTbph+orc/qmZHUYjjk+QW6omjbHK4xkNMMrmAczS57DzbcwHN1PQDi2O8efEPas1iyi8ZVHd6B0wNTZpaWKOlkh36xs5W80ZA7ngk7gc3N1BxnDL/AJLa1/7u67+2hXCV0enwagdVVAMLbHdGgyu0acvBU2bEatsEJEh48e/jz8VeHpxqFjWqeF2zOsSrBUW66QiRoO3PE8dHxPA7ntcC0j0jpuNitW4k9Urlo1oxkOoFlpIai40LIYaNkwJjEs0zImvcARuG8/Nt47beKrz4MOJeXQ/NPrcyasd9ZmQzNZW8xJFBUHZrapo8B3Nft3t2PUsAM0ePSaKfhbyOeCRkkcs9tcx7CC1zTVxEEEd4IVCqcB/h2MRU0gvE9wt3i4uD3jQ+fFWuHFfpmHyTMNntab9xtqow8M/GdrVd9bLFjmf5S6+2fJ69lump5aWGPsJZTyxSRGNreXZ5buO4tJ6b7EYvXzjW11Zq7f7Xh2Vux+0Y7dqigpKSmponCQQSGMyTF7XF5cW7lp80b7AeJ4tw5fd+05+VFs+ksWM1n+7DnXyluf0qRX4YPQfxInsW/YGVhbUi9tL2yuqocQqvoYHaH7WtzfQcdVbxoJqNU6taP4vqFXU8cFXdqMuqmRjZgnje6KQtHXZpfG4gb9AQo/8AEvx7WjTW5VeC6U0dJfMgpHOhrbhOS6iopB0LGhpBmkae/qGtI2Jcd2jTqbWeu0b8ntiE1gqzT3/IjW2q3yt9tAHVlS6aYegtYCAfBz2HwUIMOxHIc/yq24di9C+tu13qG09NED3uPUucfBoALnOPQAEnuVbwjZumlqJ6qqH8pj3Bo4WaTme4fO6mcQxmaOGKCA+25rSTxzGg7yt8yXiq4icqrHVtw1fySmc47hltrHUEbfUGU/IFh/s/68fDZnv/AGkrP2inxpr5ObRvH7ND9kaWvyq7yRg1BbVyUtLG/wARE2IteQO7dzjvtvs3uW5/aG8Lfwczfpqv/bLddtRgUB7OOEkDkxtvC5B9FrNwPFJRvvksTzcb+gKjnwD8QOrGR6sS6eZflN5ya1XK3z1Ifcql9VLRyxAOEgleS4MI3YW77bub3eNhi0PTLQzSfRxlQNOMLo7RLVtDJ6gPknnkaDvymWVzn8u/Xl3238FviouOV1NiFWZ6Vm42wyyFzzsMlaMMpZqSnEU7t4/vLNYzJ8jtOIY5c8qvtSILdaKSWtqpD7mONpc7b0nYdB4lVXX3jo4grjn8mZ2vLX26hZU89NZGxsdRMgB6RPaRvJu3o55PNuSQW9NpM+Ui1f8Arewe2aRWmq5a7JnituIaerKGJ3mNPo7SUDb1QuHiq4lddkMEhfSuqqpgdv5C4vkOvM+gVb2hxORs4ggcRu62PH9FdzpJqPatWtOLDqFaA1kN4pGyyQh3N2E4JbLET48kjXN38dt/FQb4vOL7WrGNYb1p3g18djVrsD4oN4aaN09U90TJDI98jXENPP5obsOXYnclZDyausHsO63nRW71W0VwDrvZw93dMxoFREP4zA14A6Ds5D4qUOsfCho5rjd4sizG0VkF3jjbC6ut1T2Es0bfatkBDmu28CW822w32ACg2RUez2MPjro96O3s5XyOYNjrbMdVJukqMXw9r6V+6/jnbTUXHmq3ftxOJj4W7t/NQfs1/ftxuJgf527r/Mwfs1JjXbhP4UtAsFfm2TOzSr7SoZR0VFT3OESVNQ4OcGgmLZoDWucXHuA7idgeY8NGmfC5xBZNWYZW43mGN3iKnfV0kf1wRVUVVE0gPAd7GYWvaHA7bHcAnfpsrdFXYTNTOrGUt426ncb/ANnvsq++mr45hTun9s6DectAtXGtxMWu4QV51OqqwQvDnU9VSU74pR4tcOQHY93Qg+gg9VIviu4xNRbHjOn9PpxP9bsuYY3T5HW1QibJPG2bo2CMvBDQC15LgNz5uxHXfqVm8nfw6Wq5Q3CopMhubIXc3sWsuQ7F/qd2bGOI9XN8ajd5SykpaDVjE6ChpoqempsVhihhiYGsjY2pnDWtA6AAAAAKNpqnB8YxKGOmhHshxN2gA5ZZDXnnotyaHEcOo5HzSHOwGZJ1zz4LvvAVxCZvrJYsjxzUK4fVO5Y6+mlgr3RtZJNBNzjkfygAlpj9ttuQ/rvtuuu698ROBcPuOsuuUTuq7lWAi3WimePZFW4d56+0jHi89B3Dc7AxC8mld7bj8+p9+vNZHSW+3Wuiq6qokOzYoYzUOe8+oNBPzL971qPwa8Smt+2ZWfNqetvMsNtorpPW9lRktAjiaIw4uhY49R025nku5dyRF12DwuxmYmJ3YssSGDm0G3C18zlnyW9S4jI3Do/bHaOuAXHvIvx9VzXUDygev+X1U7cdulFidve49nT26mZJKGeAdNKHOLvW0M+ILUrNxl8S9kqhVU+qtxqevnR1kMFSxw9G0jDt82xU6P8Ag8+G3+CL7+ln/qWuZr5NnR272x7cKvt9sFxa13ZPmmbV07nbdOdjgHbb+9ePHvUnBjmzbQIhDZvewHz1J9VpS4XjJJkMlz3OI+QWM4evKF2bM7jTYjrJQUdguVS5sVNd6YltDK89A2VriTCSdvO3LOvXkAUs80yNuIYbfcudT+yG2W2VVyMQdt2ghidJy7+G/Lt86pa1N01yrSTNLhgmY0QguNvePOYSYp4z1ZLG4gczHDqD394IBBAm/wANOt9dqRwnakYJkdaai8YbjFwhhled3zUD6OUQkk95YWOYT70R79TudTHtnKaNrK6h+7JFwNLEixHd88lsYVjEzy6lqftgGx43HAqPtHx5cRsGZtyupyyCopO25n2U0cTaJ0W/70AG84G3QP5uf0uPjZhpHqnjOsuB23PcVn3pq1nLNA5wMlJUN27SGTbuc0/lBDh0IKpJXeeEXiPrNA88EV3nllxC+vZDd4Bu7sD3MqmN98zfzgPbM3GxIbtM7Q7Mw1VNv0TA2RmgAtvDl15eXFRuEY1JBNu1LiWu552PPpzVmeu2otVpNpHk+oVBRR1dXZ6Pnpopd+R0z3tjYXbEEtDngkAgkA9QoBaG8bmuVTrJYaXN8r+rNkv9zgt9ZRPpIY2QtmkEbXxcjWlhYXA7b7OAIO56qYvGNXUdy4VMzuNvqoqmlqqGjmgmieHMljdVQFrmuHQgggghVbaS/dVwz5Q276TGojZbDaWqw2d88YLrkXIzFmg5cszwUhjtZPBWxNieQLA5aHM+asS4v+Ml+iNWzT/T+mpK3LJoWz1U9S3nht0bx5gLARzyuHnAE7AcpIPMAoWVPGfxN1U76h+q9ewvJPLFSUzGj1Boj2AWP4so7rFxH6gNvPP7IN4kczn7+wLWmH5uyMe3q2Wf0Cs3CNkdtZaNbb5lliv753gVsMrBbnxkjkG7Y3vY70lw5fHmHcJvD8LoMNw5kzoe0JAJIaHHMXyHIdyjKuuq62sdG2TcAJAz3Rll59VjPtx+Jn4W7p/MU/7NfUPGZxNwysmbqzcXFjg4B9NTOadvSDHsR6ipk2TyfnDBktthvOO5LkN0oKgc0VVR3qnmikHqe2Ig/lWSg8nFw8xTMlknyuZrXAmN9zYGvHoPLEDt8RBWi7H9nm3Bg/8AzatoYTi5zEv/ANyuq8NOql01n0ZsGf3yhipbjWNmgq2wgiJ8sMroy9gPcHcm+3gSR4LqCxmM41YsOsFBi+M2yG32q2QNp6WmiB5Y2DuHXqT4kkkkkkkkrJrm9U+OSd74W7rSSQOQvkFcoGvZE1shu4AXPMoiIsCyoiIiKJflLZ6yLQe0R05cIpsopWT7dxaKapIB9XMGn4wFDLg2pbVWcTWBxXgR9g2ullZz7bduynlfD3+Patj29eyso4ptLKnWHRHIcRtkRkurI23C2sG276mE87Yxv03eA5n8tVBWS8XrDsjob9appaG7WWsjqoHluz4Z4nhzdwfEOb1B+IrqGyhbWYPLRsNne0P9wyP75KkY8DT4jHUOF25HyOY/fNXrIo76DcamlWrFip4cnv1uxTJ4mNbV0NwqGwQyv26vp5XkNc0nfZpPOOoIIAcel5Rr1ovhttkuuQ6n43TwRgnljuEc0r9vBkUZc959TWkrns2GVlPMYHxne5WJ8ufgrbHW08sfateLdffyW+qJPlLqurg0LstPASIanJ6dkxHiBTVLgD84B+ZRX4qeLjItcch+pWKVlws+G28uZTUrZjG+ud4zzhp2O/uWHcNG/iSt/wBF8N1H114N8/xuvqLhc22W5w1+Lioc6V7p4I+eeniLupBYeVrQdg+Q+tWyh2fkwcwYlVvAs5t28rm2vMakcOagarFmYiJaOnaTkbHnbPTv0XJeCiClqeKDBY6yQMjFRVyAk7ee2jncwfO4NHzq3lUW4pk96wfKLXltgqDTXOzVcdZTPI6NkjcCA4eIO2xHiCQrXtFuMPR7Vqw0ktZlFtxvICwNq7Tc6psDmy7ed2L3kNlYepBaebbvAPRbW2+HVE0zKuNpc0NsbZ2zJue439Fg2ZrIY43U7zZ17i/HID4Luiqt8oVbLVbuJCumtrY2y19qoqqsDNv3/lczc7eJYyM/Pv4qemqvFVoppRZai4XLNLbdrg1hNParXVR1NTO/bzWkMJEbT75+w+M9DU/qnqLe9WdQL1qFkIYytvNR2piYd2QxtaGRxNPiGMa1oPedtz1WHYnDqllS6re0tZukZ5XJI07slk2lrIXQiBpBde/TVdW0yrKt/B7rPb3ud7FhuuPTRDwEj6gh/wDRGz+hcbwbFKvO8zseFUFTFT1N9uEFuhllBLGSSvDGl23Xbdw3UtTpZXac+TtyC6XmnfBcstuVBd3xSN2dHTmqgZA0/Gxvaf8A1VHLh0+77pz8qbZ9JYrdRVTXx1c8PB7rdWsaPeFX6mAtfTxScWj1cT7itNvdlvmHZDWWG9Uk9uu1oqnU9RE48skM0btj1HoI6EeohfeUZTkeb3+ryfK7tUXS7V7w+oqp3cz5CGho/IAAAOgAAU+/KB8NUuS0H2b8Itjpbpb4mxX+mgZu6opmjZlSAOpdGNmu/A2PQMO/KeA7hnqM+yqHVvM7W8YzYZhJbY52bNuNa0+aQD7aOIjcnuLw1vXZ4GKDaGklw7+JPsC0WI4734R1y8MzovcuEVDKz6E3Qm4PC3M9FG7UTTnIdMLxR4/lMPse5VNtprjLTEEOpxO3nbG/f3Yby8w8CSPDddNw77zjUP5W2j+zes95Qof4ydy/FdB/ZrAYef8AE61DH/O2z/2ciy/SH1dBTzv1c6MnxcF47FtPVyxN0AePQrlenuFXHUbM7Vg9nmiirrzN7GpnS9GdqWktDj4AkAb+G+/VY2rpb3il+lo6qOqtl3tFWY3tJMc1NURP2PUdWua5vzELpHCiN+I3T/8AHUX/AIFSl8oNw1TVwdrvg9sdJNGxseSU0Ee5cxo2ZWAD3oAbJ6g13cHFe6rF2UmJMopsmvbkf/lci3j7+q8wYe6oo3VMerTn0sPcoL5BkGQ5tkVZkWQ3Coul4u1QZqieTzpJpXH0D5gGgbAbAAAALJ6kaeX7S3KX4bk7Gx3SnpKSpqYR3wOnp2Tdk78JokDXeG4O3pUp+APhnqMnv8OtebWtzbLaJOaxwzx7Ctqwf38A98cR7j3F+2x8whcy48/vo8t/+VbvoMC+QYrHLiZw6C26xpJtzu0ADoDn5cEkoHx0QrJdXOAHSxN/H96rx2/7yO7f7y6b/wAtcvJwY/fOYJ/tk/0WZbfgGJ1uVcCeoE9vp3Ty2HMKe7uY0bu7NlPCyR3xNZK5x9TSuL6OZ+7SzVHGdQPY7p47LcI554mbc0kB82Vrd+nMY3PA38SF5a01NPWQR5uu8eJaLe9eiexmp5X6WafJxV26r18qH/lXgX4vrf7SNTHx3iG0Oymyx361aq4wKZ0Qle2pucNPLCNt/wB0jkc18ZHocAq7+O3W/FtYtTbfS4TWsr7NjVE6kbXMGzKmoe/mldGT7ZgAY0HuJDiNwQTQ9kqKoZirXvYQGg3uCLZEK1Y/UwuoS1rgS61rHvutf4Zf8lta/wDd3W/20K4jQUwrK6mpHOLRPKyMkd45iBv/AEqSXC/iNU/Q7XnPJYntposXdaIHkebI94dLKAfS0Mi3/jhRzsf/AK7t/wDtUX9cLo1LIHVNTu8C3/iFTp2EQQ34g/8AIradZNJcm0Uz+44Fk8W8tK7tKWpa0iOspnE9nMz1OAO48HBzT1BXTaPiTqL/AMK2QaD5jUyS1tvfQyY/VO3cZKZlVGX0zj6YwCWE+4Bb05Wgz14sOHS36/4A+CgjhhyuzNfUWaqdsOd23nU7z7yTYDf3Lg13cCDUhc7bcLNcaq0XWjmpK2imfT1FPMwtfFKwlrmOB6gggghReD19PtHTMMw/mRkE9RoR3H5hb2IUsuDzOEZ9h4I8DwPeFvnDj937Tr5UW36QxYvWbrrBnXyluf0qRZThw+7/AKdfKe2/SGLFayfdfzn5SXP6VIpgf1E/4D/kVHn/AEg/yPuC6drXNVjhi4f6bdwpTT5E/bwMns5o/KAf6Stt8m3S2uo4gKyavEZqKbHKuWh5ttxMZoGuLfX2bpPmJW45DpNX6jeT1wbILJSvqLnhzq65CJg3dJSOq6htQAPUA2T4oz4lRP0r1JyDSLPrRqDjLmGttUxf2Um/ZzxOaWyRP29y5jnD0jfcdQFEQt/iWG1NJCbPDpG+Jc4jzupCQ/Q6yGokHs7rD4BoB8rK7xFxrSXi00V1YscFfTZfbrHcy0eybTdquOnqIX+IaXkCVvoczfoRuGnoMvn3EvodpxaZbpf9RrNM9jC6Ojt9Uyrqpj4NbFGSep6cztmjxIXKXYdVsl7AxO3uVir2KyndH2oeN3nddOX5VdVTUNLNW1k7IaenjdLLK92zWMaN3OJ8AACVT3xAcSuc66ZlPep7hW2uyQO5LZaYalwjp4wejnAEB0p73O29AHQBdxyPXnNcc4FLHj+TXarqMgzioq7bQT1MjnVDrNG/aWRzndSDv2IJ72PG3crHLsdUwshLnjee4At5XBJz42AN/iodm0UMjpA1ps0Eg8+HhcnJRz4gtVanWbVvIM7e9/sOqqDBbY39Oyo4/NhG3gS0cxHvnOXZce4XaCo4N7rqfdfY9NlVdUC+Wls8gY99upw5romgncmRrpZdh7blhXDNFdM6/V/VDH9PqDna26VbRVSsHWClZ580no3EbXEb952His5xNw5TQa15PY8ngqKZlorH0NppX8wip7ZGeWkZCD0EfYhhG3fuSepK6BNH7cWH0sm5uAOPE7rTYC2WROp7u9VKN/syVc7d7euPE5k+HDqtLwLM7xp3mdlziwyclfZKyOsiBOwfynzmO/Bc3dp9TirsMKy2z57iVozOwTdrb71RxVsBPeGvaDyu9DgdwR4EEKjFWFeTX1hFyx+76L3eq3qLQ510tAc7qaaRwE8Y/iyOD/X2rvQoTbXDfpFKKxg9qPX/ABPyPvKk9mq3sZzTuOTtOo+Y+CyvlOnf8VOKN9OQ7/8A40qjNwDb/bP4z1/9muP0SVSY8p0f+K3Eh/8AHz9GkUaOAUf4z2Nf7Lcfokqw4R/4xL/jJ8VkxD+ts6s+CthVbHlN/uyYyP8AmzH9KqFZOq1/Kbfdlxr5MR/SqhVrY3+qt6O9ymto/wDQHqPeufaAVdXRaB6/zURIkdZbTC7b/k31b2P/AO45y4/p9BS1We41TV0gjpprvRxzPJ25WGZgcd/DpupRcAeGU2ouNayYLVSiJl9sVLQiUjfsnv8AZAa/b8F2zvmUT7/YrziV/rsdvlHLRXO1VL6aphf0dFKx2xH5R0Pzro1JKySsq6cGzrtPgWNHpZU6djmU0E1srEeIcT8VeuiitwzcbmAZ7i1BjuqGS0WP5bQxMp5prhKIaa48oAEzZXbMa93TmY4jzieXcd3Zsz4g9FsBtMl4yPUmwsjYwvZBT1sdRUTeqOKMl7vmGw8SAuQVOFVlLOad8Z3r5WBN+nNdChr6eeLtmvFuunVQ/wDKi2u1RXzT68xMjFyqqW4007htzOgifA6Lfx2DpZdvjPrXGeEGsq4avVijhc7sKjTC+umb4btbHyu+Ykj+UVrHExrzXcQWpMuWuo30Nqo4RQ2mjeQXxU7XF3M/bpzuc4uO3duG7kNBPeOEDS2utnD7rFq7c6d8TLvi1ztNrLm7dpDHTSOnkHpaZAxoPpjeul9k7C8BZBU/ayFu8uvbwHuVL3xXYq6WD7OZ8A21/H4qF633WrR3JdE80lxS/sMsE0Tau3VoZsyspX+1ePQR1a5vg4EdRsToSt/4gtALPxA6TU9hkENNfrdTNqbJXPH7zPyDeNxHXs5Ng1w8PNdsS0LfxjGRhFRAJPu37wPd9mx8L59y1cOw44hDLufbbYjv1uFALDOJOpPDTmmgOYVMkzZKWGTHKl27izlqonyUrj73YOewnu2c3fq0DlOkn3VsL+UNu+kxrBX+w3jFr3XY5kFvloblbZ301VTSjZ0UjTs4H5/EdD3hZ3SP7q+F/KG3fSY1vilhp4ZXw6Pu48rkWuOtrrVM8k0kbZP7bDwv8FZFxacHVHr1JFmWI3CltOYUsIp3uqQRTXCFu/K2UtBLXt32a8A9PNI25S2vLUzQHV7SGV4zzB7hQ0rXcra+Nono39em00e7AT70kO9SuWu+R49j7Y33++262tmJEZrKpkIeR37c5G6xM2ommdRC+nqM6xiWKRpY9j7nTua5p7wQXbELmWD7TV+HRiEs7SMaa3HcD8wVdcRwSlrHmTe3Hn95j/pUyYJqbqBplcvqtgOX3OyVBIL/AGLMRHLt3CSM7skHqcCFMnQ7ykFwmuVHjuuFnpPY0zmxG/W9hjMRPTnng6gt9Lo+XYdzCup6pcMvB/qV21bS3/HcVukm7vZdku1NAwu/DgLjERv37Na4++Va2Z2OgxnLrzjtqvtNeqO2V09JBcab96q42PLWys6kbOA3GxI69CR1Vxhdhm1THCSIh4GpFiOjhr0Pkq7IK3AnAskBaeRuD1H76q8unqIKuniq6WeOaCZjZI5I3BzXtI3DgR0II6gr9FwjggyO65Lw0YlUXd7ny0Lai3RSH3UEE744h/JYGs/kru65VWU5pKh9OTfdJHkbK908wqIWyj+4A+aIiLWWZERERFDbit4FW6jXSs1I0idTUeQVbjNcbTK4RQV8h75Y390crvdA+a49SWncumSi3sPxGowuYT0zrH0I5ELVq6OGuj7KYXHqOio7zLTbP9PK19Bm+HXeyTNdy/4ZSPjY/wBbHkcrx62khYa12a73upbRWW1VlfUOIDYqWB0ryT6GtBKvcc1r2lrmgg9CCOhXzFDDA0thiZGCd9mtAG/zK6N2+eGWdAN7/LLysfeq27ZRu9lLl0/X4KsDQ3gD1Q1Cq6a76jU82HY9zB0jKlu1xqGeLY4SP3Pfu5pNiO8NcrJ8Mw3HNPsXt2G4lbY6C02uEQ00DNzsN9yST1c4klxcepJJPes2iq2LY5V4w4dubNGjRoPmf2FO4fhcGHNPZC5OpOqg1xYcCNfkl3r9TNFaeF1ZWvdU3KwFwj7WUnd8tM4+aC47kxkgb7lp6hqgfkOMZHiNzks2U2G4WivhOz6atpnwyN/kuAPzq9VeW4Wu2XaD2LdbdTVsO+/Z1ELZG7+nZwIUzhe2VTQxiGob2jRob2Pnnf396ja7ZyGqeZInbhOuVx8LKi202a73+vitVitVZca2c8sVNSQOmlefQ1jQSfmCmlwwcAt9rrpRZ1rnbxQW2meJ6bHpCDPVOB3aanboyP8A1ftndzuUdDP622az2aN0NntVHQxvO7mU0DYgT6w0BexZMS21qauMxUzOzB1N7nwyFvevNHs1DA8Pmdv24WsPjdcQ4zsRvOX8NuWWfHKF9VVwR01YyniYS58cFRHJIGgd5DGuIA79tlW/wpYvfMo4hMGgstBNUG3XmluVU5jCWw08EjZJHvPc0bN2BPeS0d5CuPXlpLZbbfJNLQW+mpn1DueZ0MTWGR3pcQOp6nqVHYVtE7DKGWjDN7evY30uLaWz07lt12DtrallQXW3bXFtbG/gvUvljGRMEcbGsa0bBrRsAF9Iq0ppVg+Ubxi9WzXePJKqglbbbzaab2JU8p7N74gWSM5u7mbsCR37OafFfnp/pNm9z4Hs8vtJZal8dXfqO50sIid2lRSUo5ZpmDxYO0cd/RE/0Kzqut1vulOaS50NPVwEhxjnibIwkdx2cCF+zGMiY2ONjWMYA1rWjYADuACtzNrJI6KGlbGLxlud9Q03AtbK/VV92AsfUyTl+TgcraEqobgyxe95LxG4fJaKCWeK1VhuFbK1pLIII2OJc89zQTs0b97nAeKt6IBBBG4K81FbLbbe1+p1vpqXtn9pJ2ETWc7vS7YdT6yvUo3HsZONVDZtzdAFrXvxv3LdwrDhhsRj3t4k35L5YxkbQxjQ1rRsABsAFVf5QfGL1Z+Iy6X6uoJY6C/UdHPQ1BaezlEdPHC8B3dzNdGdx3gFp8QrUl5q+2266winudvpqyIODxHPE2RocO47OBG68YHi5waq+kbu8CCCL21se/kvWJ4eMRg7HetY35/vVRV8ndg1xt2gd2mye1ctDlF2nnp4KiPpUUhgjiLi097HFrwPSBv3FRu4neCXNdMb3XZRptZau+4bPIZY46Vrp6q3A98cjBu5zAd9pBv025tj1NoYaGgNaAABsAPBf1bdPtNU01fJWxgWec28O7xHP0WvLgsE1Kymec2jI8f+u5UMyRyQyOiljcx7CWua4bFpHeCPBdV0X4ZdV9brrTQ49j1TRWZ72+yL3WQujpIY9+rmuO3au27mM3PUb7DqLfqzGMauNX7PuGPWypqQQe2mpI3ydO7ziN1kgABsBsApyo28kfHuwQ7ruZN7eFgouHZVjX3lkuOQFviVxO86DW/CeFvI9GdOqaSpmfYa2OJ0gHbV1Y+Nzi523unu2A8AOUdwVVunuGZNluoVnxCxWaqqLrPcIoTTiJ3NERIOcvG27Gt6lxPRoB37ld+vPDbrfT1U1bT0NPFUVG3bTMia18m3dzOA3PzqHwnaeXDGSte3fc83uTx78s/RSNfgkda6Mtduhota3D4L0KEXHzwuyZDTS64af2t0lzpWAZBRU8e7qmFo2FU1o6l7AAH+lgDunKd5uoofDMRmwqpbUQ6jUcxxB/fepGto466EwyefI81TjwoYxe8o4hcGhslvlqTbrxTXOqcxpLYaaCRskkjz3NGw2BPe4tHeQsfxFYff8R11zOy3i3zRT1N8q6umBYf3eCeZ0kT2e+DmuHd47jvCuMtOM43YZqmoseP223S1juepfSUkcLpnel5aAXH1leqe3W+pqYaypoaeWopiTDK+Jrnx79/K4jdvzK1nbYisNQIfZ3d21873ve9vSygRs0Po/YmTO9727rWtdcq4TcUvWH8OmF43k9uko6+KimlnpZmFr4xNUSyta9p6h3JI3dp6g7gqL3Ex5Py6/VOszfQimiqKape6epxwvbG+Bx6k0rnbNLO/9zJBb3N3BDRP5FXaXHKqirH1kJsXkkjgbm9vlxUxPhcFTTtp5BcNAAPEWFlRbkmI5Vh1c62ZZjV0s1WwkGGvpJIH7/E8DdfNgxTKMrq20OMY5c7vUvdytioaSSd5Po2YCVelJHHK0slY17T3hw3CRxxxNDImNY0dwaNgFavr8/ct2A3v8svK3xUF9VG733uXT9fgq6OH3yeWV3+uo8m1ub9RbMxwl+oscu9bVAdQ2VzekLD47Ev23GzD1Gq+UMx7JrLrHQGptjqXFYrNS0WOCGPlpooIm7SQt280ObIXbt7+Us8NlaGvNX2y23WAU10t9NWQhweI6iJsjQ4dx2cCN1DwbW1QrhWVDQ4AEBoyAvy1zy1N8slIS4BB9FNPCbEkG+t7c+5Q08nHohW41YLprFktskpqy+xiiszZmcrxRAh0kwB8JHhgafRHuOjgTL694liuSuifkeM2m6uhBEZraKOcsB7+XnB2+ZZUAAAAbAL+qFxHEpcRq3VbsidLcBwCkqOjjo4GwNzA9TzUT+Njhjs+ZaXjJtNsOoaW/wCMPdVexrXRMifW0jthNHyxgc7m7Ne3vPmvAG7lDbgytObV3EXiVRhtNUF1vrO2ucrWnkhoNi2o7Q9wBY5zRv3uc0DrsreV56W3W+hkmloqGnp31D+eZ0UTWGR3pcQOp695UvQ7TzUlBJQyN394EAk6X1vzHHgo+qwSOoq21THbtrXAGttOiip5SPE71ftFrXe7VRyVMFgvLKmuEbS4xQPikZ2h29yHlgJ/CCjT5PHFL9duICkyaitsz7XY6GrfW1XIeyjMsLo2M5u7mcX7hvfs1x8CrR3sZIx0cjA5rgQ5pG4IPgV+FvttutNMKO1W+mo6dpJEVPE2NgJ7zytAC8Um0TqXC34buX3ri99A7XK3xXqowds9c2s3rWtlbiNM16VXf5TnE72zN8UzkUUj7RNaTazUNaSyOojmkk5XHuBc2Xdu/fyu27irEF+NXR0lwp30dfSw1MEg2fFMwPY4esHoVHYPiRwmrbVBu9a4I01W5iNEK+nMBNr8eig15MPE8goaTNswrbZPBarkKKko6iRha2okjMxk5N/bBvO0EjpudvA7dF4t+DKl1sldn2Bz01uzGKIMqI5jywXRjRs0PcPaSgAAP7iAGu2ADmyjiiigjbDDG2ONgDWsaNg0DuAA7gvtbM+P1D8SdiUHsONstRYACx56LDFhULaMUcvtAcdM73uOSo7zfTfPdNrm60Z3iVzslUCQ0VcBayT1xv8AaSD1tJHrWvQU89VMympYJJpZDysjjaXOcfQAOpV8FTS01bA+lrKeKeGQbPjlYHNcPQQehXjtuOY9ZpHS2ew26he8bOdTUrIiR6y0DdWePb4hn8yC7u51h7j8VCO2UG97MuXTP3qs3h64EdRNSbjTXzUmgrMUxdjmvkZUxmOvrW9/JHE4bxgj3bwO/wA0O8LDsuwOkGjd+01wu3QUUMuOVlnttMzoyPnpnxxt6+sjcnr4lbqiq2J49VYrM2WXINNw0aD5lTlDhUFDGWMzJ1PFUY2nC8rvmVxYPbLBXTX6aq9hCgELhM2YO5S1zdt27Hfffu2JO2yvHoIHUtDT0zyC6GJkZI7iQAF/I7db4qyS4xUNOyrmaGSTtiaJHtHcC7bcj416Fnx/HzjnZ+xuhl+N7k2vwHJYsKwkYZv+1vb1uFtL/NQ848OF5+f2h+r+BWt0uSWqENutJAzd9xpGjpI1o9tLGPncwbdS1oMG+H/GL5lmtWGWmw2+aqqGXujqZQxpIihimY+SR3oa1rSSfUrp1jbdjON2iuqrnacfttFWVx5qqop6SOOWc9+73NALvnJW3hu1c1DROo3t3siGm+l+B5gcPJYK3AY6qpFQ127zFtf3+qqd41mZyziJyj69vZfI6cG0GXm7I2/Ydj2O/Tl29ty+759+u64Wr2rpYrHfGsZerNQ3BsRJYKqnZKGk9+3MDssd9j/A/wDQmwfo2H+6pOi23ZTU7IXQfZAGRsMu6y0qnZl08zpBLqb5j9VRst60k0U1C1qyOnx7CLFUVDHyBtTXvjcKSjZ4vlk22Gw68vtj3AE9Fcf9j/A/9CbB+jYf7qzNHRUdvp2UdBSQ00EY2ZFDGGMaPUB0CyT7el0ZEENncybgeFs/NeItlQHgyyXHcP1WuaX6fWjSvT6xae2Nzn0lkpG04lcNnTSEl0kpHgXvc9xHgXLaURc+kkdK8yPNyTc9SraxjY2hjRYBERF4XpERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERf/2Q==</v>
+      </c>
+      <c r="N4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Bill should be address to JB COMMUNICATIONS.
+xerox copy of the following should be attached along with the bill.
+(a) Purchase order, (b)Necessary supporting document
+Terms of payment withing 45 days of the submission of the bill.
+In case of any variation or non conformity to your specification, the said bill shall not be eligible for any payment.
+Payment shall be process on the completion of job/delivery of materials to our satisfaction only . All dispute are subject
+to Guwahati Jurisdiction.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>id</v>
       </c>
       <c r="B1" t="str">
-        <v>specification_id</v>
+        <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>value</v>
+        <v>created_by</v>
       </c>
       <c r="D1" t="str">
-        <v>is_active</v>
+        <v>created_at</v>
       </c>
       <c r="E1" t="str">
-        <v>created_by</v>
+        <v>updated_by</v>
       </c>
       <c r="F1" t="str">
-        <v>created_at</v>
-      </c>
-      <c r="G1" t="str">
-        <v>updated_by</v>
-      </c>
-      <c r="H1" t="str">
         <v>updated_at</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SVAL-4753d66d-2ee2-4521-9922-72a71cb21c3d</v>
+        <v>ICAT-1c40a062-9e9b-4647-bdd9-6a52143bc460</v>
       </c>
       <c r="B2" t="str">
-        <v>SPEC-404b1e09-ae1f-4f77-8ef7-3ab8aaa26251</v>
+        <v>Category 1</v>
       </c>
       <c r="C2" t="str">
-        <v>3mm</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>system</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-04-21T10:16:02.402Z</v>
       </c>
       <c r="E2" t="str">
         <v>system</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-11T10:16:05.888Z</v>
-      </c>
-      <c r="G2" t="str">
-        <v>system</v>
-      </c>
-      <c r="H2" t="str">
-        <v>2026-04-11T10:16:05.888Z</v>
+        <v>2026-04-21T10:16:02.402Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SVAL-9c3a89d1-9d89-47c9-824f-ccc3f06306e3</v>
+        <v>ICAT-f1a08ea5-8240-4253-8abf-9e47c97f4a1b</v>
       </c>
       <c r="B3" t="str">
-        <v>SPEC-404b1e09-ae1f-4f77-8ef7-3ab8aaa26251</v>
+        <v>Category 2</v>
       </c>
       <c r="C3" t="str">
-        <v>5mm</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
+        <v>system</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-04-21T10:16:12.634Z</v>
       </c>
       <c r="E3" t="str">
         <v>system</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-04-11T10:16:12.503Z</v>
-      </c>
-      <c r="G3" t="str">
-        <v>system</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2026-04-11T10:16:12.503Z</v>
+        <v>2026-04-21T10:16:12.634Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SVAL-684d8e7e-891e-486f-a312-da373a3783ae</v>
+        <v>ICAT-3207409b-b935-456d-945b-e0ad2700308f</v>
       </c>
       <c r="B4" t="str">
-        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
+        <v>ACP Sheet</v>
       </c>
       <c r="C4" t="str">
-        <v>GOLD(glossy)</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
+        <v>system</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-04-24T13:03:58.137Z</v>
       </c>
       <c r="E4" t="str">
         <v>system</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-04-11T10:17:34.687Z</v>
-      </c>
-      <c r="G4" t="str">
-        <v>system</v>
-      </c>
-      <c r="H4" t="str">
-        <v>2026-04-11T10:17:34.687Z</v>
+        <v>2026-04-24T13:03:58.137Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SVAL-22d313eb-62ce-4331-89e0-294ec960db8e</v>
+        <v>ICAT-7d81d3cb-d58b-484e-b9d9-f7055e03b8fb</v>
       </c>
       <c r="B5" t="str">
-        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
+        <v>Electrical Items</v>
       </c>
       <c r="C5" t="str">
-        <v>ROSE-GOLD(glossy)</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
+        <v>system</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-04-24T13:04:47.274Z</v>
       </c>
       <c r="E5" t="str">
         <v>system</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-04-11T10:17:53.183Z</v>
-      </c>
-      <c r="G5" t="str">
-        <v>system</v>
-      </c>
-      <c r="H5" t="str">
-        <v>2026-04-11T10:17:53.183Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>SVAL-4dbb2b70-0c3e-4160-8cfe-68e282871756</v>
-      </c>
-      <c r="B6" t="str">
-        <v>SPEC-58e069a4-3bcb-436d-af2a-9b7b07f301a8</v>
-      </c>
-      <c r="C6" t="str">
-        <v>ddd</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="str">
-        <v>system</v>
-      </c>
-      <c r="F6" t="str">
-        <v>2026-04-11T10:53:53.681Z</v>
-      </c>
-      <c r="G6" t="str">
-        <v>system</v>
-      </c>
-      <c r="H6" t="str">
-        <v>2026-04-11T10:53:53.681Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>SVAL-0ad45ad2-1c75-4b0c-904d-f9f93b592f91</v>
-      </c>
-      <c r="B7" t="str">
-        <v>SPEC-58e069a4-3bcb-436d-af2a-9b7b07f301a8</v>
-      </c>
-      <c r="C7" t="str">
-        <v>5213</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="str">
-        <v>system</v>
-      </c>
-      <c r="F7" t="str">
-        <v>2026-04-11T11:00:38.155Z</v>
-      </c>
-      <c r="G7" t="str">
-        <v>system</v>
-      </c>
-      <c r="H7" t="str">
-        <v>2026-04-11T11:00:38.155Z</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>SVAL-6711c6da-9794-4895-9ca8-8a96476122d8</v>
-      </c>
-      <c r="B8" t="str">
-        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
-      </c>
-      <c r="C8" t="str">
-        <v>66kk</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="str">
-        <v>system</v>
-      </c>
-      <c r="F8" t="str">
-        <v>2026-04-11T12:04:36.170Z</v>
-      </c>
-      <c r="G8" t="str">
-        <v>system</v>
-      </c>
-      <c r="H8" t="str">
-        <v>2026-04-11T12:04:36.170Z</v>
+        <v>2026-04-24T13:04:47.274Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:I12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>id</v>
       </c>
       <c r="B1" t="str">
-        <v>item_name_id</v>
+        <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>item_code</v>
+        <v>category</v>
       </c>
       <c r="D1" t="str">
-        <v>specifications_json</v>
+        <v>created_by</v>
       </c>
       <c r="E1" t="str">
-        <v>unique_key</v>
+        <v>created_at</v>
       </c>
       <c r="F1" t="str">
-        <v>description</v>
+        <v>updated_by</v>
       </c>
       <c r="G1" t="str">
-        <v>unit</v>
+        <v>updated_at</v>
       </c>
       <c r="H1" t="str">
-        <v>is_active</v>
+        <v>unit_id</v>
       </c>
       <c r="I1" t="str">
-        <v>created_by</v>
-      </c>
-      <c r="J1" t="str">
-        <v>created_at</v>
-      </c>
-      <c r="K1" t="str">
-        <v>updated_by</v>
-      </c>
-      <c r="L1" t="str">
-        <v>updated_at</v>
+        <v>item_category_id</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ITEM-3f67bd42-a0db-4971-87dc-1aaf0a3dff05</v>
+        <v>INAME-dac69e05-de04-45b7-9a04-1ad9d5146b57</v>
       </c>
       <c r="B2" t="str">
-        <v>INAME-dac69e05-de04-45b7-9a04-1ad9d5146b57</v>
+        <v>Item AAA</v>
       </c>
       <c r="C2" t="str">
-        <v>ITEM-F8DC9EA0</v>
+        <v>Category 1</v>
       </c>
       <c r="D2" t="str">
-        <v>{"Wire":"3mm","Paint":"ddd"}</v>
+        <v>system</v>
       </c>
       <c r="E2" t="str">
-        <v>ccff95a59c20cb51808e0e0e6a942fc91e43c348bf07522ffc56a9beb27551e0</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
+        <v>2026-04-11T10:33:55.418Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v>system</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-04-21T10:17:54.366Z</v>
+      </c>
+      <c r="H2" t="str">
+        <v>UNIT-30922999-42e8-45ba-96e9-05a337e77b41</v>
       </c>
       <c r="I2" t="str">
-        <v>system</v>
-      </c>
-      <c r="J2" t="str">
-        <v>2026-04-11T10:53:53.681Z</v>
-      </c>
-      <c r="K2" t="str">
-        <v>system</v>
-      </c>
-      <c r="L2" t="str">
-        <v>2026-04-11T10:53:53.681Z</v>
+        <v>ICAT-1c40a062-9e9b-4647-bdd9-6a52143bc460</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ITEM-eb445764-d6e4-4ba4-9cc7-f01eee138890</v>
+        <v>INAME-f48a847e-7e4b-428a-acda-afce1f2c9094</v>
       </c>
       <c r="B3" t="str">
-        <v>INAME-dac69e05-de04-45b7-9a04-1ad9d5146b57</v>
+        <v>dddd</v>
       </c>
       <c r="C3" t="str">
-        <v>ITEM-701E6FD6</v>
+        <v>Category 2</v>
       </c>
       <c r="D3" t="str">
-        <v>{"Steel":"66kk","Paint":"ddd"}</v>
+        <v>system</v>
       </c>
       <c r="E3" t="str">
-        <v>782cc0e665d5b9edb7af6ecd525d3f4d562d91bc9f6538a03f6f655c20ceae80</v>
+        <v>2026-04-12T06:42:37.062Z</v>
       </c>
       <c r="F3" t="str">
-        <v>wdscx</v>
+        <v>system</v>
       </c>
       <c r="G3" t="str">
-        <v>ds</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
+        <v>2026-04-21T10:17:38.319Z</v>
+      </c>
+      <c r="H3" t="str">
+        <v>UNIT-30922999-42e8-45ba-96e9-05a337e77b41</v>
       </c>
       <c r="I3" t="str">
-        <v>system</v>
-      </c>
-      <c r="J3" t="str">
-        <v>2026-04-12T06:06:26.254Z</v>
-      </c>
-      <c r="K3" t="str">
-        <v>system</v>
-      </c>
-      <c r="L3" t="str">
-        <v>2026-04-12T06:06:26.254Z</v>
+        <v>ICAT-f1a08ea5-8240-4253-8abf-9e47c97f4a1b</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>INAME-38ba5a01-e685-453f-bba8-4a2d53ca6ecc</v>
+      </c>
+      <c r="B4" t="str">
+        <v>gjedsfvcfds</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Category 2</v>
+      </c>
+      <c r="D4" t="str">
+        <v>system</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-04-12T06:54:17.140Z</v>
+      </c>
+      <c r="F4" t="str">
+        <v>system</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-04-21T10:17:45.799Z</v>
+      </c>
+      <c r="H4" t="str">
+        <v>UNIT-9fd34519-c330-46d3-a628-7b661a216079</v>
+      </c>
+      <c r="I4" t="str">
+        <v>ICAT-f1a08ea5-8240-4253-8abf-9e47c97f4a1b</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>INAME-42fe2278-980a-4214-9188-6d984e4b7997</v>
+      </c>
+      <c r="B5" t="str">
+        <v>12</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Category 1</v>
+      </c>
+      <c r="D5" t="str">
+        <v>system</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-04-20T07:01:20.930Z</v>
+      </c>
+      <c r="F5" t="str">
+        <v>system</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-04-21T10:17:30.982Z</v>
+      </c>
+      <c r="H5" t="str">
+        <v>UNIT-c972386c-560d-438f-9fa9-a8bbfebf830b</v>
+      </c>
+      <c r="I5" t="str">
+        <v>ICAT-1c40a062-9e9b-4647-bdd9-6a52143bc460</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>INAME-05816031-b29a-4354-8449-d435aa01e811</v>
+      </c>
+      <c r="B6" t="str">
+        <v>silv</v>
+      </c>
+      <c r="D6" t="str">
+        <v>system</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-04-21T11:07:44.769Z</v>
+      </c>
+      <c r="F6" t="str">
+        <v>system</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-04-21T11:07:44.769Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>INAME-ab6c1f52-c9dc-4254-8757-0ef4f32e0bde</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Pen</v>
+      </c>
+      <c r="D7" t="str">
+        <v>system</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-04-21T11:08:15.599Z</v>
+      </c>
+      <c r="F7" t="str">
+        <v>system</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-04-21T11:08:15.599Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>INAME-106b6fc7-34dd-4f0e-9759-fb4f7f0b20c9</v>
+      </c>
+      <c r="B8" t="str">
+        <v>bott</v>
+      </c>
+      <c r="D8" t="str">
+        <v>system</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-04-21T11:09:54.198Z</v>
+      </c>
+      <c r="F8" t="str">
+        <v>system</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-04-21T11:09:54.198Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>INAME-81d85224-259d-4d91-b7b3-365ea3d99e7c</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bottle</v>
+      </c>
+      <c r="D9" t="str">
+        <v>system</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-04-21T11:10:02.354Z</v>
+      </c>
+      <c r="F9" t="str">
+        <v>system</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-04-21T11:10:02.354Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>INAME-f57af96d-2e35-4fc2-86b7-a46bc4df16a1</v>
+      </c>
+      <c r="B10" t="str">
+        <v>c</v>
+      </c>
+      <c r="D10" t="str">
+        <v>system</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-04-21T11:48:53.079Z</v>
+      </c>
+      <c r="F10" t="str">
+        <v>system</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-04-21T11:48:53.079Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>INAME-ae300898-5b1a-4b85-b82d-c647478e7687</v>
+      </c>
+      <c r="B11" t="str">
+        <v>ui</v>
+      </c>
+      <c r="D11" t="str">
+        <v>system</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-04-21T12:04:11.942Z</v>
+      </c>
+      <c r="F11" t="str">
+        <v>system</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-04-21T12:04:11.942Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>INAME-e0893cbb-365e-4c05-970c-9cdeeb46946a</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Wire</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Electrical Items</v>
+      </c>
+      <c r="D12" t="str">
+        <v>system</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-04-24T13:05:30.298Z</v>
+      </c>
+      <c r="F12" t="str">
+        <v>system</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-04-24T13:05:30.298Z</v>
+      </c>
+      <c r="H12" t="str">
+        <v>UNIT-c972386c-560d-438f-9fa9-a8bbfebf830b</v>
+      </c>
+      <c r="I12" t="str">
+        <v>ICAT-7d81d3cb-d58b-484e-b9d9-f7055e03b8fb</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Name</v>
+        <v>id</v>
       </c>
       <c r="B1" t="str">
-        <v>Category</v>
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>created_by</v>
+      </c>
+      <c r="D1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="E1" t="str">
+        <v>updated_by</v>
+      </c>
+      <c r="F1" t="str">
+        <v>updated_at</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>SPEC-404b1e09-ae1f-4f77-8ef7-3ab8aaa26251</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Wire</v>
+      </c>
+      <c r="C2" t="str">
+        <v>system</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-04-11T10:15:38.662Z</v>
+      </c>
+      <c r="E2" t="str">
+        <v>system</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-04-11T10:15:38.662Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>Steel</v>
+      </c>
+      <c r="C3" t="str">
+        <v>system</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-04-11T10:17:13.668Z</v>
+      </c>
+      <c r="E3" t="str">
+        <v>system</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-04-11T10:17:13.668Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>SPEC-58e069a4-3bcb-436d-af2a-9b7b07f301a8</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Paint</v>
+      </c>
+      <c r="C4" t="str">
+        <v>system</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-04-11T10:26:05.774Z</v>
+      </c>
+      <c r="E4" t="str">
+        <v>system</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-04-11T10:26:05.774Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>SPEC-b186aceb-106c-4c31-82ad-6ff5fa01638c</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>Color</v>
+      </c>
+      <c r="C5" t="str">
+        <v>system</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-04-21T11:09:05.923Z</v>
+      </c>
+      <c r="E5" t="str">
+        <v>system</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-04-21T11:09:05.923Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>SPEC-5526d08b-17f3-4cfd-9fc7-5cc4306b9ab3</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>Material</v>
+      </c>
+      <c r="C6" t="str">
+        <v>system</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-04-21T11:09:37.187Z</v>
+      </c>
+      <c r="E6" t="str">
+        <v>system</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-04-21T11:09:37.187Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>SPEC-47fa81ef-33f4-427b-8711-154b0e9044ed</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>Lid</v>
+      </c>
+      <c r="C7" t="str">
+        <v>system</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-04-21T11:10:22.226Z</v>
+      </c>
+      <c r="E7" t="str">
+        <v>system</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-04-21T11:10:22.226Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>SPEC-425d474f-4211-46fa-858b-658f6671b608</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>Size</v>
+      </c>
+      <c r="C8" t="str">
+        <v>system</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-04-21T11:10:39.084Z</v>
+      </c>
+      <c r="E8" t="str">
+        <v>system</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-04-21T11:10:39.084Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>SPEC-9988104a-6eee-461c-9195-d11662e85e62</v>
       </c>
       <c r="B9" t="str">
-        <v/>
+        <v>Shape</v>
+      </c>
+      <c r="C9" t="str">
+        <v>system</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-04-21T11:11:43.846Z</v>
+      </c>
+      <c r="E9" t="str">
+        <v>system</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-04-21T11:11:43.846Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>SPEC-6b4a9bf9-f2f1-495e-8ecc-df3548485811</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>Make</v>
+      </c>
+      <c r="C10" t="str">
+        <v>system</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-04-24T13:08:33.988Z</v>
+      </c>
+      <c r="E10" t="str">
+        <v>system</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-04-24T13:08:33.988Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>SPEC-42581c22-a215-4436-8f17-941797305689</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>Brand</v>
+      </c>
+      <c r="C11" t="str">
+        <v>system</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2026-04-24T13:10:00.742Z</v>
+      </c>
+      <c r="E11" t="str">
+        <v>system</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-04-24T13:10:00.742Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>SPEC-6ff96d44-8bdd-4aab-b4e0-4edc18529e5f</v>
       </c>
       <c r="B12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v/>
-      </c>
-      <c r="B13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v/>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v/>
-      </c>
-      <c r="B16" t="str">
-        <v/>
+        <v>Thickness</v>
+      </c>
+      <c r="C12" t="str">
+        <v>system</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2026-04-24T13:11:13.152Z</v>
+      </c>
+      <c r="E12" t="str">
+        <v>system</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-04-24T13:11:13.152Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H26"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>specification_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>value</v>
+      </c>
+      <c r="D1" t="str">
+        <v>is_active</v>
+      </c>
+      <c r="E1" t="str">
+        <v>created_by</v>
+      </c>
+      <c r="F1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="G1" t="str">
+        <v>updated_by</v>
+      </c>
+      <c r="H1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SVAL-4753d66d-2ee2-4521-9922-72a71cb21c3d</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SPEC-404b1e09-ae1f-4f77-8ef7-3ab8aaa26251</v>
+      </c>
+      <c r="C2" t="str">
+        <v>3mm</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>system</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-04-11T10:16:05.888Z</v>
+      </c>
+      <c r="G2" t="str">
+        <v>system</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2026-04-11T10:16:05.888Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SVAL-9c3a89d1-9d89-47c9-824f-ccc3f06306e3</v>
+      </c>
+      <c r="B3" t="str">
+        <v>SPEC-404b1e09-ae1f-4f77-8ef7-3ab8aaa26251</v>
+      </c>
+      <c r="C3" t="str">
+        <v>5mm</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>system</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-04-11T10:16:12.503Z</v>
+      </c>
+      <c r="G3" t="str">
+        <v>system</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-04-11T10:16:12.503Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SVAL-684d8e7e-891e-486f-a312-da373a3783ae</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
+      </c>
+      <c r="C4" t="str">
+        <v>GOLD(glossy)</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>system</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-04-11T10:17:34.687Z</v>
+      </c>
+      <c r="G4" t="str">
+        <v>system</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-04-11T10:17:34.687Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SVAL-22d313eb-62ce-4331-89e0-294ec960db8e</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ROSE-GOLD(glossy)</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>system</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-04-11T10:17:53.183Z</v>
+      </c>
+      <c r="G5" t="str">
+        <v>system</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-04-11T10:17:53.183Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>SVAL-4dbb2b70-0c3e-4160-8cfe-68e282871756</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SPEC-58e069a4-3bcb-436d-af2a-9b7b07f301a8</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ddd</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>system</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-04-11T10:53:53.681Z</v>
+      </c>
+      <c r="G6" t="str">
+        <v>system</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-04-11T10:53:53.681Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SVAL-0ad45ad2-1c75-4b0c-904d-f9f93b592f91</v>
+      </c>
+      <c r="B7" t="str">
+        <v>SPEC-58e069a4-3bcb-436d-af2a-9b7b07f301a8</v>
+      </c>
+      <c r="C7" t="str">
+        <v>5213</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>system</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-04-11T11:00:38.155Z</v>
+      </c>
+      <c r="G7" t="str">
+        <v>system</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-04-11T11:00:38.155Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SVAL-6711c6da-9794-4895-9ca8-8a96476122d8</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
+      </c>
+      <c r="C8" t="str">
+        <v>66kk</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>system</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-04-11T12:04:36.170Z</v>
+      </c>
+      <c r="G8" t="str">
+        <v>system</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-04-11T12:04:36.170Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>SVAL-29073161-d3bd-41b4-9562-506e7eef385c</v>
+      </c>
+      <c r="B9" t="str">
+        <v>SPEC-404b1e09-ae1f-4f77-8ef7-3ab8aaa26251</v>
+      </c>
+      <c r="C9" t="str">
+        <v>75mm</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="str">
+        <v>system</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-04-17T10:07:31.233Z</v>
+      </c>
+      <c r="G9" t="str">
+        <v>system</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-04-17T10:07:31.233Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>SVAL-b74c13e0-9c38-4549-9f0b-ea150079036d</v>
+      </c>
+      <c r="B10" t="str">
+        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Silver (Flashy)</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>system</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-04-20T07:02:26.248Z</v>
+      </c>
+      <c r="G10" t="str">
+        <v>system</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-04-20T07:02:26.248Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>SVAL-8c29b1c8-7765-4355-acf1-64d04b747e96</v>
+      </c>
+      <c r="B11" t="str">
+        <v>SPEC-b186aceb-106c-4c31-82ad-6ff5fa01638c</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Green</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="str">
+        <v>system</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-04-21T11:09:13.447Z</v>
+      </c>
+      <c r="G11" t="str">
+        <v>system</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-04-21T11:09:13.447Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>SVAL-50012dac-d153-45d8-a074-c901925c653b</v>
+      </c>
+      <c r="B12" t="str">
+        <v>SPEC-5526d08b-17f3-4cfd-9fc7-5cc4306b9ab3</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Plastic</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="str">
+        <v>system</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-04-21T11:09:43.102Z</v>
+      </c>
+      <c r="G12" t="str">
+        <v>system</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-04-21T11:09:43.102Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>SVAL-1a59dfa5-002d-4d9e-82c1-4ebee6a80a4c</v>
+      </c>
+      <c r="B13" t="str">
+        <v>SPEC-47fa81ef-33f4-427b-8711-154b0e9044ed</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Plastic</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="str">
+        <v>system</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-04-21T11:10:29.047Z</v>
+      </c>
+      <c r="G13" t="str">
+        <v>system</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2026-04-21T11:10:29.047Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>SVAL-583fdcfd-c788-4332-8312-f43b488163e2</v>
+      </c>
+      <c r="B14" t="str">
+        <v>SPEC-425d474f-4211-46fa-858b-658f6671b608</v>
+      </c>
+      <c r="C14" t="str">
+        <v>500 ML</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>system</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-04-21T11:10:53.327Z</v>
+      </c>
+      <c r="G14" t="str">
+        <v>system</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2026-04-21T11:10:53.327Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>SVAL-ed68c3c1-ffd9-4dfa-a8ac-b83dffc0c1db</v>
+      </c>
+      <c r="B15" t="str">
+        <v>SPEC-9988104a-6eee-461c-9195-d11662e85e62</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Round</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="str">
+        <v>system</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-04-21T11:11:50.054Z</v>
+      </c>
+      <c r="G15" t="str">
+        <v>system</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2026-04-21T11:11:50.054Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>SVAL-d5ebd179-b443-4741-a175-656789f20557</v>
+      </c>
+      <c r="B16" t="str">
+        <v>SPEC-6b4a9bf9-f2f1-495e-8ecc-df3548485811</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Flexible</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="str">
+        <v>system</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-04-24T13:09:12.841Z</v>
+      </c>
+      <c r="G16" t="str">
+        <v>system</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2026-04-24T13:09:12.841Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>SVAL-1634e63e-dc06-4ca4-a17c-628db71ba814</v>
+      </c>
+      <c r="B17" t="str">
+        <v>SPEC-6b4a9bf9-f2f1-495e-8ecc-df3548485811</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Copper</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="str">
+        <v>system</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2026-04-24T13:09:30.568Z</v>
+      </c>
+      <c r="G17" t="str">
+        <v>system</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2026-04-24T13:09:30.568Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>SVAL-1ec3a80b-3f7b-4ecb-92e9-907309545f31</v>
+      </c>
+      <c r="B18" t="str">
+        <v>SPEC-6b4a9bf9-f2f1-495e-8ecc-df3548485811</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Aluminium</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="str">
+        <v>system</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2026-04-24T13:09:42.179Z</v>
+      </c>
+      <c r="G18" t="str">
+        <v>system</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2026-04-24T13:09:42.179Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>SVAL-48783b0c-46ab-4fd6-83e3-bebfba1fc24c</v>
+      </c>
+      <c r="B19" t="str">
+        <v>SPEC-42581c22-a215-4436-8f17-941797305689</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Anchor</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="str">
+        <v>system</v>
+      </c>
+      <c r="F19" t="str">
+        <v>2026-04-24T13:10:13.710Z</v>
+      </c>
+      <c r="G19" t="str">
+        <v>system</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2026-04-24T13:10:13.710Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>SVAL-a9330473-cbb3-43e0-b0f5-1066674f5eea</v>
+      </c>
+      <c r="B20" t="str">
+        <v>SPEC-42581c22-a215-4436-8f17-941797305689</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Havells</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="str">
+        <v>system</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2026-04-24T13:10:43.313Z</v>
+      </c>
+      <c r="G20" t="str">
+        <v>system</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2026-04-24T13:10:43.313Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>SVAL-88d33802-0c63-4a7e-b2d3-3176895e0a5b</v>
+      </c>
+      <c r="B21" t="str">
+        <v>SPEC-42581c22-a215-4436-8f17-941797305689</v>
+      </c>
+      <c r="C21" t="str">
+        <v>KEI</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="str">
+        <v>system</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2026-04-24T13:10:50.929Z</v>
+      </c>
+      <c r="G21" t="str">
+        <v>system</v>
+      </c>
+      <c r="H21" t="str">
+        <v>2026-04-24T13:10:50.929Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>SVAL-42674f02-874d-49db-99bd-9a48e6eae3bc</v>
+      </c>
+      <c r="B22" t="str">
+        <v>SPEC-6ff96d44-8bdd-4aab-b4e0-4edc18529e5f</v>
+      </c>
+      <c r="C22" t="str">
+        <v>0.5 mm</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="str">
+        <v>system</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2026-04-24T13:11:31.249Z</v>
+      </c>
+      <c r="G22" t="str">
+        <v>system</v>
+      </c>
+      <c r="H22" t="str">
+        <v>2026-04-24T13:11:31.249Z</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>SVAL-d87cc8ad-82bb-405c-97fe-fd425da43408</v>
+      </c>
+      <c r="B23" t="str">
+        <v>SPEC-6ff96d44-8bdd-4aab-b4e0-4edc18529e5f</v>
+      </c>
+      <c r="C23" t="str">
+        <v>1 mm</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="str">
+        <v>system</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2026-04-24T13:11:37.777Z</v>
+      </c>
+      <c r="G23" t="str">
+        <v>system</v>
+      </c>
+      <c r="H23" t="str">
+        <v>2026-04-24T13:11:37.777Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>SVAL-a7a639e5-07a2-4805-bf8c-9771ceed7b59</v>
+      </c>
+      <c r="B24" t="str">
+        <v>SPEC-6ff96d44-8bdd-4aab-b4e0-4edc18529e5f</v>
+      </c>
+      <c r="C24" t="str">
+        <v>2 mm</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="str">
+        <v>system</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2026-04-24T13:11:43.536Z</v>
+      </c>
+      <c r="G24" t="str">
+        <v>system</v>
+      </c>
+      <c r="H24" t="str">
+        <v>2026-04-24T13:11:43.536Z</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>SVAL-1e068149-6e2e-4d87-8068-2e7a15cc9c1a</v>
+      </c>
+      <c r="B25" t="str">
+        <v>SPEC-b186aceb-106c-4c31-82ad-6ff5fa01638c</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Red</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25" t="str">
+        <v>system</v>
+      </c>
+      <c r="F25" t="str">
+        <v>2026-04-24T13:16:50.777Z</v>
+      </c>
+      <c r="G25" t="str">
+        <v>system</v>
+      </c>
+      <c r="H25" t="str">
+        <v>2026-04-24T13:16:50.777Z</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>SVAL-488d8efa-7ac4-4a7f-bb6a-ce9db9103e72</v>
+      </c>
+      <c r="B26" t="str">
+        <v>SPEC-6ff96d44-8bdd-4aab-b4e0-4edc18529e5f</v>
+      </c>
+      <c r="C26" t="str">
+        <v>4 mm</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26" t="str">
+        <v>system</v>
+      </c>
+      <c r="F26" t="str">
+        <v>2026-04-24T13:17:15.106Z</v>
+      </c>
+      <c r="G26" t="str">
+        <v>system</v>
+      </c>
+      <c r="H26" t="str">
+        <v>2026-04-24T13:17:15.106Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>item_name_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>item_code</v>
+      </c>
+      <c r="D1" t="str">
+        <v>specifications_json</v>
+      </c>
+      <c r="E1" t="str">
+        <v>unique_key</v>
+      </c>
+      <c r="F1" t="str">
+        <v>description</v>
+      </c>
+      <c r="G1" t="str">
+        <v>unit</v>
+      </c>
+      <c r="H1" t="str">
+        <v>is_active</v>
+      </c>
+      <c r="I1" t="str">
+        <v>created_by</v>
+      </c>
+      <c r="J1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="K1" t="str">
+        <v>updated_by</v>
+      </c>
+      <c r="L1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ITEM-3f67bd42-a0db-4971-87dc-1aaf0a3dff05</v>
+      </c>
+      <c r="B2" t="str">
+        <v>INAME-dac69e05-de04-45b7-9a04-1ad9d5146b57</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ITEM-F8DC9EA0</v>
+      </c>
+      <c r="D2" t="str">
+        <v>{"Wire":"3mm","Paint":"ddd"}</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ccff95a59c20cb51808e0e0e6a942fc91e43c348bf07522ffc56a9beb27551e0</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="str">
+        <v>system</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2026-04-11T10:53:53.681Z</v>
+      </c>
+      <c r="K2" t="str">
+        <v>system</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2026-04-11T10:53:53.681Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ITEM-eb445764-d6e4-4ba4-9cc7-f01eee138890</v>
+      </c>
+      <c r="B3" t="str">
+        <v>INAME-dac69e05-de04-45b7-9a04-1ad9d5146b57</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ITEM-701E6FD6</v>
+      </c>
+      <c r="D3" t="str">
+        <v>{"Steel":"66kk","Paint":"ddd"}</v>
+      </c>
+      <c r="E3" t="str">
+        <v>782cc0e665d5b9edb7af6ecd525d3f4d562d91bc9f6538a03f6f655c20ceae80</v>
+      </c>
+      <c r="F3" t="str">
+        <v>wdscx</v>
+      </c>
+      <c r="G3" t="str">
+        <v>ds</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" t="str">
+        <v>system</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2026-04-12T06:06:26.254Z</v>
+      </c>
+      <c r="K3" t="str">
+        <v>system</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2026-04-12T06:06:26.254Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ITEM-1bf4b9cf-227a-46d9-81fd-d9e74643a35c</v>
+      </c>
+      <c r="B4" t="str">
+        <v>INAME-dac69e05-de04-45b7-9a04-1ad9d5146b57</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ITEM-A8110768</v>
+      </c>
+      <c r="D4" t="str">
+        <v>{"Wire":"75mm","Steel":"GOLD(glossy)"}</v>
+      </c>
+      <c r="E4" t="str">
+        <v>781cd2ac721d2db8b9e79a8f48ee1c511ea1b4c99d780d1ad0c944f236fa1f28</v>
+      </c>
+      <c r="F4" t="str">
+        <v>vhjbhj</v>
+      </c>
+      <c r="G4" t="str">
+        <v>kg</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="str">
+        <v>system</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2026-04-17T10:07:44.585Z</v>
+      </c>
+      <c r="K4" t="str">
+        <v>system</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2026-04-17T10:07:44.585Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ITEM-3afb9f80-26c6-455c-9ac2-b146bbab2c95</v>
+      </c>
+      <c r="B5" t="str">
+        <v>INAME-f48a847e-7e4b-428a-acda-afce1f2c9094</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ITEM-98DC1ED0</v>
+      </c>
+      <c r="D5" t="str">
+        <v>{"Steel":"Silver (Flashy)"}</v>
+      </c>
+      <c r="E5" t="str">
+        <v>e9e36a35ae2d1866c4dad1f887e3fd8b993770bd62334859d810d87a2521efb8</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5" t="str">
+        <v>system</v>
+      </c>
+      <c r="J5" t="str">
+        <v>2026-04-20T07:02:30.636Z</v>
+      </c>
+      <c r="K5" t="str">
+        <v>system</v>
+      </c>
+      <c r="L5" t="str">
+        <v>2026-04-20T07:02:30.636Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ITEM-0bf5a113-f693-4dc7-8cad-79df1492049e</v>
+      </c>
+      <c r="B6" t="str">
+        <v>INAME-ab6c1f52-c9dc-4254-8757-0ef4f32e0bde</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ITEM-DF38112D</v>
+      </c>
+      <c r="D6" t="str">
+        <v>{"Color":"Green","Material":"Plastic"}</v>
+      </c>
+      <c r="E6" t="str">
+        <v>82d138ed0e8d39ebd538366311159fa31cec3642b7eff2f2276f6d7197d170b8</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Ink the pen.</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Nos</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="str">
+        <v>system</v>
+      </c>
+      <c r="J6" t="str">
+        <v>2026-04-21T11:09:45.159Z</v>
+      </c>
+      <c r="K6" t="str">
+        <v>system</v>
+      </c>
+      <c r="L6" t="str">
+        <v>2026-04-21T11:09:45.159Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ITEM-11d31d6e-5399-4532-a639-a320c6d9e3d0</v>
+      </c>
+      <c r="B7" t="str">
+        <v>INAME-81d85224-259d-4d91-b7b3-365ea3d99e7c</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ITEM-085944B0</v>
+      </c>
+      <c r="D7" t="str">
+        <v>{"Color":"Green","Lid":"Plastic","Size":"500 ML","Shape":"Round"}</v>
+      </c>
+      <c r="E7" t="str">
+        <v>1c0f51b25695db5ad43fbe677fe7ce6a979da7cd55c09a8bbf4b645771ef350f</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Nos</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="str">
+        <v>system</v>
+      </c>
+      <c r="J7" t="str">
+        <v>2026-04-21T11:11:51.918Z</v>
+      </c>
+      <c r="K7" t="str">
+        <v>system</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2026-04-21T11:11:51.918Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ITEM-47a00781-e386-495a-aef8-005fb3ee2077</v>
+      </c>
+      <c r="B8" t="str">
+        <v>INAME-e0893cbb-365e-4c05-970c-9cdeeb46946a</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ITEM-9BD25B53</v>
+      </c>
+      <c r="D8" t="str">
+        <v>{"Brand":"Anchor","Color":"Green","Thickness":"0.5 mm"}</v>
+      </c>
+      <c r="E8" t="str">
+        <v>10c7ef8b5bd1785dba65c2fe8b9ab3aa11a9e77aaf9d9d353f3e4481ba244a00</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Inch</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8" t="str">
+        <v>system</v>
+      </c>
+      <c r="J8" t="str">
+        <v>2026-04-24T13:12:43.952Z</v>
+      </c>
+      <c r="K8" t="str">
+        <v>system</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2026-04-24T13:12:43.952Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ITEM-be881e83-46dc-443e-8557-d191eaa20648</v>
+      </c>
+      <c r="B9" t="str">
+        <v>INAME-e0893cbb-365e-4c05-970c-9cdeeb46946a</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ITEM-659613F7</v>
+      </c>
+      <c r="D9" t="str">
+        <v>{"Brand":"Havells","Color":"Red","Thickness":"4 mm"}</v>
+      </c>
+      <c r="E9" t="str">
+        <v>35812378f502ed820e5d1301b7c9cd3526232f0e8aa650025994c7d5405f2f4c</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Inch</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="str">
+        <v>system</v>
+      </c>
+      <c r="J9" t="str">
+        <v>2026-04-24T13:17:18.841Z</v>
+      </c>
+      <c r="K9" t="str">
+        <v>system</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-04-24T13:17:18.841Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C16"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Category</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I16"/>
   <sheetData>
@@ -1447,7 +2946,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1527,16 +3026,88 @@
         <v>2026-04-11T08:38:18.325Z</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>STORE-23f370d3-cfc1-4c20-b45c-d1429303c5a3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>FIRM-1</v>
+      </c>
+      <c r="C4" t="str">
+        <v>dsadasdsadsad</v>
+      </c>
+      <c r="E4" t="str">
+        <v>system</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-04-20T05:06:53.010Z</v>
+      </c>
+      <c r="G4" t="str">
+        <v>system</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-04-20T05:06:53.010Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>STORE-6ce2bb76-4b27-4fca-b325-5db3ef96bad8</v>
+      </c>
+      <c r="B5" t="str">
+        <v>FIRM-a7ed8c9d-a4f2-47b5-b070-c7e82f1aaa49</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Default Store</v>
+      </c>
+      <c r="E5" t="str">
+        <v>system</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-04-23T11:38:28.553Z</v>
+      </c>
+      <c r="G5" t="str">
+        <v>system</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-04-23T11:38:28.553Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>STORE-424b2e01-769d-431d-b225-2957ed67968b</v>
+      </c>
+      <c r="B6" t="str">
+        <v>FIRM-2</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ground Floor</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Bishnupur</v>
+      </c>
+      <c r="E6" t="str">
+        <v>system</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-04-24T12:59:41.777Z</v>
+      </c>
+      <c r="G6" t="str">
+        <v>system</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-04-24T12:59:41.777Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1566,16 +3137,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>USER-1</v>
+        <v>USER-6</v>
       </c>
       <c r="B2" t="str">
-        <v>Alex Thompson</v>
+        <v>Amit Jain</v>
       </c>
       <c r="C2" t="str">
-        <v>employee</v>
+        <v>Owner</v>
+      </c>
+      <c r="D2" t="str">
+        <v>9864081643</v>
       </c>
       <c r="E2" t="str">
-        <v>alex@example.com</v>
+        <v>amit@umangcommunications.com</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1583,57 +3157,20 @@
       <c r="G2" t="str">
         <v>2026-04-11T08:38:18.325Z</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>USER-2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Dept Head</v>
-      </c>
-      <c r="C3" t="str">
-        <v>approver</v>
-      </c>
-      <c r="E3" t="str">
-        <v>head@example.com</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-04-11T08:38:18.325Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>USER-6</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Accounts Team</v>
-      </c>
-      <c r="C4" t="str">
-        <v>accounts</v>
-      </c>
-      <c r="E4" t="str">
-        <v>accounts@example.com</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="str">
-        <v>2026-04-11T08:38:18.325Z</v>
+      <c r="H2" t="str">
+        <v>scrypt$CmJnHsE2TdI/A8CPBAW+vA==$2OESBk79KPevC6zHdXPOL9W4p8qmF4rnSvd/7EuXzVue0M4KyzplkiJBMPNy42sC9bXlNGme6g4dND9kh4dlog==</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1672,6 +3209,9 @@
       <c r="L1" t="str">
         <v>payment_terms</v>
       </c>
+      <c r="M1" t="str">
+        <v>gst_type</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1680,6 +3220,15 @@
       <c r="B2" t="str">
         <v>Supplier 1</v>
       </c>
+      <c r="C2" t="str">
+        <v>18AABCU2874Q5ZH</v>
+      </c>
+      <c r="D2" t="str">
+        <v>8638215544</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Paltan Bazar, Guwahati</v>
+      </c>
       <c r="H2" t="str">
         <v>system</v>
       </c>
@@ -1690,7 +3239,13 @@
         <v>system</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-04-11T10:14:50.786Z</v>
+        <v>2026-04-20T10:11:38.294Z</v>
+      </c>
+      <c r="L2" t="str">
+        <v>29</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Intra-State</v>
       </c>
     </row>
     <row r="3">
@@ -1700,6 +3255,15 @@
       <c r="B3" t="str">
         <v>ABCD Traders</v>
       </c>
+      <c r="C3" t="str">
+        <v>18AABCU2874Q5ZH</v>
+      </c>
+      <c r="D3" t="str">
+        <v>986402369</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Nalbari, Assam</v>
+      </c>
       <c r="H3" t="str">
         <v>system</v>
       </c>
@@ -1710,7 +3274,13 @@
         <v>system</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-04-11T10:15:23.373Z</v>
+        <v>2026-04-20T10:10:56.454Z</v>
+      </c>
+      <c r="L3" t="str">
+        <v>25</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Inter-State</v>
       </c>
     </row>
     <row r="4">
@@ -1720,6 +3290,15 @@
       <c r="B4" t="str">
         <v>ghg</v>
       </c>
+      <c r="C4" t="str">
+        <v>18AABCU2874Q5ZH</v>
+      </c>
+      <c r="D4" t="str">
+        <v>8638215773</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Paltan Bazar Ghy</v>
+      </c>
       <c r="H4" t="str">
         <v>system</v>
       </c>
@@ -1730,52 +3309,223 @@
         <v>system</v>
       </c>
       <c r="K4" t="str">
-        <v>2026-04-12T12:34:06.002Z</v>
+        <v>2026-04-20T10:10:18.285Z</v>
       </c>
       <c r="L4" t="str">
         <v>15</v>
       </c>
+      <c r="M4" t="str">
+        <v>Intra-State</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>phone</v>
+      </c>
+      <c r="D1" t="str">
+        <v>created_by</v>
+      </c>
+      <c r="E1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="F1" t="str">
+        <v>updated_by</v>
+      </c>
+      <c r="G1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TRN-e300d8b2-3a52-4ecb-85ba-795bc3c92bfc</v>
+      </c>
+      <c r="B2" t="str">
+        <v>DTDC</v>
+      </c>
+      <c r="C2" t="str">
+        <v>9864023964</v>
+      </c>
+      <c r="D2" t="str">
+        <v>system</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-04-18T06:35:25.229Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v>system</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-04-18T06:35:25.229Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TRN-72b24fc3-eb23-4f26-8a84-9ecf81dc78c1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Good Luck</v>
+      </c>
+      <c r="D3" t="str">
+        <v>system</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-04-18T06:35:34.552Z</v>
+      </c>
+      <c r="F3" t="str">
+        <v>system</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-04-18T06:35:34.552Z</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:J1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>gst_number</v>
+      </c>
+      <c r="D1" t="str">
+        <v>phone</v>
+      </c>
+      <c r="E1" t="str">
+        <v>email</v>
+      </c>
+      <c r="F1" t="str">
+        <v>address</v>
+      </c>
+      <c r="G1" t="str">
+        <v>created_by</v>
+      </c>
+      <c r="H1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="I1" t="str">
+        <v>updated_by</v>
+      </c>
+      <c r="J1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:K2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>firm_id</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>client_name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>start_date</v>
+      </c>
+      <c r="F1" t="str">
+        <v>end_date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>created_by</v>
+      </c>
+      <c r="I1" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="J1" t="str">
+        <v>updated_by</v>
+      </c>
+      <c r="K1" t="str">
+        <v>updated_at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PROJ-838a7e51-20c3-483e-ba25-7fc92e56fb50</v>
+      </c>
+      <c r="B2" t="str">
+        <v>FIRM-1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Testing Project</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Bizskill</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-04-21</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-04-23</v>
+      </c>
+      <c r="H2" t="str">
+        <v>system</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-04-20T07:22:31.626Z</v>
+      </c>
+      <c r="J2" t="str">
+        <v>system</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-04-20T07:22:31.626Z</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:F1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1785,91 +3535,28 @@
         <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>category</v>
+        <v>created_by</v>
       </c>
       <c r="D1" t="str">
-        <v>created_by</v>
+        <v>created_at</v>
       </c>
       <c r="E1" t="str">
-        <v>created_at</v>
+        <v>updated_by</v>
       </c>
       <c r="F1" t="str">
-        <v>updated_by</v>
-      </c>
-      <c r="G1" t="str">
         <v>updated_at</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>INAME-dac69e05-de04-45b7-9a04-1ad9d5146b57</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Item AAA</v>
-      </c>
-      <c r="D2" t="str">
-        <v>system</v>
-      </c>
-      <c r="E2" t="str">
-        <v>2026-04-11T10:33:55.418Z</v>
-      </c>
-      <c r="F2" t="str">
-        <v>system</v>
-      </c>
-      <c r="G2" t="str">
-        <v>2026-04-11T10:33:55.418Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>INAME-f48a847e-7e4b-428a-acda-afce1f2c9094</v>
-      </c>
-      <c r="B3" t="str">
-        <v>dddd</v>
-      </c>
-      <c r="D3" t="str">
-        <v>system</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-04-12T06:42:37.062Z</v>
-      </c>
-      <c r="F3" t="str">
-        <v>system</v>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-04-12T06:42:37.062Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>INAME-38ba5a01-e685-453f-bba8-4a2d53ca6ecc</v>
-      </c>
-      <c r="B4" t="str">
-        <v>gjedsfvcfds</v>
-      </c>
-      <c r="D4" t="str">
-        <v>system</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2026-04-12T06:54:17.140Z</v>
-      </c>
-      <c r="F4" t="str">
-        <v>system</v>
-      </c>
-      <c r="G4" t="str">
-        <v>2026-04-12T06:54:17.140Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1893,87 +3580,67 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SPEC-404b1e09-ae1f-4f77-8ef7-3ab8aaa26251</v>
+        <v>UNIT-9fd34519-c330-46d3-a628-7b661a216079</v>
       </c>
       <c r="B2" t="str">
-        <v>Wire</v>
+        <v>Nos</v>
       </c>
       <c r="C2" t="str">
         <v>system</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-04-11T10:15:38.662Z</v>
+        <v>2026-04-21T10:15:29.510Z</v>
       </c>
       <c r="E2" t="str">
         <v>system</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-04-11T10:15:38.662Z</v>
+        <v>2026-04-21T10:15:29.510Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SPEC-9b0e6d9b-b623-4918-8aa5-1c7111a0a71a</v>
+        <v>UNIT-30922999-42e8-45ba-96e9-05a337e77b41</v>
       </c>
       <c r="B3" t="str">
-        <v>Steel</v>
+        <v>KG</v>
       </c>
       <c r="C3" t="str">
         <v>system</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-04-11T10:17:13.668Z</v>
+        <v>2026-04-21T10:15:35.282Z</v>
       </c>
       <c r="E3" t="str">
         <v>system</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-04-11T10:17:13.668Z</v>
+        <v>2026-04-21T10:15:35.282Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SPEC-58e069a4-3bcb-436d-af2a-9b7b07f301a8</v>
+        <v>UNIT-c972386c-560d-438f-9fa9-a8bbfebf830b</v>
       </c>
       <c r="B4" t="str">
-        <v>Paint</v>
+        <v>Inch</v>
       </c>
       <c r="C4" t="str">
         <v>system</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-04-11T10:26:05.774Z</v>
+        <v>2026-04-21T10:15:46.866Z</v>
       </c>
       <c r="E4" t="str">
         <v>system</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-04-11T10:26:05.774Z</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>SPEC-a6bd89c7-c958-474e-8dd1-ab4a17ebdabc</v>
-      </c>
-      <c r="B5" t="str">
-        <v>dcyh</v>
-      </c>
-      <c r="C5" t="str">
-        <v>system</v>
-      </c>
-      <c r="D5" t="str">
-        <v>2026-04-12T07:27:27.053Z</v>
-      </c>
-      <c r="E5" t="str">
-        <v>system</v>
-      </c>
-      <c r="F5" t="str">
-        <v>2026-04-12T07:27:27.053Z</v>
+        <v>2026-04-21T10:15:46.866Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
commit to git hub
</commit_message>
<xml_diff>
--- a/data/master_data.xlsx
+++ b/data/master_data.xlsx
@@ -3404,7 +3404,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3438,9 +3438,36 @@
         <v>updated_at</v>
       </c>
     </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>CUS-ab8e166e-76ce-4900-8581-ad335405f06a</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABCD</v>
+      </c>
+      <c r="D2" t="str">
+        <v>09864023964</v>
+      </c>
+      <c r="F2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Paltan Bazar
+Sanmati Bhawan</v>
+      </c>
+      <c r="G2" t="str">
+        <v>system</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2026-04-28T10:13:22.154Z</v>
+      </c>
+      <c r="I2" t="str">
+        <v>system</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2026-04-28T10:13:22.154Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Download pdf & Excel
</commit_message>
<xml_diff>
--- a/data/master_data.xlsx
+++ b/data/master_data.xlsx
@@ -412,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,6 +457,9 @@
       <c r="N1" t="str">
         <v>terms_conditions</v>
       </c>
+      <c r="O1" t="str">
+        <v>sort_name</v>
+      </c>
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
@@ -484,7 +487,7 @@
         <v>system</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-04-22T12:34:58.074Z</v>
+        <v>2026-04-29T05:49:47.940Z</v>
       </c>
       <c r="L2" t="str">
         <v>U74900AS2011PTC010451</v>
@@ -500,6 +503,9 @@
 4.In case of any variation or non conformity to your specification, the said bill shall not be eligible for any payment.
 5.Payment shall be process on the completion of job/delivery of materials to our satisfaction only . All dispute are subject to Guwahati Jurisdiction.</v>
       </c>
+      <c r="O2" t="str">
+        <v>UC</v>
+      </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
@@ -527,7 +533,7 @@
         <v>system</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-04-21T06:43:54.353Z</v>
+        <v>2026-04-29T05:50:00.253Z</v>
       </c>
       <c r="L3" t="str">
         <v>U74900AS2011PTC010451</v>
@@ -544,6 +550,9 @@
 Payment shall be process on the completion of job/delivery of materials to our satisfaction only . All dispute are subject
 to Guwahati Jurisdiction.</v>
       </c>
+      <c r="O3" t="str">
+        <v>UC 2</v>
+      </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
@@ -574,7 +583,7 @@
         <v>system</v>
       </c>
       <c r="K4" t="str">
-        <v>2026-04-21T06:43:29.695Z</v>
+        <v>2026-04-29T05:49:37.302Z</v>
       </c>
       <c r="M4" t="str">
         <v>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/4gHYSUNDX1BST0ZJTEUAAQEAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADb/2wBDAAMCAgICAgMCAgIDAwMDBAYEBAQEBAgGBgUGCQgKCgkICQkKDA8MCgsOCwkJDRENDg8QEBEQCgwSExIQEw8QEBD/2wBDAQMDAwQDBAgEBAgQCwkLEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBD/wAARCAD2AfIDASIAAhEBAxEB/8QAHQABAAIDAQEBAQAAAAAAAAAAAAgJBQYHBAIDAf/EAGMQAAEDAwIDAwQJDQoICgsAAAEAAgMEBQYHEQgSIRMxQQkiUWEUMkJSV3F2gbQVFhcYNzhidZGUldHTIzNVcoKTobKz0iQoNkdWY3R3GSdTZoWSlqKxtTQ1RGRlc4OjpMHD/8QAHAEBAAIDAQEBAAAAAAAAAAAAAAUGAwQHAgEI/8QAQBEAAQMCAwUFBAgFBAIDAAAAAQACAwQRBSExBhJBUXETYYGRoSKxwdEUFjIzUlPh8BUjNUJyNJKy8TZUYqKj/9oADAMBAAIRAxEAPwC1NERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERFr901CwGyVn1PvWcY/QVXNy9hVXOGKTf0crnA7rN0tVS11OyroqmKoglHMyWJ4exw9II6Fe3RvaAXCwK8h7XGwK/VEReF6RF46m8Wmil7CsulJBJtvySzta7b4iV+f1w2D+HLf+cs/WvQY46BfN4c1kEWP+uGwfw5b/AM5Z+tPrhsH8OW/85Z+tNx3JfN4c1kEWP+uGwfw5b/zln60+uGwfw5b/AM5Z+tNx3JN4c1kEWP8ArhsH8OW/85Z+tPrhsH8OW/8AOWfrTcdyTeHNZBFj/rhsH8OW/wDOWfrXsp6mnqoxNSzxzRnufG4OB+cL4WkahfQQdF+iIi+L6iIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIirt46+KjLZ80r9GsBvdRarRZwILvU0khjmraktBfFztO4jYCGlo25nc++4AViSpD1brJ7jqtmdfUu5pqnILjLIfS51TIT/4q57FUMVVVvllF9wZA8ydfBVzaWqkgp2xxm28c+gWpklxLnEknqSfFb/pLrrqZoreobrg+SVMFO2QPqLbLI59FVN36tkiJ5TuOnMNnDfoQtARdTmhjqGGOVoLTwKoscj4nB8ZsRyV3OkmpFp1d05seodljMVPeKbtHQudzGCZriyWInx5Xtc3fx238VFLj14pcjwm4xaN6cXeW218lM2pvdxpn8s8LJOsdPG4dY3Fuz3OGx5XMAI3K3vyc88s3DqI5HlzYL7Wxxg+5btG7b8rifnVf3Edcq+66+6h1dycXTtyW4U438I4p3Rxj5mMaPmXNcCwaB2NTRvF2RE2B65X52HqrpimIyjDY3tNnPtc+GfmueVFRUVc76mqnkmmlcXPkkcXOc495JPUlfCIunaKkIiIvqIiIiIiIiIsjZMjyHGattwxy/XG1VTCHNnoqp8EgPpDmEFY5F5c0OFnC4X0EtNwpR6Q+UE1iwOeGgzmRmaWYOAeKwiOujb+BOB5x8f3QOJ7twrD9JNYMF1rxSLLsFunsmnJEdTTyAMqKOXbcxys3PK719QR1BI6qk1dB0N1qyvQnO6TMsamdJDuIrjQOeWxV1Nv50b/AEHxa7Y8rtj16g1LG9lKaujMtI0MkHLIHuI0HXzVgwzHpqZ4ZUHeZ36j98ldOiwWDZpYNRMRtWbYxViotl4pm1MD/EA97HDwc1wLXDwLSPBZ1clex0bixwsRkVfmuDwHN0KIiLyvqIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiKjzU37pOWfjyv8ApD1eGqPNTfuk5Z+PK/6Q9dA2C+9n6N95VT2r+7i6n4LWkRF0tUtWh+Tj+94k+UFb/UhXF+OjhSy1uY3HWjT60VF2td1aKi80lKznmop2tDXTBg850bwA5xAJa7nJ2aRt2jycf3vEnygrf6kKkxeb3Z8ctdRe8gutJbbfSM7SoqquZsUUTfS57iAB8a4/UYpPhOOTTQC5LiCOYvp8l0KKiir8LjjlNsgb8lRIQQdiNiEVh2sHEVwGXe9zSX7TwZnXmT93uFpszI3SO8S6d74XSfHu4egrL6PWTgA1urPqRiGC26nvHKXi13Lt6epe0Dcln7qWSbDckMc4gDcgBXh20kkMHbz0kjRxyFh6g+YCrIwZskvZRTsJ6/8AfvVbSK4P7Tnhn+CS1fz0/wC0T7Tnhn+CS1fz0/7RaH17ofy3+nzW19Vqr8bfX5KnxFcH9pzwz/BJav56f9on2nPDP8Elq/np/wBon17ofy3+nzT6rVX42+vyVPiK4P7Tnhn+CS1fz0/7RPtOeGf4JLV/PT/tE+vdD+W/0+afVaq/G31+Sp8RWzZNwIcNORUjoKfCJ7LOWkNqrbcJ2PZv4hsjnxn52lQC4nuGe+8OmUU1K+vN1x67h77Xcez5HHlI54ZWjoJGhzeo6OBBG3VrZbC9pqHFZOxju1/AOGvSxIWhXYLVUDO0fYt5jh10XFkRFYVEKfHkzdU55osj0duNRzMp2/Vy2Bx6taXNjqGD1bmJwA8S8+KngqhOC7JZMX4lcLqA8iKvqZbZK0H24nhfG0H4nuYfmCt7XINsqRtNiRe0ZPAd46H3X8V0LZyoM1Huu/tNvDUe9ERFU1PIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIqPNTfuk5Z+PK/wCkPV4ao81N+6Tln48r/pD10DYL72fo33lVPav7uLqfgtaREXS1S1aH5OP73iT5QVv9SFRU47NcL9qJq5dMCp6+WPGsQqXUMNIxxDJqtg5ZppB7pwfzMbv3Nb02Lnbyr8nH97xJ8oK3+pCq9Nduut+oZP8ApVdvpcqoWC08cu0FVK8XLSbd1zqrViUz2YTAxpyda/gFo69dou9zsF0pL3Za+air6CZlRTVELy2SKRp3a5pHcQQvIivhAcLFVYEg3Cuq0H1JGrukWM6guaxtRdKMezGMGzW1UbjHMAPAdox+3qIW/KAvBlxVaN6S6N/WdqJltRQXGK61M8ULbfUThsDwwjZ0bHN6u5ztvuu7jj14XfhAqR/0LW/slxTEcCrIquRkELiwONrNJFr5cF0mjxSmfTsdLI0OsL3I1Ug0UfRx58Lnwhz/AKFrv2K+hx5cLfwjTD/oWv8A2K0v4NiP/rv/ANrvktn+I0f5rf8AcPmpAIuAfb48LXwkS/oWv/Yr5l48+FyNhezUSeQj3LbLXbn8sIH9KfwbEf8A13/7XfJP4jR/mt/3D5qQKh35TS9WKDSbHMfqjG67Vl+bVUjNxzthigkbK/07byxt+Nw9C+M98pdplaaeaDT3Erzf60DaOasDaOl39O+7pDt6ORu/pHeoI6s6uZvrTl02ZZ1chUVb2iKCGJpZBSwgkiKJm55WjcnvJJJJJJJVp2a2brWVjKupbuNbnnqT04d91B4zjNM6ndBCd4uy7gtMREXUFSFvegk0tPrnp5LCSHtyq1bbeO9XGCPnV1qp94O8NnzXiNwukjgc+G114vNQ4d0bKUdq1x9RkbG343BXBLl23cjTVxMGob7z+ivGyzCKd7joT8EREVFVoRERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERUeam/dJyz8eV/0h6vDVHmpv3Scs/Hlf9IeugbBfez9G+8qp7V/dxdT8FrSIi6WqWrQ/Jx/e8SfKCt/qQqvTXX7t2oXyqu30uVWF+Tj+94k+UFb/UhVemuv3btQvlVdvpcqpOA/1ut6/FWXFf6ZTdPgtHREV2VaRERERERERERERERERfcEE1TNHTU0L5ZZXBkcbGlznuJ2AAHUknwXwurcNestl0O1Ipcwv2FUWQUoAie6Rm9VRA981MSeUSAekdRuA5u5KwVMkkUTnxN3nAZC9r911khYx8ga926DqeSnjwO8NFboxitTmmZ0fY5bkkTWup3gc9voweZsJ9D3nZzx4crG97TvKFYLCM2xjUXF6DMcOu0VxtVyjEkE0Z+YtcO9r2ncFp6gggrOrhGI1c9bVPmqftk5jlbK3gup0cEVNA2OH7I9e/xRERaS2UREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREXEOKviToeHbDKero6OG4ZLenPhtNHKT2Y5AOeaXYg8jOZvQEFxcBuBuR29Va+UTySpvPERPZ5JSYbDaaOkiZ4NL2mdx+M9sOvqHoU/s1hseJ4g2KbNoBcRztw8yFE41WPoqQvj+0TYeP6Ll2X8TOvecV0lde9VchYJHb+x6GtfR07R4ARQlrenpIJ9JK9OC8Uuven1yhuFo1MvVZFE4F1FdKt9bTSN36tMcpOwPcS0td6CFylF2A4fSGPsuybu8rCy56KuoD9/fN+dyrneHrWu0696aUWc2+nbSVYe6judEHc3sarYAXNB8WkOa9p7+V4367rpagZ5Lm7VLmah2J73GnYbbVxt36Ne72Q15+MhrP8Aqqea4vjtEzDsQlp4/sg5dCAbeF7LpGF1LqykZM/U6+BsiIiiFIIiIiIqPNTfuk5Z+PK/6Q9XhqjjUaZlTqFk9REd2S3mte0+kGd5C6BsF97P0b7yqltX9iLqfgteREXS1TFaH5OP73iT5QVv9SFV5a5HfWvUA+nKbr9LlViXk6IHw8OjJHNIE18rXtJ8RtG3f8rT+RV162nfWfPj6cnuv0uRUnAc8brevxVlxX+m03T4LS0RFdlWluuIaK6s5/aTfsK09vd6t7ZnQGpo6V0kYkaAXN3HiA4flWaPDBxDD/M3lf6Ok/Up5eTg+96n+UVZ/ZwqU655iW2VTQ1clO2NpDSRx+at1Fs7DU07JnPILhfgqZDwx8Qo/wAzWWfoyT9S/h4ZeIQf5msu/Rcv6lc4i0fr5V/lN9fmtr6rQfmH0VMY4ZOIRwJGjWW9PTa5R/8ApY646Ca4WiIz3HSDM4Im98jrHU8g+NwZsrrUXobeVV84m+ZXw7KwcJD6Kh6toK621L6O40c9LUR+3injLHt+Np6hfgry8swXDM7oHWvM8VtV6pXNLezrqVk3Lv4tLhu0+sbEKB3FnwLW3CLDXanaNsqfqXQNM9zskj3SupoQN3TQvcS5zGjq5rtyBu4O2GwnsL2xpa+QQzt7Nx0zuL9creXioqu2dnpWGSJ28BrwPkoSoiK4quqSnBDxD1WkOokGH36ucMSymoZT1LXu8yjq3bNiqR70b8rH/gkE78gVqioXVyHCzqQ/VTQnFcnq6gzXCOk+p9wc47vNTTns3Pd63hrZP5a5rtxhjY3Mr4x9rJ3XgfK48ArnsxWl4dSvOmY6cQusIiLnytqIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiKqryhNCKTiUuc4iLfZtsoJydvb7Rdnv8A/b2+ZWqqu7ynmKy02b4bmrIHdlcLXNbHyAdOeCUyAH1kVB29PKfQrZsZKI8UDT/c0j4/BQO0kZfQkjgQfh8VChERdfXPVNjyX94jgzbOLAduettVLWN9O0MzmH+3CsQVNvC/q3HotrPY8xrpHttMjnW+6hvX/BJvNc7YdTyO5JNvHswFcZR1dLcKSGvoamKopqmNs0M0Tw5kjHDdrmuHQgggghck21pHw4h25HsvAz7xkR7vNX/ZqobJSdlxaT5HP5r9kRFT1YURERFgs6yikwnCr9mFc8MgsttqK95PiI43O29ZO2wHiSqNpZJJpHzSvL3vcXOcT1JPeVY/5RbW6lxvBYNHLLWsddslLKi5NYd3U9Ax3M0H0GSRoA/BY/fvCreXVdiKF1PRvqXi3aHLoOPmSqJtNVNmqGwt/sGfU/sIiL12i1V99u1FY7VTuqK241EdJTQt75JZHBrGj1lxAV1JAFyq2ASbBW08EVkksfDHhkU0RZLVxVVc7cbbiWqlew/9QsVZGvtuqrTrjn9DWxlkrMluT9j4tdUPc13xFrgR8auTw3G6XDsRsmJUW3sey26mt8Ww23bFG1gP/dUAvKIaBXi2Zedb8ctslRZ7vFFDeTCzf2JVMaGNleB3MewMHN3BzTud3jfmOy+KRnF5i827W5HW9wPK6uuOULxh8Ybn2dr9LWuoWIi2fTrTPNtVslp8UwWw1Fyrp3DnLGnsqdhOxklf3RsHi4/ENzsF0ySRkTS+Q2A1JVLYx0jg1ouSrHPJxRvZw8yOewgSZBWOaSO8ckI3Hzgj5lKVaJofpbQ6M6XWLTuinbUOtkBNVUBuwnqZHF8rx47F7jsD3NDR4Le1wfFallXXSzx/Zc4kdF1OghdT00cT9QBdERFHrbRERERflVUtNXUs1FWQMmp6iN0Usbxu17HDZzSPEEEhfqvPcbhRWm31N1uVSynpKOF9RPM87NjjY0uc4nwAAJX0XvlqvhtbNUc5vZIsazS/45ASY7VdKqiZud/Nilcwf1VhVl8wvv10Zbe8l5HM+q1xqa7ld3jtZXP2P/WWIX6Gi3uzbv62F1yJ9t47uiKxnyYmQPq9N8vxh8nMLbeoqxoPuRUQhv5N6c/0quZT+8lw0i16jP8ATUWsfkbU/rVd2vaHYRITwLf+QHxUxs84jEGAcb+4qdSIi40ujIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIuEcamlc+qmg14prXRmou9ge29UDGjd73RAiVg8STC6TYDvcGru6LYpKl9HOyoj1aQfJYaiFtTE6J+hFlQuikLxp6A1GjGqFRdrPQcmKZPLJW210bfMp5Sd5qY+95XHdo945u25a7aPS7zR1cddA2oiPsuF/wBOo0XLKmnfSyuhk1CKUHDDxu5JotSwYVmtHUZBiEZ2gbG8ezLcD4QlxAfH/q3Ebe5cO4xfRea2hp8RiMFS27fd3jkV9pqqWjk7WE2Kui064h9GdU6SGfD8/tM1RN09gVE7aesa70GCTZ/q3AIPgSujKhdZCDIsgpYzFS324QsI2LY6p7QR6NgVSZ9goy68ExA5EX9QR7lZYtqnhtpY7nuNvSx96u9yfN8NwqkNdl+V2iyU4G/aXCtjgB+LnI3PqCixrh5RHAcXoqqyaPxHJr05pYy4yxujt9O733nbPmI9AAaffHuVbcksk0jpZpHSPcd3OcdyT6yvlblDsRSU7g+peZLcLWHjqfVa9VtNUSt3YWhvfqfh7llcqyrIc3yGuyvK7tPcrtcpTNU1Ux3c93d3DoAAAA0AAAAAABYpEV0a1rGhrRYBVskuNzqilT5PfR2pzjVsah3Cj5rJhg7cPePNlr3tIhYPSWDmkO3cWs39sFHfT7Acm1OzC24PiFAau53SYRRt7mRt73SPPuWNaC5x8ACritD9IbFofpxbMAsT+3NMDNW1ZYGuq6p+xklI8N9gAOuzWtG523VU2txhtBSGmYf5kgt0bxPwH6KewDDzVVAmcPYZn1PAfE/qt9X51FPBVwSUtVDHNDMwxyRyNDmvaRsWkHoQR4L9FBfjw4rMkxa9v0W02u0ttqI4GSX25Uz+WdpkbzMpo3DqzzC17nN6+c0AjZ2/MsLw2bFakU8GupPADmrrXVkdBCZpdOXM8l1zPdJuBrGb06tzuz4DZri13O6lkuApSSeu/sZkjQR/I2WwYvr9wl4fbW2PENQMJstDEelPRFlPHv6dmtAJ9fUqoWWWSaR800jpJHuLnOcdy4nvJPiV8rox2OE0YZU1L3W78vAG6p42iMby6GFrff5iyuU+2m4dfhixj89CfbTcOvwxYx+ehU1osP1Do/zXenyWT601H4G+vzVyn203Dr8MWMfnoT7abh1+GLGPz0KmtE+odH+a70+SfWmo/A31+auU+2m4dfhixj89CfbTcOvwxYx+ehU1on1Do/zXenyT601H4G+vzVyh4p+HUAn7MWM9P/fAofcXnG/btQLJWaW6QyVH1Fq/3K63iRjonVke/WGFp2c2M+6c4AuHm7Bu5dCxFvYfsfQ0M4nJLyNL2tfnkFq1e0NTVRGIANB1tqiIitigUVmvk2cXNo0PuWRyxbS36+TPY7b20EMbI2/keJlWpabVcL7daOyWmmfU1twqI6WmhYN3SSvcGsaPWSQFdppXgdBphpzj2AW7lMVkoIqZ72jYSy7byyfG+QvcfW5UjbisEVGymGrzfwH62Vm2Ypy+pdMdGj1P6XW1IiLlavSIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIiIi03VvSnFNZsHrsEzCmL6SrAfDPHt2tJO3fkmjJ7nN3PqIJadwSFUdrfoTnOg2WSY3l1EX00rnOt1ziafY9dED7Zh8HDcczD1aT4ggm6NYDN8DxDUfHqjFc3sFJd7ZUjz4Khm/K7wexw85jxv0c0gjwKseAbRS4M/ccN6M6jl3jv7uKhsVwhmIt3gbPGh+B/eSo2RTh1g8mtfKOee7aK5HFcKU7vFou0giqGfgxzgcj/VzhmwHVxUU810U1b06lezNNO77a2M33nko3Opzt37TM3jd8ziuqUONUOIgGCQE8jkfIqjVWG1VGbSsNueo81pSIilFooiLa8I0p1J1Jqm0mC4ReL04nYyU1K4xM/jynZjB63OAXiSRkTd+QgDmcl6Yx0h3WC57lqi3DS/SXPtYsjZjGA2Ca4VJ2dPL7WCljJ/fJpD0Y3v7+p22AJ6KVejXk2sjuM8V21svkdpo2kO+pNrlbNUyeqSbrHGP4vOT6W96nTgOnWE6X49Di2B47S2i3RHm7OFpLpH+L5Hnd0jj75xJ6BU7F9saakBjo/wCY/n/aPHj4Zd6sOH7Oz1BD6n2W8uJ+Xj5LnnDZwx4hw9Y7y0ojuWT18YFzu72bOf3HsYgerIgfDvcQC7uAb2dEXL6mqlrJTNO67jqVeIII6eMRRCwCKl/iSnuVRxAaiSXYu7cZJcGN5v8AkmzubF83Zhm3q2V0CgVx0cJeV3zJ6nWfTKzTXVtdE03u20rOaoZKxoaKiNg6yBzQ0Oa0cwI5tiHEttGxtdBR1rmzG2+LAnnfTx96hNo6WSopg6MX3Tcju/RQMRfc8E9LNJTVML4ZonFj45GlrmuHeCD1BXwutrn6IiL6iIiIiIiIiIiIiIs9ieA5vnlaLfheJXe+VG4BZQUck3J63FoIaPWdgpk8P3k6rrNW02T68TR01JEWyx4/STh8sx79qiVvmtb6Wxkk7+2btsYzEMXo8MYXVDwDy4noP2Fu0mH1Fa7diblz4ea8nk9OHSrul7ZrvltAWW2388WPxSt/9IqerX1Ox9wwczWnxeSRtydbDF56CgobVQ09stlHDSUlJG2GCCCMMjijaNmta0dAAAAAF6FxvF8UkxeqNRJkNAOQ5fPvXRcPoWYfAIWeJ5lERFFreREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREREWuXjTbTrIXukv8AgOOXJ7/bOrLVBMXfGXtO6wQ4etBQS4aK4L169cepD/8AzXQEWdtVOwWa8jxKxOgicbuaPJalZ9ItJ8em9kWDTDE7ZLvv2lHZaaF2/wAbGArbGta1oa1oAA2AA6AL+osb5Hym7yT1XtrGsFmiyIiLwvSIiIiIiIi17IdPNP8ALn9rlmDY/en++uNsgqT+WRpWLt2iejdo7T6l6T4dSdtsZOxsdMzm23232Z4bn8q3VFmbUTNbuteQOVysZhjJ3i0X6LV/sWaY/Bzi/wCiKf8AuJ9izTH4OcX/AERT/wBxbQifSJvxnzKdlH+EeS1f7FmmPwc4v+iKf+4n2LNMfg5xf9EU/wDcW0In0ib8Z8ynZR/hHktX+xZpj8HOL/oin/uJ9izTH4OcX/RFP/cW0In0ib8Z8ynZR/hHktX+xZpj8HOL/oin/uL+waXaZ0z+1ptO8YifvvzMtFO07/GGLZ0T6RL+I+ZTso/wjyX5wQQUsTYKaGOKJg2axjQ1rR6AB3L9ERYVkRERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERRu4neM/FdCZZMSx2jiyDMSwOdSl5FNQBw3a6oc3qXEEERt2JHUloIJ6bxA6pR6NaRZFn7RG+soqbsqCN43a+rlIZCCPFoc4OI961ypsqqq+5hkMtXVSVN0vN5rC97iC+apqZX+rqXOc78pVx2VwCPEy6pqvu2m1uZ1z7gq7juLPogIYPtu48h8yupZlxf8RebVb6ms1Qu1rjc7dlPZpfYEcY96DDyvI9bnOPrWs/Z/14+GzPf+0lZ+0U2dFPJy4PQWGlu+tNRWXa81MYkltdJVGClpNxv2ZfHs+R48XBwbvuADsHHqX2hvC38HM36ar/2ysMm0mBUjjDHFcDi1rbepCiGYNilQO0fJYnm439AVDfhM4ktaY9cMZxu9ZxkOT2rIK1luq6O510tZytfuBKwyFxYWHZ5Ldt2tIKtIXMtNuGrRDSO6G+YFgVJQXItLBWSzzVUzGkbEMfM95ZuOh5dtwto1G1ExXSrDrhnOZ1xpbXbmNMjmM55Huc4NZGxo9s5ziAB69yQASKZjldT4vVtdQxFuQFrC5N+Qv0Vjwymmw+ncKp9+OuQHUrk3EpxfYTw/sFjgphkGWTxh7LXDMGNpmkbtkqH7HkB7w0AucPQDzKCuY8dfEjltQ59PmcVgpi4ubTWijjia30DtHh0h+d67DppbeDXih1PudDXWHNbblF7nqLhGbldd2Vrur3tY5jnbODdzyHoGt6E7bLuH/B58Nv8ABF9/Sz/1Kw0r8GwECKthcZbXJc0HyF7WUTO3EcVJkppAGcLEjzyvdQjxfjd4lcXq2TjUOS7QtcHPprpSxVEcnqLuUSAfxXtU2uGrjcxDWyrgw/KaKLG8ulG0MHac1JXkeEL3dWv/ANW7r6HO67aHqn5NXCq20VFdpJkdytt2ijLoaK5ytnpZ3D3POGh8ZPvjzDu6DvVf1xt9/wANyGe23CCqtV5s1WY5WEmOamqI3ekdQ5rh0I9G4UsKPBdp4XfRQGPHIbpHK40I/dwtA1OJYJIO3Jc08zcHoeBVxHEpqjc9G9F8i1AslLDUXKhZDDSNmG8bZZpmRNe4eIbz823jtt4qv/Szj11rxfOYLrn+SS5Lj9VMBcaGWnhY5kZPV8BY1vI9o6hvtT3EdxHadS9ZZdb/ACfdzym5yRuvVHV0Nsu/INgaqKsg8/bw52OjfsOgLyB3KvxYdmcDp3Uk0NZGC8PLSSM8gNDw1uCFkxrE5RURyU7yG7oI8SdQr2bBfrRlFkocjsFfFW225U7KqlqIju2WJ43a4fMe7vC9xIA3J2AVdvk/OJT62rtHobmdw5bVdZi6wTyu6U1W47up9z3MkPVvok3HXn6dc4+OI77HWJfYoxKv5MkyWnPs2WJ3nUNA7cO6+D5erR4hoeehLSqjUbOVMWJjD2Z3zB4bvPw49/grBDjEL6L6W7hqO/l48O5cX4n+OrOrjnNVi+iuTfUjHrPKYHXGmjY+W4zNOznh7gdogRs0N9sAXEkEAbthfGpqTPwp5Tnd2io63LrBc6ez01e6na2OUVABbNJG3ZpewCToAGkhm49tvABd4w77zfUP5W2j+o9dAq8Bw+CmiiEYNnsF7Zm7gDc8b8eCqVPitXLNJIXnNrsuAyNrDuW16M8eur2LZzT1Wp2SzZJjVdMGXGCWmibJTsces0Bja3Yt7+T2pG42BIcLO7XdLde7bSXm0VsVXQ10LKimqIXczJYntDmvaR3ggghUQqdHk+OJT2FUR6C5pcP8HqHOkxuold0jkO7n0hJ8HHdzPwuZvumhRO1ezsbofplGwAt+0ALXHOw4j3dFv4DjDxJ9HqHXDtCeB5ePvU/pJI4Y3SyvaxjAXOc47BoHeSfAKtTiN479RL7nVVaNG8mdZMZtUxhgq6aJjpbi9p2MznPadoyQeVo23b1duTs3sXlA+I760MfOimIV/Ler5BzXqaJ3nUlC7uh3Hc+Ud48I9+nngquJYdkdn43x/TqtgN/sgi4tzt38PPiFk2gxZzX/AEWnda2pHu+asAt3GnqPLwiXLUOqFIcypL+zGYbgKZnZuc+ETCpMW3JzhnONtuXmDTttu1afwe8WWsuS622jBc7yubILTkXbwubVRR89PK2F8jJI3NaCBuzlLd+XZxO24C5Lb/vIrt/vLpv/AC1y8fBj985gn+2T/RZlKPwihZRVhETbgvtlpZtxblY8lpNr6l1TTgvP9t89bnO/NW/KI/HxxD6gaPUeNYvp1chaqu+tqairr2xMfKyKMsa2OPnBDeYvcS7bccrdiNypcKvXyof+VeBfi+t/tI1Rdl6eKpxSOOZoc3PI6ZAq0Y5K+Ghe+M2OWY6hZThb4xdTbph+orc/qmZHUYjjk+QW6omjbHK4xkNMMrmAczS57DzbcwHN1PQDi2O8efEPas1iyi8ZVHd6B0wNTZpaWKOlkh36xs5W80ZA7ngk7gc3N1BxnDL/AJLa1/7u67+2hXCV0enwagdVVAMLbHdGgyu0acvBU2bEatsEJEh48e/jz8VeHpxqFjWqeF2zOsSrBUW66QiRoO3PE8dHxPA7ntcC0j0jpuNitW4k9Urlo1oxkOoFlpIai40LIYaNkwJjEs0zImvcARuG8/Nt47beKrz4MOJeXQ/NPrcyasd9ZmQzNZW8xJFBUHZrapo8B3Nft3t2PUsAM0ePSaKfhbyOeCRkkcs9tcx7CC1zTVxEEEd4IVCqcB/h2MRU0gvE9wt3i4uD3jQ+fFWuHFfpmHyTMNntab9xtqow8M/GdrVd9bLFjmf5S6+2fJ69lump5aWGPsJZTyxSRGNreXZ5buO4tJ6b7EYvXzjW11Zq7f7Xh2Vux+0Y7dqigpKSmponCQQSGMyTF7XF5cW7lp80b7AeJ4tw5fd+05+VFs+ksWM1n+7DnXyluf0qRX4YPQfxInsW/YGVhbUi9tL2yuqocQqvoYHaH7WtzfQcdVbxoJqNU6taP4vqFXU8cFXdqMuqmRjZgnje6KQtHXZpfG4gb9AQo/8AEvx7WjTW5VeC6U0dJfMgpHOhrbhOS6iopB0LGhpBmkae/qGtI2Jcd2jTqbWeu0b8ntiE1gqzT3/IjW2q3yt9tAHVlS6aYegtYCAfBz2HwUIMOxHIc/yq24di9C+tu13qG09NED3uPUucfBoALnOPQAEnuVbwjZumlqJ6qqH8pj3Bo4WaTme4fO6mcQxmaOGKCA+25rSTxzGg7yt8yXiq4icqrHVtw1fySmc47hltrHUEbfUGU/IFh/s/68fDZnv/AGkrP2inxpr5ObRvH7ND9kaWvyq7yRg1BbVyUtLG/wARE2IteQO7dzjvtvs3uW5/aG8Lfwczfpqv/bLddtRgUB7OOEkDkxtvC5B9FrNwPFJRvvksTzcb+gKjnwD8QOrGR6sS6eZflN5ya1XK3z1Ifcql9VLRyxAOEgleS4MI3YW77bub3eNhi0PTLQzSfRxlQNOMLo7RLVtDJ6gPknnkaDvymWVzn8u/Xl3238FviouOV1NiFWZ6Vm42wyyFzzsMlaMMpZqSnEU7t4/vLNYzJ8jtOIY5c8qvtSILdaKSWtqpD7mONpc7b0nYdB4lVXX3jo4grjn8mZ2vLX26hZU89NZGxsdRMgB6RPaRvJu3o55PNuSQW9NpM+Ui1f8Arewe2aRWmq5a7JnituIaerKGJ3mNPo7SUDb1QuHiq4lddkMEhfSuqqpgdv5C4vkOvM+gVb2hxORs4ggcRu62PH9FdzpJqPatWtOLDqFaA1kN4pGyyQh3N2E4JbLET48kjXN38dt/FQb4vOL7WrGNYb1p3g18djVrsD4oN4aaN09U90TJDI98jXENPP5obsOXYnclZDyausHsO63nRW71W0VwDrvZw93dMxoFREP4zA14A6Ds5D4qUOsfCho5rjd4sizG0VkF3jjbC6ut1T2Es0bfatkBDmu28CW822w32ACg2RUez2MPjro96O3s5XyOYNjrbMdVJukqMXw9r6V+6/jnbTUXHmq3ftxOJj4W7t/NQfs1/ftxuJgf527r/Mwfs1JjXbhP4UtAsFfm2TOzSr7SoZR0VFT3OESVNQ4OcGgmLZoDWucXHuA7idgeY8NGmfC5xBZNWYZW43mGN3iKnfV0kf1wRVUVVE0gPAd7GYWvaHA7bHcAnfpsrdFXYTNTOrGUt426ncb/ANnvsq++mr45hTun9s6DectAtXGtxMWu4QV51OqqwQvDnU9VSU74pR4tcOQHY93Qg+gg9VIviu4xNRbHjOn9PpxP9bsuYY3T5HW1QibJPG2bo2CMvBDQC15LgNz5uxHXfqVm8nfw6Wq5Q3CopMhubIXc3sWsuQ7F/qd2bGOI9XN8ajd5SykpaDVjE6ChpoqempsVhihhiYGsjY2pnDWtA6AAAAAKNpqnB8YxKGOmhHshxN2gA5ZZDXnnotyaHEcOo5HzSHOwGZJ1zz4LvvAVxCZvrJYsjxzUK4fVO5Y6+mlgr3RtZJNBNzjkfygAlpj9ttuQ/rvtuuu698ROBcPuOsuuUTuq7lWAi3WimePZFW4d56+0jHi89B3Dc7AxC8mld7bj8+p9+vNZHSW+3Wuiq6qokOzYoYzUOe8+oNBPzL971qPwa8Smt+2ZWfNqetvMsNtorpPW9lRktAjiaIw4uhY49R025nku5dyRF12DwuxmYmJ3YssSGDm0G3C18zlnyW9S4jI3Do/bHaOuAXHvIvx9VzXUDygev+X1U7cdulFidve49nT26mZJKGeAdNKHOLvW0M+ILUrNxl8S9kqhVU+qtxqevnR1kMFSxw9G0jDt82xU6P8Ag8+G3+CL7+ln/qWuZr5NnR272x7cKvt9sFxa13ZPmmbV07nbdOdjgHbb+9ePHvUnBjmzbQIhDZvewHz1J9VpS4XjJJkMlz3OI+QWM4evKF2bM7jTYjrJQUdguVS5sVNd6YltDK89A2VriTCSdvO3LOvXkAUs80yNuIYbfcudT+yG2W2VVyMQdt2ghidJy7+G/Lt86pa1N01yrSTNLhgmY0QguNvePOYSYp4z1ZLG4gczHDqD394IBBAm/wANOt9dqRwnakYJkdaai8YbjFwhhled3zUD6OUQkk95YWOYT70R79TudTHtnKaNrK6h+7JFwNLEixHd88lsYVjEzy6lqftgGx43HAqPtHx5cRsGZtyupyyCopO25n2U0cTaJ0W/70AG84G3QP5uf0uPjZhpHqnjOsuB23PcVn3pq1nLNA5wMlJUN27SGTbuc0/lBDh0IKpJXeeEXiPrNA88EV3nllxC+vZDd4Bu7sD3MqmN98zfzgPbM3GxIbtM7Q7Mw1VNv0TA2RmgAtvDl15eXFRuEY1JBNu1LiWu552PPpzVmeu2otVpNpHk+oVBRR1dXZ6Pnpopd+R0z3tjYXbEEtDngkAgkA9QoBaG8bmuVTrJYaXN8r+rNkv9zgt9ZRPpIY2QtmkEbXxcjWlhYXA7b7OAIO56qYvGNXUdy4VMzuNvqoqmlqqGjmgmieHMljdVQFrmuHQgggghVbaS/dVwz5Q276TGojZbDaWqw2d88YLrkXIzFmg5cszwUhjtZPBWxNieQLA5aHM+asS4v+Ml+iNWzT/T+mpK3LJoWz1U9S3nht0bx5gLARzyuHnAE7AcpIPMAoWVPGfxN1U76h+q9ewvJPLFSUzGj1Boj2AWP4so7rFxH6gNvPP7IN4kczn7+wLWmH5uyMe3q2Wf0Cs3CNkdtZaNbb5lliv753gVsMrBbnxkjkG7Y3vY70lw5fHmHcJvD8LoMNw5kzoe0JAJIaHHMXyHIdyjKuuq62sdG2TcAJAz3Rll59VjPtx+Jn4W7p/MU/7NfUPGZxNwysmbqzcXFjg4B9NTOadvSDHsR6ipk2TyfnDBktthvOO5LkN0oKgc0VVR3qnmikHqe2Ig/lWSg8nFw8xTMlknyuZrXAmN9zYGvHoPLEDt8RBWi7H9nm3Bg/8AzatoYTi5zEv/ANyuq8NOql01n0ZsGf3yhipbjWNmgq2wgiJ8sMroy9gPcHcm+3gSR4LqCxmM41YsOsFBi+M2yG32q2QNp6WmiB5Y2DuHXqT4kkkkkkkkrJrm9U+OSd74W7rSSQOQvkFcoGvZE1shu4AXPMoiIsCyoiIiKJflLZ6yLQe0R05cIpsopWT7dxaKapIB9XMGn4wFDLg2pbVWcTWBxXgR9g2ullZz7bduynlfD3+Patj29eyso4ptLKnWHRHIcRtkRkurI23C2sG276mE87Yxv03eA5n8tVBWS8XrDsjob9appaG7WWsjqoHluz4Z4nhzdwfEOb1B+IrqGyhbWYPLRsNne0P9wyP75KkY8DT4jHUOF25HyOY/fNXrIo76DcamlWrFip4cnv1uxTJ4mNbV0NwqGwQyv26vp5XkNc0nfZpPOOoIIAcel5Rr1ovhttkuuQ6n43TwRgnljuEc0r9vBkUZc959TWkrns2GVlPMYHxne5WJ8ufgrbHW08sfateLdffyW+qJPlLqurg0LstPASIanJ6dkxHiBTVLgD84B+ZRX4qeLjItcch+pWKVlws+G28uZTUrZjG+ud4zzhp2O/uWHcNG/iSt/wBF8N1H114N8/xuvqLhc22W5w1+Lioc6V7p4I+eeniLupBYeVrQdg+Q+tWyh2fkwcwYlVvAs5t28rm2vMakcOagarFmYiJaOnaTkbHnbPTv0XJeCiClqeKDBY6yQMjFRVyAk7ee2jncwfO4NHzq3lUW4pk96wfKLXltgqDTXOzVcdZTPI6NkjcCA4eIO2xHiCQrXtFuMPR7Vqw0ktZlFtxvICwNq7Tc6psDmy7ed2L3kNlYepBaebbvAPRbW2+HVE0zKuNpc0NsbZ2zJue439Fg2ZrIY43U7zZ17i/HID4Luiqt8oVbLVbuJCumtrY2y19qoqqsDNv3/lczc7eJYyM/Pv4qemqvFVoppRZai4XLNLbdrg1hNParXVR1NTO/bzWkMJEbT75+w+M9DU/qnqLe9WdQL1qFkIYytvNR2piYd2QxtaGRxNPiGMa1oPedtz1WHYnDqllS6re0tZukZ5XJI07slk2lrIXQiBpBde/TVdW0yrKt/B7rPb3ud7FhuuPTRDwEj6gh/wDRGz+hcbwbFKvO8zseFUFTFT1N9uEFuhllBLGSSvDGl23Xbdw3UtTpZXac+TtyC6XmnfBcstuVBd3xSN2dHTmqgZA0/Gxvaf8A1VHLh0+77pz8qbZ9JYrdRVTXx1c8PB7rdWsaPeFX6mAtfTxScWj1cT7itNvdlvmHZDWWG9Uk9uu1oqnU9RE48skM0btj1HoI6EeohfeUZTkeb3+ryfK7tUXS7V7w+oqp3cz5CGho/IAAAOgAAU+/KB8NUuS0H2b8Itjpbpb4mxX+mgZu6opmjZlSAOpdGNmu/A2PQMO/KeA7hnqM+yqHVvM7W8YzYZhJbY52bNuNa0+aQD7aOIjcnuLw1vXZ4GKDaGklw7+JPsC0WI4734R1y8MzovcuEVDKz6E3Qm4PC3M9FG7UTTnIdMLxR4/lMPse5VNtprjLTEEOpxO3nbG/f3Yby8w8CSPDddNw77zjUP5W2j+zes95Qof4ydy/FdB/ZrAYef8AE61DH/O2z/2ciy/SH1dBTzv1c6MnxcF47FtPVyxN0AePQrlenuFXHUbM7Vg9nmiirrzN7GpnS9GdqWktDj4AkAb+G+/VY2rpb3il+lo6qOqtl3tFWY3tJMc1NURP2PUdWua5vzELpHCiN+I3T/8AHUX/AIFSl8oNw1TVwdrvg9sdJNGxseSU0Ee5cxo2ZWAD3oAbJ6g13cHFe6rF2UmJMopsmvbkf/lci3j7+q8wYe6oo3VMerTn0sPcoL5BkGQ5tkVZkWQ3Coul4u1QZqieTzpJpXH0D5gGgbAbAAAALJ6kaeX7S3KX4bk7Gx3SnpKSpqYR3wOnp2Tdk78JokDXeG4O3pUp+APhnqMnv8OtebWtzbLaJOaxwzx7Ctqwf38A98cR7j3F+2x8whcy48/vo8t/+VbvoMC+QYrHLiZw6C26xpJtzu0ADoDn5cEkoHx0QrJdXOAHSxN/H96rx2/7yO7f7y6b/wAtcvJwY/fOYJ/tk/0WZbfgGJ1uVcCeoE9vp3Ty2HMKe7uY0bu7NlPCyR3xNZK5x9TSuL6OZ+7SzVHGdQPY7p47LcI554mbc0kB82Vrd+nMY3PA38SF5a01NPWQR5uu8eJaLe9eiexmp5X6WafJxV26r18qH/lXgX4vrf7SNTHx3iG0Oymyx361aq4wKZ0Qle2pucNPLCNt/wB0jkc18ZHocAq7+O3W/FtYtTbfS4TWsr7NjVE6kbXMGzKmoe/mldGT7ZgAY0HuJDiNwQTQ9kqKoZirXvYQGg3uCLZEK1Y/UwuoS1rgS61rHvutf4Zf8lta/wDd3W/20K4jQUwrK6mpHOLRPKyMkd45iBv/AEqSXC/iNU/Q7XnPJYntposXdaIHkebI94dLKAfS0Mi3/jhRzsf/AK7t/wDtUX9cLo1LIHVNTu8C3/iFTp2EQQ34g/8AIradZNJcm0Uz+44Fk8W8tK7tKWpa0iOspnE9nMz1OAO48HBzT1BXTaPiTqL/AMK2QaD5jUyS1tvfQyY/VO3cZKZlVGX0zj6YwCWE+4Bb05Wgz14sOHS36/4A+CgjhhyuzNfUWaqdsOd23nU7z7yTYDf3Lg13cCDUhc7bcLNcaq0XWjmpK2imfT1FPMwtfFKwlrmOB6gggghReD19PtHTMMw/mRkE9RoR3H5hb2IUsuDzOEZ9h4I8DwPeFvnDj937Tr5UW36QxYvWbrrBnXyluf0qRZThw+7/AKdfKe2/SGLFayfdfzn5SXP6VIpgf1E/4D/kVHn/AEg/yPuC6drXNVjhi4f6bdwpTT5E/bwMns5o/KAf6Stt8m3S2uo4gKyavEZqKbHKuWh5ttxMZoGuLfX2bpPmJW45DpNX6jeT1wbILJSvqLnhzq65CJg3dJSOq6htQAPUA2T4oz4lRP0r1JyDSLPrRqDjLmGttUxf2Um/ZzxOaWyRP29y5jnD0jfcdQFEQt/iWG1NJCbPDpG+Jc4jzupCQ/Q6yGokHs7rD4BoB8rK7xFxrSXi00V1YscFfTZfbrHcy0eybTdquOnqIX+IaXkCVvoczfoRuGnoMvn3EvodpxaZbpf9RrNM9jC6Ojt9Uyrqpj4NbFGSep6cztmjxIXKXYdVsl7AxO3uVir2KyndH2oeN3nddOX5VdVTUNLNW1k7IaenjdLLK92zWMaN3OJ8AACVT3xAcSuc66ZlPep7hW2uyQO5LZaYalwjp4wejnAEB0p73O29AHQBdxyPXnNcc4FLHj+TXarqMgzioq7bQT1MjnVDrNG/aWRzndSDv2IJ72PG3crHLsdUwshLnjee4At5XBJz42AN/iodm0UMjpA1ps0Eg8+HhcnJRz4gtVanWbVvIM7e9/sOqqDBbY39Oyo4/NhG3gS0cxHvnOXZce4XaCo4N7rqfdfY9NlVdUC+Wls8gY99upw5romgncmRrpZdh7blhXDNFdM6/V/VDH9PqDna26VbRVSsHWClZ580no3EbXEb952His5xNw5TQa15PY8ngqKZlorH0NppX8wip7ZGeWkZCD0EfYhhG3fuSepK6BNH7cWH0sm5uAOPE7rTYC2WROp7u9VKN/syVc7d7euPE5k+HDqtLwLM7xp3mdlziwyclfZKyOsiBOwfynzmO/Bc3dp9TirsMKy2z57iVozOwTdrb71RxVsBPeGvaDyu9DgdwR4EEKjFWFeTX1hFyx+76L3eq3qLQ510tAc7qaaRwE8Y/iyOD/X2rvQoTbXDfpFKKxg9qPX/ABPyPvKk9mq3sZzTuOTtOo+Y+CyvlOnf8VOKN9OQ7/8A40qjNwDb/bP4z1/9muP0SVSY8p0f+K3Eh/8AHz9GkUaOAUf4z2Nf7Lcfokqw4R/4xL/jJ8VkxD+ts6s+CthVbHlN/uyYyP8AmzH9KqFZOq1/Kbfdlxr5MR/SqhVrY3+qt6O9ymto/wDQHqPeufaAVdXRaB6/zURIkdZbTC7b/k31b2P/AO45y4/p9BS1We41TV0gjpprvRxzPJ25WGZgcd/DpupRcAeGU2ouNayYLVSiJl9sVLQiUjfsnv8AZAa/b8F2zvmUT7/YrziV/rsdvlHLRXO1VL6aphf0dFKx2xH5R0Pzro1JKySsq6cGzrtPgWNHpZU6djmU0E1srEeIcT8VeuiitwzcbmAZ7i1BjuqGS0WP5bQxMp5prhKIaa48oAEzZXbMa93TmY4jzieXcd3Zsz4g9FsBtMl4yPUmwsjYwvZBT1sdRUTeqOKMl7vmGw8SAuQVOFVlLOad8Z3r5WBN+nNdChr6eeLtmvFuunVQ/wDKi2u1RXzT68xMjFyqqW4007htzOgifA6Lfx2DpZdvjPrXGeEGsq4avVijhc7sKjTC+umb4btbHyu+Ykj+UVrHExrzXcQWpMuWuo30Nqo4RQ2mjeQXxU7XF3M/bpzuc4uO3duG7kNBPeOEDS2utnD7rFq7c6d8TLvi1ztNrLm7dpDHTSOnkHpaZAxoPpjeul9k7C8BZBU/ayFu8uvbwHuVL3xXYq6WD7OZ8A21/H4qF633WrR3JdE80lxS/sMsE0Tau3VoZsyspX+1ePQR1a5vg4EdRsToSt/4gtALPxA6TU9hkENNfrdTNqbJXPH7zPyDeNxHXs5Ng1w8PNdsS0LfxjGRhFRAJPu37wPd9mx8L59y1cOw44hDLufbbYjv1uFALDOJOpPDTmmgOYVMkzZKWGTHKl27izlqonyUrj73YOewnu2c3fq0DlOkn3VsL+UNu+kxrBX+w3jFr3XY5kFvloblbZ301VTSjZ0UjTs4H5/EdD3hZ3SP7q+F/KG3fSY1vilhp4ZXw6Pu48rkWuOtrrVM8k0kbZP7bDwv8FZFxacHVHr1JFmWI3CltOYUsIp3uqQRTXCFu/K2UtBLXt32a8A9PNI25S2vLUzQHV7SGV4zzB7hQ0rXcra+Nono39em00e7AT70kO9SuWu+R49j7Y33++262tmJEZrKpkIeR37c5G6xM2ommdRC+nqM6xiWKRpY9j7nTua5p7wQXbELmWD7TV+HRiEs7SMaa3HcD8wVdcRwSlrHmTe3Hn95j/pUyYJqbqBplcvqtgOX3OyVBIL/AGLMRHLt3CSM7skHqcCFMnQ7ykFwmuVHjuuFnpPY0zmxG/W9hjMRPTnng6gt9Lo+XYdzCup6pcMvB/qV21bS3/HcVukm7vZdku1NAwu/DgLjERv37Na4++Va2Z2OgxnLrzjtqvtNeqO2V09JBcab96q42PLWys6kbOA3GxI69CR1Vxhdhm1THCSIh4GpFiOjhr0Pkq7IK3AnAskBaeRuD1H76q8unqIKuniq6WeOaCZjZI5I3BzXtI3DgR0II6gr9FwjggyO65Lw0YlUXd7ny0Lai3RSH3UEE744h/JYGs/kru65VWU5pKh9OTfdJHkbK908wqIWyj+4A+aIiLWWZERERFDbit4FW6jXSs1I0idTUeQVbjNcbTK4RQV8h75Y390crvdA+a49SWncumSi3sPxGowuYT0zrH0I5ELVq6OGuj7KYXHqOio7zLTbP9PK19Bm+HXeyTNdy/4ZSPjY/wBbHkcrx62khYa12a73upbRWW1VlfUOIDYqWB0ryT6GtBKvcc1r2lrmgg9CCOhXzFDDA0thiZGCd9mtAG/zK6N2+eGWdAN7/LLysfeq27ZRu9lLl0/X4KsDQ3gD1Q1Cq6a76jU82HY9zB0jKlu1xqGeLY4SP3Pfu5pNiO8NcrJ8Mw3HNPsXt2G4lbY6C02uEQ00DNzsN9yST1c4klxcepJJPes2iq2LY5V4w4dubNGjRoPmf2FO4fhcGHNPZC5OpOqg1xYcCNfkl3r9TNFaeF1ZWvdU3KwFwj7WUnd8tM4+aC47kxkgb7lp6hqgfkOMZHiNzks2U2G4WivhOz6atpnwyN/kuAPzq9VeW4Wu2XaD2LdbdTVsO+/Z1ELZG7+nZwIUzhe2VTQxiGob2jRob2Pnnf396ja7ZyGqeZInbhOuVx8LKi202a73+vitVitVZca2c8sVNSQOmlefQ1jQSfmCmlwwcAt9rrpRZ1rnbxQW2meJ6bHpCDPVOB3aanboyP8A1ftndzuUdDP622az2aN0NntVHQxvO7mU0DYgT6w0BexZMS21qauMxUzOzB1N7nwyFvevNHs1DA8Pmdv24WsPjdcQ4zsRvOX8NuWWfHKF9VVwR01YyniYS58cFRHJIGgd5DGuIA79tlW/wpYvfMo4hMGgstBNUG3XmluVU5jCWw08EjZJHvPc0bN2BPeS0d5CuPXlpLZbbfJNLQW+mpn1DueZ0MTWGR3pcQOp6nqVHYVtE7DKGWjDN7evY30uLaWz07lt12DtrallQXW3bXFtbG/gvUvljGRMEcbGsa0bBrRsAF9Iq0ppVg+Ubxi9WzXePJKqglbbbzaab2JU8p7N74gWSM5u7mbsCR37OafFfnp/pNm9z4Hs8vtJZal8dXfqO50sIid2lRSUo5ZpmDxYO0cd/RE/0Kzqut1vulOaS50NPVwEhxjnibIwkdx2cCF+zGMiY2ONjWMYA1rWjYADuACtzNrJI6KGlbGLxlud9Q03AtbK/VV92AsfUyTl+TgcraEqobgyxe95LxG4fJaKCWeK1VhuFbK1pLIII2OJc89zQTs0b97nAeKt6IBBBG4K81FbLbbe1+p1vpqXtn9pJ2ETWc7vS7YdT6yvUo3HsZONVDZtzdAFrXvxv3LdwrDhhsRj3t4k35L5YxkbQxjQ1rRsABsAFVf5QfGL1Z+Iy6X6uoJY6C/UdHPQ1BaezlEdPHC8B3dzNdGdx3gFp8QrUl5q+2266winudvpqyIODxHPE2RocO47OBG68YHi5waq+kbu8CCCL21se/kvWJ4eMRg7HetY35/vVRV8ndg1xt2gd2mye1ctDlF2nnp4KiPpUUhgjiLi097HFrwPSBv3FRu4neCXNdMb3XZRptZau+4bPIZY46Vrp6q3A98cjBu5zAd9pBv025tj1NoYaGgNaAABsAPBf1bdPtNU01fJWxgWec28O7xHP0WvLgsE1Kymec2jI8f+u5UMyRyQyOiljcx7CWua4bFpHeCPBdV0X4ZdV9brrTQ49j1TRWZ72+yL3WQujpIY9+rmuO3au27mM3PUb7DqLfqzGMauNX7PuGPWypqQQe2mpI3ydO7ziN1kgABsBsApyo28kfHuwQ7ruZN7eFgouHZVjX3lkuOQFviVxO86DW/CeFvI9GdOqaSpmfYa2OJ0gHbV1Y+Nzi523unu2A8AOUdwVVunuGZNluoVnxCxWaqqLrPcIoTTiJ3NERIOcvG27Gt6lxPRoB37ld+vPDbrfT1U1bT0NPFUVG3bTMia18m3dzOA3PzqHwnaeXDGSte3fc83uTx78s/RSNfgkda6Mtduhota3D4L0KEXHzwuyZDTS64af2t0lzpWAZBRU8e7qmFo2FU1o6l7AAH+lgDunKd5uoofDMRmwqpbUQ6jUcxxB/fepGto466EwyefI81TjwoYxe8o4hcGhslvlqTbrxTXOqcxpLYaaCRskkjz3NGw2BPe4tHeQsfxFYff8R11zOy3i3zRT1N8q6umBYf3eCeZ0kT2e+DmuHd47jvCuMtOM43YZqmoseP223S1juepfSUkcLpnel5aAXH1leqe3W+pqYaypoaeWopiTDK+Jrnx79/K4jdvzK1nbYisNQIfZ3d21873ve9vSygRs0Po/YmTO9727rWtdcq4TcUvWH8OmF43k9uko6+KimlnpZmFr4xNUSyta9p6h3JI3dp6g7gqL3Ex5Py6/VOszfQimiqKape6epxwvbG+Bx6k0rnbNLO/9zJBb3N3BDRP5FXaXHKqirH1kJsXkkjgbm9vlxUxPhcFTTtp5BcNAAPEWFlRbkmI5Vh1c62ZZjV0s1WwkGGvpJIH7/E8DdfNgxTKMrq20OMY5c7vUvdytioaSSd5Po2YCVelJHHK0slY17T3hw3CRxxxNDImNY0dwaNgFavr8/ct2A3v8svK3xUF9VG733uXT9fgq6OH3yeWV3+uo8m1ub9RbMxwl+oscu9bVAdQ2VzekLD47Ev23GzD1Gq+UMx7JrLrHQGptjqXFYrNS0WOCGPlpooIm7SQt280ObIXbt7+Us8NlaGvNX2y23WAU10t9NWQhweI6iJsjQ4dx2cCN1DwbW1QrhWVDQ4AEBoyAvy1zy1N8slIS4BB9FNPCbEkG+t7c+5Q08nHohW41YLprFktskpqy+xiiszZmcrxRAh0kwB8JHhgafRHuOjgTL694liuSuifkeM2m6uhBEZraKOcsB7+XnB2+ZZUAAAAbAL+qFxHEpcRq3VbsidLcBwCkqOjjo4GwNzA9TzUT+Njhjs+ZaXjJtNsOoaW/wCMPdVexrXRMifW0jthNHyxgc7m7Ne3vPmvAG7lDbgytObV3EXiVRhtNUF1vrO2ucrWnkhoNi2o7Q9wBY5zRv3uc0DrsreV56W3W+hkmloqGnp31D+eZ0UTWGR3pcQOp695UvQ7TzUlBJQyN394EAk6X1vzHHgo+qwSOoq21THbtrXAGttOiip5SPE71ftFrXe7VRyVMFgvLKmuEbS4xQPikZ2h29yHlgJ/CCjT5PHFL9duICkyaitsz7XY6GrfW1XIeyjMsLo2M5u7mcX7hvfs1x8CrR3sZIx0cjA5rgQ5pG4IPgV+FvttutNMKO1W+mo6dpJEVPE2NgJ7zytAC8Um0TqXC34buX3ri99A7XK3xXqowds9c2s3rWtlbiNM16VXf5TnE72zN8UzkUUj7RNaTazUNaSyOojmkk5XHuBc2Xdu/fyu27irEF+NXR0lwp30dfSw1MEg2fFMwPY4esHoVHYPiRwmrbVBu9a4I01W5iNEK+nMBNr8eig15MPE8goaTNswrbZPBarkKKko6iRha2okjMxk5N/bBvO0EjpudvA7dF4t+DKl1sldn2Bz01uzGKIMqI5jywXRjRs0PcPaSgAAP7iAGu2ADmyjiiigjbDDG2ONgDWsaNg0DuAA7gvtbM+P1D8SdiUHsONstRYACx56LDFhULaMUcvtAcdM73uOSo7zfTfPdNrm60Z3iVzslUCQ0VcBayT1xv8AaSD1tJHrWvQU89VMympYJJpZDysjjaXOcfQAOpV8FTS01bA+lrKeKeGQbPjlYHNcPQQehXjtuOY9ZpHS2ew26he8bOdTUrIiR6y0DdWePb4hn8yC7u51h7j8VCO2UG97MuXTP3qs3h64EdRNSbjTXzUmgrMUxdjmvkZUxmOvrW9/JHE4bxgj3bwO/wA0O8LDsuwOkGjd+01wu3QUUMuOVlnttMzoyPnpnxxt6+sjcnr4lbqiq2J49VYrM2WXINNw0aD5lTlDhUFDGWMzJ1PFUY2nC8rvmVxYPbLBXTX6aq9hCgELhM2YO5S1zdt27Hfffu2JO2yvHoIHUtDT0zyC6GJkZI7iQAF/I7db4qyS4xUNOyrmaGSTtiaJHtHcC7bcj416Fnx/HzjnZ+xuhl+N7k2vwHJYsKwkYZv+1vb1uFtL/NQ848OF5+f2h+r+BWt0uSWqENutJAzd9xpGjpI1o9tLGPncwbdS1oMG+H/GL5lmtWGWmw2+aqqGXujqZQxpIihimY+SR3oa1rSSfUrp1jbdjON2iuqrnacfttFWVx5qqop6SOOWc9+73NALvnJW3hu1c1DROo3t3siGm+l+B5gcPJYK3AY6qpFQ127zFtf3+qqd41mZyziJyj69vZfI6cG0GXm7I2/Ydj2O/Tl29ty+759+u64Wr2rpYrHfGsZerNQ3BsRJYKqnZKGk9+3MDssd9j/A/wDQmwfo2H+6pOi23ZTU7IXQfZAGRsMu6y0qnZl08zpBLqb5j9VRst60k0U1C1qyOnx7CLFUVDHyBtTXvjcKSjZ4vlk22Gw68vtj3AE9Fcf9j/A/9CbB+jYf7qzNHRUdvp2UdBSQ00EY2ZFDGGMaPUB0CyT7el0ZEENncybgeFs/NeItlQHgyyXHcP1WuaX6fWjSvT6xae2Nzn0lkpG04lcNnTSEl0kpHgXvc9xHgXLaURc+kkdK8yPNyTc9SraxjY2hjRYBERF4XpERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERERf/2Q==</v>
@@ -588,10 +597,13 @@
 Payment shall be process on the completion of job/delivery of materials to our satisfaction only . All dispute are subject
 to Guwahati Jurisdiction.</v>
       </c>
+      <c r="O4" t="str">
+        <v>JB</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>